<commit_message>
changed VH route for out_04
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/SystemDocumentation/github/uactechdoc/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57BE20EA-1D71-4144-91A6-6796A5FA9626}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C533099-6638-234B-8899-0C0135B5933B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="5780" yWindow="1640" windowWidth="24460" windowHeight="16580" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -18,8 +18,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId3"/>
-    <pivotCache cacheId="3" r:id="rId4"/>
+    <pivotCache cacheId="4" r:id="rId3"/>
+    <pivotCache cacheId="5" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -8230,7 +8230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="121">
+  <cellXfs count="120">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -8445,7 +8445,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8746,19 +8745,6 @@
         <family val="2"/>
         <scheme val="major"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri Light"/>
-        <family val="2"/>
-        <scheme val="major"/>
-      </font>
       <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
@@ -8802,6 +8788,19 @@
         <vertical/>
         <horizontal/>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </font>
     </dxf>
     <dxf>
       <border outline="0">
@@ -17329,70 +17328,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="12">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="7"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of Tag" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B56" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -17648,13 +17584,76 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Tag" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BD7E3698-8860-904B-8BDB-00EF1039C49C}" name="Table1" displayName="Table1" ref="A1:M950" totalsRowCount="1" headerRowDxfId="20" dataDxfId="19" tableBorderDxfId="18">
   <autoFilter ref="A1:M949" xr:uid="{BD7E3698-8860-904B-8BDB-00EF1039C49C}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{4D442337-BE86-B24A-84A4-338FB80A6A49}" name="Tag" dataDxfId="15"/>
-    <tableColumn id="2" xr3:uid="{74A36D7B-C989-3B4B-B1E5-AB1FA4C2DD45}" name="SrcTag" dataDxfId="17" totalsRowDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{B4B079C1-C2FD-4543-BF85-C40BEF0990F3}" name="SrcPort" dataDxfId="16" totalsRowDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{4D442337-BE86-B24A-84A4-338FB80A6A49}" name="Tag" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{74A36D7B-C989-3B4B-B1E5-AB1FA4C2DD45}" name="SrcTag" dataDxfId="16" totalsRowDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{B4B079C1-C2FD-4543-BF85-C40BEF0990F3}" name="SrcPort" dataDxfId="15" totalsRowDxfId="3"/>
     <tableColumn id="4" xr3:uid="{AC3F24B7-C4B3-CC4C-A7E3-6BB3319549AD}" name="DstTag" dataDxfId="14" totalsRowDxfId="2"/>
     <tableColumn id="5" xr3:uid="{723F3509-3335-1241-A5F2-61206DF5595A}" name="DstPort" dataDxfId="13"/>
     <tableColumn id="6" xr3:uid="{7D4B1BBD-F461-7E4D-A272-8B68F8EE10FB}" name="Type" dataDxfId="12"/>
@@ -46215,7 +46214,7 @@
         <v>1151</v>
       </c>
       <c r="C894" s="83" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="D894" s="83" t="s">
         <v>1151</v>
@@ -48008,7 +48007,7 @@
       </c>
       <c r="J949" s="29"/>
       <c r="K949" s="29"/>
-      <c r="L949" s="120"/>
+      <c r="L949" s="31"/>
       <c r="M949" s="29"/>
     </row>
     <row r="950" spans="1:13" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
updates including 85in TV
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9492C04D-52D6-2C46-99CC-F3C01445A124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43C9FBFF-0FF0-E846-B08C-BF5B18C3C68F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3740" yWindow="1740" windowWidth="26500" windowHeight="14260" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -18,8 +18,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="16" r:id="rId3"/>
-    <pivotCache cacheId="22" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
+    <pivotCache cacheId="1" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7881" uniqueCount="2638">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7906" uniqueCount="2649">
   <si>
     <t>Tag</t>
   </si>
@@ -7955,6 +7955,39 @@
   </si>
   <si>
     <t>in_77</t>
+  </si>
+  <si>
+    <t>d_o_120</t>
+  </si>
+  <si>
+    <t>ip127</t>
+  </si>
+  <si>
+    <t>A&amp;H</t>
+  </si>
+  <si>
+    <t>reference Mic</t>
+  </si>
+  <si>
+    <t>rt970</t>
+  </si>
+  <si>
+    <t>ZVIU-A005</t>
+  </si>
+  <si>
+    <t>2605-0500</t>
+  </si>
+  <si>
+    <t>Stg Dsp TV</t>
+  </si>
+  <si>
+    <t>2310-0904</t>
+  </si>
+  <si>
+    <t>33m</t>
+  </si>
+  <si>
+    <t>avshop.ca</t>
   </si>
 </sst>
 </file>
@@ -8377,7 +8410,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="137">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -8592,25 +8625,7 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="14" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -8621,9 +8636,6 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="3" borderId="5" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -8693,6 +8705,52 @@
         <scheme val="none"/>
       </font>
       <numFmt numFmtId="30" formatCode="@"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor indexed="65"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -8813,86 +8871,6 @@
         <scheme val="major"/>
       </font>
       <numFmt numFmtId="30" formatCode="@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79998168889431442"/>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri Light"/>
-        <family val="2"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri Light"/>
-        <family val="2"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri Light"/>
-        <family val="2"/>
-        <scheme val="major"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor indexed="65"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri Light"/>
-        <family val="2"/>
-        <scheme val="major"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <name val="Calibri Light"/>
-        <family val="2"/>
-        <scheme val="major"/>
-      </font>
-      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <border diagonalUp="0" diagonalDown="0">
         <left/>
@@ -8955,6 +8933,40 @@
         <vertical/>
         <horizontal/>
       </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <name val="Calibri Light"/>
+        <family val="2"/>
+        <scheme val="major"/>
+      </font>
     </dxf>
     <dxf>
       <border outline="0">
@@ -17482,7 +17494,70 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Tag" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B56" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -17738,86 +17813,23 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="12">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="7"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of Tag" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BD7E3698-8860-904B-8BDB-00EF1039C49C}" name="Table1" displayName="Table1" ref="A1:M973" totalsRowCount="1" headerRowDxfId="20" dataDxfId="19" tableBorderDxfId="18">
   <autoFilter ref="A1:M972" xr:uid="{BD7E3698-8860-904B-8BDB-00EF1039C49C}"/>
   <tableColumns count="13">
-    <tableColumn id="1" xr3:uid="{4D442337-BE86-B24A-84A4-338FB80A6A49}" name="Tag" dataDxfId="11"/>
-    <tableColumn id="2" xr3:uid="{74A36D7B-C989-3B4B-B1E5-AB1FA4C2DD45}" name="SrcTag" dataDxfId="10" totalsRowDxfId="4"/>
-    <tableColumn id="3" xr3:uid="{B4B079C1-C2FD-4543-BF85-C40BEF0990F3}" name="SrcPort" dataDxfId="17" totalsRowDxfId="3"/>
-    <tableColumn id="4" xr3:uid="{AC3F24B7-C4B3-CC4C-A7E3-6BB3319549AD}" name="DstTag" dataDxfId="16" totalsRowDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{723F3509-3335-1241-A5F2-61206DF5595A}" name="DstPort" dataDxfId="15"/>
-    <tableColumn id="6" xr3:uid="{7D4B1BBD-F461-7E4D-A272-8B68F8EE10FB}" name="Type" dataDxfId="9"/>
-    <tableColumn id="13" xr3:uid="{AECEAF7F-6B15-0348-8A77-06BCE8B4829E}" name="Protocol" dataDxfId="8"/>
-    <tableColumn id="7" xr3:uid="{342ADFC8-8081-D246-A6B4-8A5EE1D7A44F}" name="Length" dataDxfId="7"/>
-    <tableColumn id="8" xr3:uid="{52DF302F-1C2C-3641-87D6-1971497058A4}" name="Labelled?" dataDxfId="6"/>
-    <tableColumn id="9" xr3:uid="{C0483DE7-3B56-B145-9C6E-0E6DE59EDB05}" name="Usage" dataDxfId="5"/>
-    <tableColumn id="10" xr3:uid="{5CD47A7F-4A34-3A46-926E-FFBED1348BD5}" name="Notes" dataDxfId="14" totalsRowDxfId="1"/>
-    <tableColumn id="11" xr3:uid="{5C50ECE5-BC4B-6C47-90C1-11D93DE5D81A}" name="Invoice" dataDxfId="13" totalsRowDxfId="0"/>
-    <tableColumn id="12" xr3:uid="{939C157F-5419-B846-9271-37F3BBF6433E}" name="Pathway" dataDxfId="12"/>
+    <tableColumn id="1" xr3:uid="{4D442337-BE86-B24A-84A4-338FB80A6A49}" name="Tag" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{74A36D7B-C989-3B4B-B1E5-AB1FA4C2DD45}" name="SrcTag" dataDxfId="16" totalsRowDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{B4B079C1-C2FD-4543-BF85-C40BEF0990F3}" name="SrcPort" dataDxfId="15" totalsRowDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{AC3F24B7-C4B3-CC4C-A7E3-6BB3319549AD}" name="DstTag" dataDxfId="14" totalsRowDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{723F3509-3335-1241-A5F2-61206DF5595A}" name="DstPort" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{7D4B1BBD-F461-7E4D-A272-8B68F8EE10FB}" name="Type" dataDxfId="12"/>
+    <tableColumn id="13" xr3:uid="{AECEAF7F-6B15-0348-8A77-06BCE8B4829E}" name="Protocol" dataDxfId="11"/>
+    <tableColumn id="7" xr3:uid="{342ADFC8-8081-D246-A6B4-8A5EE1D7A44F}" name="Length" dataDxfId="10"/>
+    <tableColumn id="8" xr3:uid="{52DF302F-1C2C-3641-87D6-1971497058A4}" name="Labelled?" dataDxfId="9"/>
+    <tableColumn id="9" xr3:uid="{C0483DE7-3B56-B145-9C6E-0E6DE59EDB05}" name="Usage" dataDxfId="8"/>
+    <tableColumn id="10" xr3:uid="{5CD47A7F-4A34-3A46-926E-FFBED1348BD5}" name="Notes" dataDxfId="7" totalsRowDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{5C50ECE5-BC4B-6C47-90C1-11D93DE5D81A}" name="Invoice" dataDxfId="6" totalsRowDxfId="0"/>
+    <tableColumn id="12" xr3:uid="{939C157F-5419-B846-9271-37F3BBF6433E}" name="Pathway" dataDxfId="5"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -21756,10 +21768,18 @@
       <c r="A120" s="21" t="s">
         <v>316</v>
       </c>
-      <c r="B120" s="22"/>
-      <c r="C120" s="23"/>
-      <c r="D120" s="22"/>
-      <c r="E120" s="23"/>
+      <c r="B120" s="22" t="s">
+        <v>2643</v>
+      </c>
+      <c r="C120" s="23" t="s">
+        <v>162</v>
+      </c>
+      <c r="D120" s="22" t="s">
+        <v>2644</v>
+      </c>
+      <c r="E120" s="23" t="s">
+        <v>344</v>
+      </c>
       <c r="F120" s="23" t="s">
         <v>38</v>
       </c>
@@ -21772,7 +21792,9 @@
       <c r="I120" s="23" t="s">
         <v>110</v>
       </c>
-      <c r="J120" s="23"/>
+      <c r="J120" s="23" t="s">
+        <v>2645</v>
+      </c>
       <c r="K120" s="23"/>
       <c r="L120" s="23"/>
       <c r="M120" s="24"/>
@@ -48047,13 +48069,13 @@
       <c r="E945" s="82" t="s">
         <v>2571</v>
       </c>
-      <c r="F945" s="126" t="s">
+      <c r="F945" s="31" t="s">
         <v>1771</v>
       </c>
-      <c r="G945" s="126" t="s">
+      <c r="G945" s="31" t="s">
         <v>354</v>
       </c>
-      <c r="H945" s="127">
+      <c r="H945" s="23">
         <v>0</v>
       </c>
       <c r="I945" s="19" t="s">
@@ -48063,7 +48085,7 @@
         <v>1280</v>
       </c>
       <c r="K945" s="29"/>
-      <c r="L945" s="126"/>
+      <c r="L945" s="31"/>
       <c r="M945" s="29"/>
     </row>
     <row r="946" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
@@ -48082,13 +48104,13 @@
       <c r="E946" s="82" t="s">
         <v>2572</v>
       </c>
-      <c r="F946" s="126" t="s">
+      <c r="F946" s="31" t="s">
         <v>1771</v>
       </c>
-      <c r="G946" s="126" t="s">
+      <c r="G946" s="31" t="s">
         <v>354</v>
       </c>
-      <c r="H946" s="127">
+      <c r="H946" s="23">
         <v>0</v>
       </c>
       <c r="I946" s="19" t="s">
@@ -48098,256 +48120,256 @@
         <v>1281</v>
       </c>
       <c r="K946" s="29"/>
-      <c r="L946" s="126"/>
+      <c r="L946" s="31"/>
       <c r="M946" s="29"/>
     </row>
     <row r="947" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A947" s="29" t="s">
         <v>2591</v>
       </c>
-      <c r="B947" s="128" t="s">
+      <c r="B947" s="100" t="s">
         <v>2570</v>
       </c>
-      <c r="C947" s="122" t="s">
+      <c r="C947" s="83" t="s">
         <v>876</v>
       </c>
-      <c r="D947" s="123" t="s">
+      <c r="D947" s="85" t="s">
         <v>1250</v>
       </c>
-      <c r="E947" s="122" t="s">
+      <c r="E947" s="83" t="s">
         <v>2573</v>
       </c>
-      <c r="F947" s="126" t="s">
+      <c r="F947" s="31" t="s">
         <v>1771</v>
       </c>
-      <c r="G947" s="126" t="s">
+      <c r="G947" s="31" t="s">
         <v>354</v>
       </c>
-      <c r="H947" s="129">
+      <c r="H947" s="29">
         <v>0</v>
       </c>
-      <c r="I947" s="125" t="s">
+      <c r="I947" s="120" t="s">
         <v>71</v>
       </c>
       <c r="J947" s="29" t="s">
         <v>1282</v>
       </c>
       <c r="K947" s="29"/>
-      <c r="L947" s="126"/>
+      <c r="L947" s="31"/>
       <c r="M947" s="29"/>
     </row>
     <row r="948" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A948" s="29" t="s">
         <v>2592</v>
       </c>
-      <c r="B948" s="128" t="s">
+      <c r="B948" s="100" t="s">
         <v>2570</v>
       </c>
-      <c r="C948" s="122" t="s">
+      <c r="C948" s="83" t="s">
         <v>875</v>
       </c>
-      <c r="D948" s="123" t="s">
+      <c r="D948" s="85" t="s">
         <v>1250</v>
       </c>
-      <c r="E948" s="122" t="s">
+      <c r="E948" s="83" t="s">
         <v>2574</v>
       </c>
-      <c r="F948" s="126" t="s">
+      <c r="F948" s="31" t="s">
         <v>1771</v>
       </c>
-      <c r="G948" s="126" t="s">
+      <c r="G948" s="31" t="s">
         <v>354</v>
       </c>
-      <c r="H948" s="129">
+      <c r="H948" s="29">
         <v>0</v>
       </c>
-      <c r="I948" s="125" t="s">
+      <c r="I948" s="120" t="s">
         <v>71</v>
       </c>
       <c r="J948" s="29" t="s">
         <v>1283</v>
       </c>
       <c r="K948" s="29"/>
-      <c r="L948" s="126"/>
+      <c r="L948" s="31"/>
       <c r="M948" s="29"/>
     </row>
     <row r="949" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A949" s="29" t="s">
         <v>2593</v>
       </c>
-      <c r="B949" s="128" t="s">
+      <c r="B949" s="100" t="s">
         <v>357</v>
       </c>
-      <c r="C949" s="122" t="s">
+      <c r="C949" s="83" t="s">
         <v>520</v>
       </c>
-      <c r="D949" s="123" t="s">
+      <c r="D949" s="85" t="s">
         <v>1250</v>
       </c>
-      <c r="E949" s="122" t="s">
+      <c r="E949" s="83" t="s">
         <v>2575</v>
       </c>
-      <c r="F949" s="126" t="s">
+      <c r="F949" s="31" t="s">
         <v>1771</v>
       </c>
-      <c r="G949" s="126" t="s">
+      <c r="G949" s="31" t="s">
         <v>354</v>
       </c>
-      <c r="H949" s="129">
+      <c r="H949" s="29">
         <v>0</v>
       </c>
-      <c r="I949" s="125" t="s">
+      <c r="I949" s="120" t="s">
         <v>71</v>
       </c>
       <c r="J949" s="29" t="s">
         <v>1284</v>
       </c>
       <c r="K949" s="29"/>
-      <c r="L949" s="126"/>
+      <c r="L949" s="31"/>
       <c r="M949" s="29"/>
     </row>
     <row r="950" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A950" s="29" t="s">
         <v>2594</v>
       </c>
-      <c r="B950" s="128" t="s">
+      <c r="B950" s="100" t="s">
         <v>357</v>
       </c>
-      <c r="C950" s="122" t="s">
+      <c r="C950" s="83" t="s">
         <v>522</v>
       </c>
-      <c r="D950" s="123" t="s">
+      <c r="D950" s="85" t="s">
         <v>1250</v>
       </c>
-      <c r="E950" s="122" t="s">
+      <c r="E950" s="83" t="s">
         <v>2576</v>
       </c>
-      <c r="F950" s="126" t="s">
+      <c r="F950" s="31" t="s">
         <v>1771</v>
       </c>
-      <c r="G950" s="126" t="s">
+      <c r="G950" s="31" t="s">
         <v>354</v>
       </c>
-      <c r="H950" s="129">
+      <c r="H950" s="29">
         <v>0</v>
       </c>
-      <c r="I950" s="125" t="s">
+      <c r="I950" s="120" t="s">
         <v>71</v>
       </c>
       <c r="J950" s="29" t="s">
         <v>1285</v>
       </c>
       <c r="K950" s="29"/>
-      <c r="L950" s="126"/>
+      <c r="L950" s="31"/>
       <c r="M950" s="29"/>
     </row>
     <row r="951" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A951" s="29" t="s">
         <v>2595</v>
       </c>
-      <c r="B951" s="128" t="s">
+      <c r="B951" s="100" t="s">
         <v>357</v>
       </c>
-      <c r="C951" s="122" t="s">
+      <c r="C951" s="83" t="s">
         <v>876</v>
       </c>
-      <c r="D951" s="123" t="s">
+      <c r="D951" s="85" t="s">
         <v>1250</v>
       </c>
-      <c r="E951" s="122" t="s">
+      <c r="E951" s="83" t="s">
         <v>2577</v>
       </c>
-      <c r="F951" s="126" t="s">
+      <c r="F951" s="31" t="s">
         <v>1771</v>
       </c>
-      <c r="G951" s="126" t="s">
+      <c r="G951" s="31" t="s">
         <v>354</v>
       </c>
-      <c r="H951" s="129">
+      <c r="H951" s="29">
         <v>0</v>
       </c>
-      <c r="I951" s="125" t="s">
+      <c r="I951" s="120" t="s">
         <v>71</v>
       </c>
       <c r="J951" s="29" t="s">
         <v>1286</v>
       </c>
       <c r="K951" s="29"/>
-      <c r="L951" s="126"/>
+      <c r="L951" s="31"/>
       <c r="M951" s="29"/>
     </row>
     <row r="952" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A952" s="29" t="s">
         <v>2596</v>
       </c>
-      <c r="B952" s="128" t="s">
+      <c r="B952" s="100" t="s">
         <v>357</v>
       </c>
-      <c r="C952" s="122" t="s">
+      <c r="C952" s="83" t="s">
         <v>875</v>
       </c>
-      <c r="D952" s="123" t="s">
+      <c r="D952" s="85" t="s">
         <v>1250</v>
       </c>
-      <c r="E952" s="122" t="s">
+      <c r="E952" s="83" t="s">
         <v>2578</v>
       </c>
-      <c r="F952" s="126" t="s">
+      <c r="F952" s="31" t="s">
         <v>1771</v>
       </c>
-      <c r="G952" s="126" t="s">
+      <c r="G952" s="31" t="s">
         <v>354</v>
       </c>
-      <c r="H952" s="129">
+      <c r="H952" s="29">
         <v>0</v>
       </c>
-      <c r="I952" s="125" t="s">
+      <c r="I952" s="120" t="s">
         <v>71</v>
       </c>
       <c r="J952" s="29" t="s">
         <v>1287</v>
       </c>
       <c r="K952" s="29"/>
-      <c r="L952" s="126"/>
+      <c r="L952" s="31"/>
       <c r="M952" s="29"/>
     </row>
     <row r="953" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A953" s="29" t="s">
         <v>2597</v>
       </c>
-      <c r="B953" s="128" t="s">
+      <c r="B953" s="100" t="s">
         <v>358</v>
       </c>
-      <c r="C953" s="122" t="s">
+      <c r="C953" s="83" t="s">
         <v>520</v>
       </c>
-      <c r="D953" s="123" t="s">
+      <c r="D953" s="85" t="s">
         <v>1250</v>
       </c>
-      <c r="E953" s="122" t="s">
+      <c r="E953" s="83" t="s">
         <v>2579</v>
       </c>
-      <c r="F953" s="126" t="s">
+      <c r="F953" s="31" t="s">
         <v>1771</v>
       </c>
-      <c r="G953" s="126" t="s">
+      <c r="G953" s="31" t="s">
         <v>354</v>
       </c>
-      <c r="H953" s="129">
+      <c r="H953" s="29">
         <v>0</v>
       </c>
-      <c r="I953" s="125" t="s">
+      <c r="I953" s="120" t="s">
         <v>71</v>
       </c>
       <c r="J953" s="29" t="s">
         <v>1288</v>
       </c>
       <c r="K953" s="29"/>
-      <c r="L953" s="126"/>
+      <c r="L953" s="31"/>
       <c r="M953" s="29"/>
     </row>
     <row r="954" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A954" s="124" t="s">
+      <c r="A954" s="29" t="s">
         <v>2598</v>
       </c>
       <c r="B954" s="113" t="s">
@@ -48362,503 +48384,543 @@
       <c r="E954" s="82" t="s">
         <v>2580</v>
       </c>
-      <c r="F954" s="130" t="s">
+      <c r="F954" s="31" t="s">
         <v>1771</v>
       </c>
-      <c r="G954" s="130" t="s">
+      <c r="G954" s="31" t="s">
         <v>354</v>
       </c>
-      <c r="H954" s="127">
+      <c r="H954" s="23">
         <v>0</v>
       </c>
       <c r="I954" s="19" t="s">
         <v>71</v>
       </c>
-      <c r="J954" s="124" t="s">
+      <c r="J954" s="29" t="s">
         <v>1289</v>
       </c>
-      <c r="K954" s="124"/>
-      <c r="L954" s="130"/>
-      <c r="M954" s="124"/>
+      <c r="K954" s="29"/>
+      <c r="L954" s="31"/>
+      <c r="M954" s="29"/>
     </row>
     <row r="955" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A955" s="124" t="s">
+      <c r="A955" s="29" t="s">
         <v>2599</v>
       </c>
-      <c r="B955" s="128" t="s">
+      <c r="B955" s="100" t="s">
         <v>358</v>
       </c>
-      <c r="C955" s="122" t="s">
+      <c r="C955" s="83" t="s">
         <v>876</v>
       </c>
-      <c r="D955" s="123" t="s">
+      <c r="D955" s="85" t="s">
         <v>1250</v>
       </c>
-      <c r="E955" s="122" t="s">
+      <c r="E955" s="83" t="s">
         <v>2581</v>
       </c>
-      <c r="F955" s="130" t="s">
+      <c r="F955" s="31" t="s">
         <v>1771</v>
       </c>
-      <c r="G955" s="130" t="s">
+      <c r="G955" s="31" t="s">
         <v>354</v>
       </c>
-      <c r="H955" s="129">
+      <c r="H955" s="29">
         <v>0</v>
       </c>
-      <c r="I955" s="125" t="s">
+      <c r="I955" s="120" t="s">
         <v>71</v>
       </c>
-      <c r="J955" s="124" t="s">
+      <c r="J955" s="29" t="s">
         <v>1291</v>
       </c>
-      <c r="K955" s="124"/>
-      <c r="L955" s="130"/>
-      <c r="M955" s="124"/>
+      <c r="K955" s="29"/>
+      <c r="L955" s="31"/>
+      <c r="M955" s="29"/>
     </row>
     <row r="956" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A956" s="124" t="s">
+      <c r="A956" s="29" t="s">
         <v>2600</v>
       </c>
-      <c r="B956" s="128" t="s">
+      <c r="B956" s="100" t="s">
         <v>358</v>
       </c>
-      <c r="C956" s="122" t="s">
+      <c r="C956" s="83" t="s">
         <v>875</v>
       </c>
-      <c r="D956" s="123" t="s">
+      <c r="D956" s="85" t="s">
         <v>1250</v>
       </c>
-      <c r="E956" s="122" t="s">
+      <c r="E956" s="83" t="s">
         <v>2582</v>
       </c>
-      <c r="F956" s="130" t="s">
+      <c r="F956" s="31" t="s">
         <v>1771</v>
       </c>
-      <c r="G956" s="130" t="s">
+      <c r="G956" s="31" t="s">
         <v>354</v>
       </c>
-      <c r="H956" s="129">
+      <c r="H956" s="29">
         <v>0</v>
       </c>
-      <c r="I956" s="125" t="s">
+      <c r="I956" s="120" t="s">
         <v>71</v>
       </c>
-      <c r="J956" s="124" t="s">
+      <c r="J956" s="29" t="s">
         <v>1292</v>
       </c>
-      <c r="K956" s="124"/>
-      <c r="L956" s="130"/>
-      <c r="M956" s="124"/>
+      <c r="K956" s="29"/>
+      <c r="L956" s="31"/>
+      <c r="M956" s="29"/>
     </row>
     <row r="957" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A957" s="124" t="s">
+      <c r="A957" s="29" t="s">
         <v>2601</v>
       </c>
-      <c r="B957" s="128" t="s">
+      <c r="B957" s="100" t="s">
         <v>359</v>
       </c>
-      <c r="C957" s="122" t="s">
+      <c r="C957" s="83" t="s">
         <v>520</v>
       </c>
-      <c r="D957" s="123" t="s">
+      <c r="D957" s="85" t="s">
         <v>1250</v>
       </c>
-      <c r="E957" s="122" t="s">
+      <c r="E957" s="83" t="s">
         <v>2583</v>
       </c>
-      <c r="F957" s="130" t="s">
+      <c r="F957" s="31" t="s">
         <v>1771</v>
       </c>
-      <c r="G957" s="130" t="s">
+      <c r="G957" s="31" t="s">
         <v>354</v>
       </c>
-      <c r="H957" s="129">
+      <c r="H957" s="29">
         <v>0</v>
       </c>
-      <c r="I957" s="125" t="s">
+      <c r="I957" s="120" t="s">
         <v>71</v>
       </c>
-      <c r="J957" s="124" t="s">
+      <c r="J957" s="29" t="s">
         <v>1293</v>
       </c>
-      <c r="K957" s="124"/>
-      <c r="L957" s="130"/>
-      <c r="M957" s="124"/>
+      <c r="K957" s="29"/>
+      <c r="L957" s="31"/>
+      <c r="M957" s="29"/>
     </row>
     <row r="958" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A958" s="124" t="s">
+      <c r="A958" s="29" t="s">
         <v>2602</v>
       </c>
-      <c r="B958" s="128" t="s">
+      <c r="B958" s="100" t="s">
         <v>359</v>
       </c>
-      <c r="C958" s="122" t="s">
+      <c r="C958" s="83" t="s">
         <v>522</v>
       </c>
-      <c r="D958" s="123" t="s">
+      <c r="D958" s="85" t="s">
         <v>1250</v>
       </c>
-      <c r="E958" s="122" t="s">
+      <c r="E958" s="83" t="s">
         <v>2584</v>
       </c>
-      <c r="F958" s="130" t="s">
+      <c r="F958" s="31" t="s">
         <v>1771</v>
       </c>
-      <c r="G958" s="130" t="s">
+      <c r="G958" s="31" t="s">
         <v>354</v>
       </c>
-      <c r="H958" s="129">
+      <c r="H958" s="29">
         <v>0</v>
       </c>
-      <c r="I958" s="125" t="s">
+      <c r="I958" s="120" t="s">
         <v>71</v>
       </c>
-      <c r="J958" s="124" t="s">
+      <c r="J958" s="29" t="s">
         <v>2587</v>
       </c>
-      <c r="K958" s="124"/>
-      <c r="L958" s="130"/>
-      <c r="M958" s="124"/>
+      <c r="K958" s="29"/>
+      <c r="L958" s="31"/>
+      <c r="M958" s="29"/>
     </row>
     <row r="959" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A959" s="124" t="s">
+      <c r="A959" s="29" t="s">
         <v>2603</v>
       </c>
-      <c r="B959" s="128" t="s">
+      <c r="B959" s="100" t="s">
         <v>359</v>
       </c>
-      <c r="C959" s="122" t="s">
+      <c r="C959" s="83" t="s">
         <v>876</v>
       </c>
-      <c r="D959" s="123" t="s">
+      <c r="D959" s="85" t="s">
         <v>1250</v>
       </c>
-      <c r="E959" s="122" t="s">
+      <c r="E959" s="83" t="s">
         <v>2585</v>
       </c>
-      <c r="F959" s="130" t="s">
+      <c r="F959" s="31" t="s">
         <v>1771</v>
       </c>
-      <c r="G959" s="130" t="s">
+      <c r="G959" s="31" t="s">
         <v>354</v>
       </c>
-      <c r="H959" s="129">
+      <c r="H959" s="29">
         <v>0</v>
       </c>
-      <c r="I959" s="125" t="s">
+      <c r="I959" s="120" t="s">
         <v>71</v>
       </c>
-      <c r="J959" s="124" t="s">
+      <c r="J959" s="29" t="s">
         <v>2588</v>
       </c>
-      <c r="K959" s="124"/>
-      <c r="L959" s="130"/>
-      <c r="M959" s="124"/>
+      <c r="K959" s="29"/>
+      <c r="L959" s="31"/>
+      <c r="M959" s="29"/>
     </row>
     <row r="960" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A960" s="124" t="s">
+      <c r="A960" s="29" t="s">
         <v>2604</v>
       </c>
-      <c r="B960" s="128" t="s">
+      <c r="B960" s="100" t="s">
         <v>359</v>
       </c>
-      <c r="C960" s="122" t="s">
+      <c r="C960" s="83" t="s">
         <v>875</v>
       </c>
-      <c r="D960" s="123" t="s">
+      <c r="D960" s="85" t="s">
         <v>1250</v>
       </c>
-      <c r="E960" s="122" t="s">
+      <c r="E960" s="83" t="s">
         <v>2586</v>
       </c>
-      <c r="F960" s="130" t="s">
+      <c r="F960" s="31" t="s">
         <v>1771</v>
       </c>
-      <c r="G960" s="130" t="s">
+      <c r="G960" s="31" t="s">
         <v>354</v>
       </c>
-      <c r="H960" s="129">
+      <c r="H960" s="29">
         <v>0</v>
       </c>
-      <c r="I960" s="125" t="s">
+      <c r="I960" s="120" t="s">
         <v>71</v>
       </c>
-      <c r="J960" s="124" t="s">
+      <c r="J960" s="29" t="s">
         <v>1296</v>
       </c>
-      <c r="K960" s="124"/>
-      <c r="L960" s="130"/>
-      <c r="M960" s="124"/>
+      <c r="K960" s="29"/>
+      <c r="L960" s="31"/>
+      <c r="M960" s="29"/>
     </row>
     <row r="961" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A961" s="124" t="s">
+      <c r="A961" s="29" t="s">
         <v>1254</v>
       </c>
-      <c r="B961" s="128" t="s">
+      <c r="B961" s="100" t="s">
         <v>2620</v>
       </c>
-      <c r="C961" s="122"/>
-      <c r="D961" s="123" t="s">
+      <c r="C961" s="83"/>
+      <c r="D961" s="85" t="s">
         <v>2605</v>
       </c>
-      <c r="E961" s="122" t="s">
+      <c r="E961" s="83" t="s">
         <v>519</v>
       </c>
-      <c r="F961" s="130"/>
-      <c r="G961" s="130"/>
-      <c r="H961" s="129"/>
-      <c r="I961" s="125"/>
+      <c r="F961" s="31"/>
+      <c r="G961" s="31"/>
+      <c r="H961" s="29"/>
+      <c r="I961" s="120"/>
       <c r="J961" s="35" t="s">
         <v>2606</v>
       </c>
-      <c r="K961" s="124"/>
-      <c r="L961" s="130"/>
-      <c r="M961" s="124"/>
+      <c r="K961" s="29"/>
+      <c r="L961" s="31"/>
+      <c r="M961" s="29"/>
     </row>
     <row r="962" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A962" s="124" t="s">
+      <c r="A962" s="29" t="s">
         <v>1255</v>
       </c>
-      <c r="B962" s="128"/>
-      <c r="C962" s="122"/>
-      <c r="D962" s="123" t="s">
+      <c r="B962" s="100"/>
+      <c r="C962" s="83"/>
+      <c r="D962" s="85" t="s">
         <v>2605</v>
       </c>
-      <c r="E962" s="122" t="s">
+      <c r="E962" s="83" t="s">
         <v>524</v>
       </c>
-      <c r="F962" s="130"/>
-      <c r="G962" s="130"/>
-      <c r="H962" s="129"/>
-      <c r="I962" s="125"/>
+      <c r="F962" s="31"/>
+      <c r="G962" s="31"/>
+      <c r="H962" s="29"/>
+      <c r="I962" s="120"/>
       <c r="J962" s="35" t="s">
         <v>2606</v>
       </c>
-      <c r="K962" s="124"/>
-      <c r="L962" s="130"/>
-      <c r="M962" s="124"/>
+      <c r="K962" s="29"/>
+      <c r="L962" s="31"/>
+      <c r="M962" s="29"/>
     </row>
     <row r="963" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A963" s="124" t="s">
+      <c r="A963" s="29" t="s">
         <v>1257</v>
       </c>
-      <c r="B963" s="128" t="s">
+      <c r="B963" s="100" t="s">
         <v>2616</v>
       </c>
-      <c r="C963" s="122"/>
-      <c r="D963" s="123" t="s">
+      <c r="C963" s="83"/>
+      <c r="D963" s="85" t="s">
         <v>2605</v>
       </c>
-      <c r="E963" s="122" t="s">
+      <c r="E963" s="83" t="s">
         <v>871</v>
       </c>
-      <c r="F963" s="130"/>
-      <c r="G963" s="130"/>
-      <c r="H963" s="129"/>
-      <c r="I963" s="125"/>
+      <c r="F963" s="31"/>
+      <c r="G963" s="31"/>
+      <c r="H963" s="29"/>
+      <c r="I963" s="120"/>
       <c r="J963" s="33" t="s">
         <v>2607</v>
       </c>
-      <c r="K963" s="124"/>
-      <c r="L963" s="130"/>
-      <c r="M963" s="124"/>
+      <c r="K963" s="29"/>
+      <c r="L963" s="31"/>
+      <c r="M963" s="29"/>
     </row>
     <row r="964" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A964" s="124" t="s">
+      <c r="A964" s="29" t="s">
         <v>1259</v>
       </c>
-      <c r="B964" s="128" t="s">
+      <c r="B964" s="100" t="s">
         <v>2617</v>
       </c>
-      <c r="C964" s="122"/>
-      <c r="D964" s="123" t="s">
+      <c r="C964" s="83"/>
+      <c r="D964" s="85" t="s">
         <v>2605</v>
       </c>
-      <c r="E964" s="122" t="s">
+      <c r="E964" s="83" t="s">
         <v>872</v>
       </c>
-      <c r="F964" s="130"/>
-      <c r="G964" s="130"/>
-      <c r="H964" s="129"/>
-      <c r="I964" s="125"/>
+      <c r="F964" s="31"/>
+      <c r="G964" s="31"/>
+      <c r="H964" s="29"/>
+      <c r="I964" s="120"/>
       <c r="J964" s="33" t="s">
         <v>2607</v>
       </c>
-      <c r="K964" s="124"/>
-      <c r="L964" s="130"/>
-      <c r="M964" s="124"/>
+      <c r="K964" s="29"/>
+      <c r="L964" s="31"/>
+      <c r="M964" s="29"/>
     </row>
     <row r="965" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A965" s="124" t="s">
+      <c r="A965" s="29" t="s">
         <v>2615</v>
       </c>
-      <c r="B965" s="128"/>
-      <c r="C965" s="122"/>
-      <c r="D965" s="123" t="s">
+      <c r="B965" s="100"/>
+      <c r="C965" s="83"/>
+      <c r="D965" s="85" t="s">
         <v>2605</v>
       </c>
-      <c r="E965" s="122" t="s">
+      <c r="E965" s="83" t="s">
         <v>2367</v>
       </c>
-      <c r="F965" s="130"/>
-      <c r="G965" s="130"/>
-      <c r="H965" s="129"/>
-      <c r="I965" s="125"/>
+      <c r="F965" s="31"/>
+      <c r="G965" s="31"/>
+      <c r="H965" s="29"/>
+      <c r="I965" s="120"/>
       <c r="J965" s="19" t="s">
         <v>1077</v>
       </c>
-      <c r="K965" s="124"/>
-      <c r="L965" s="130"/>
-      <c r="M965" s="124"/>
+      <c r="K965" s="29"/>
+      <c r="L965" s="31"/>
+      <c r="M965" s="29"/>
     </row>
     <row r="966" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A966" s="124" t="s">
+      <c r="A966" s="29" t="s">
         <v>2614</v>
       </c>
       <c r="B966" s="113"/>
-      <c r="C966" s="131"/>
+      <c r="C966" s="121"/>
       <c r="D966" s="79" t="s">
         <v>2605</v>
       </c>
       <c r="E966" s="80" t="s">
         <v>2610</v>
       </c>
-      <c r="F966" s="130"/>
-      <c r="G966" s="130"/>
-      <c r="H966" s="127"/>
+      <c r="F966" s="31"/>
+      <c r="G966" s="31"/>
+      <c r="H966" s="23"/>
       <c r="I966" s="19"/>
       <c r="J966" s="35" t="s">
         <v>1077</v>
       </c>
-      <c r="K966" s="124"/>
-      <c r="L966" s="130"/>
-      <c r="M966" s="124"/>
+      <c r="K966" s="29"/>
+      <c r="L966" s="31"/>
+      <c r="M966" s="29"/>
     </row>
     <row r="967" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A967" s="124" t="s">
+      <c r="A967" s="29" t="s">
         <v>1741</v>
       </c>
-      <c r="B967" s="128" t="s">
+      <c r="B967" s="100" t="s">
         <v>2618</v>
       </c>
-      <c r="C967" s="132"/>
-      <c r="D967" s="123" t="s">
+      <c r="C967" s="122"/>
+      <c r="D967" s="85" t="s">
         <v>2605</v>
       </c>
       <c r="E967" s="69" t="s">
         <v>2611</v>
       </c>
-      <c r="F967" s="130"/>
-      <c r="G967" s="130"/>
-      <c r="H967" s="129"/>
-      <c r="I967" s="125"/>
+      <c r="F967" s="31"/>
+      <c r="G967" s="31"/>
+      <c r="H967" s="29"/>
+      <c r="I967" s="120"/>
       <c r="J967" s="33" t="s">
         <v>2608</v>
       </c>
-      <c r="K967" s="124"/>
-      <c r="L967" s="130"/>
-      <c r="M967" s="124"/>
+      <c r="K967" s="29"/>
+      <c r="L967" s="31"/>
+      <c r="M967" s="29"/>
     </row>
     <row r="968" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A968" s="124" t="s">
+      <c r="A968" s="29" t="s">
         <v>2613</v>
       </c>
-      <c r="B968" s="128" t="s">
+      <c r="B968" s="100" t="s">
         <v>2619</v>
       </c>
-      <c r="C968" s="133"/>
-      <c r="D968" s="123" t="s">
+      <c r="C968" s="123"/>
+      <c r="D968" s="85" t="s">
         <v>2605</v>
       </c>
-      <c r="E968" s="136" t="s">
+      <c r="E968" s="125" t="s">
         <v>2612</v>
       </c>
-      <c r="F968" s="130"/>
-      <c r="G968" s="130"/>
-      <c r="H968" s="129"/>
-      <c r="I968" s="125"/>
+      <c r="F968" s="31"/>
+      <c r="G968" s="31"/>
+      <c r="H968" s="29"/>
+      <c r="I968" s="120"/>
       <c r="J968" s="35" t="s">
         <v>2609</v>
       </c>
-      <c r="K968" s="124"/>
-      <c r="L968" s="130"/>
-      <c r="M968" s="124"/>
+      <c r="K968" s="29"/>
+      <c r="L968" s="31"/>
+      <c r="M968" s="29"/>
     </row>
     <row r="969" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A969" s="120" t="s">
+      <c r="A969" t="s">
         <v>2566</v>
       </c>
       <c r="B969" s="15" t="s">
         <v>1463</v>
       </c>
-      <c r="C969" s="121"/>
       <c r="D969" s="15" t="s">
         <v>2567</v>
       </c>
-      <c r="E969" s="120"/>
-      <c r="F969" s="120" t="s">
+      <c r="F969" t="s">
         <v>1771</v>
       </c>
-      <c r="G969" s="120" t="s">
+      <c r="G969" t="s">
         <v>2568</v>
       </c>
-      <c r="H969" s="120" t="s">
+      <c r="H969" t="s">
         <v>1359</v>
       </c>
-      <c r="I969" s="120" t="s">
+      <c r="I969" t="s">
         <v>71</v>
       </c>
-      <c r="J969" s="120" t="s">
+      <c r="J969" t="s">
         <v>2569</v>
       </c>
-      <c r="K969" s="124"/>
-      <c r="L969" s="130"/>
-      <c r="M969" s="124"/>
+      <c r="K969" s="29"/>
+      <c r="L969" s="31"/>
+      <c r="M969" s="29"/>
     </row>
     <row r="970" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A970" s="124"/>
-      <c r="B970" s="128"/>
-      <c r="C970" s="134"/>
-      <c r="D970" s="135"/>
-      <c r="E970" s="122"/>
-      <c r="F970" s="130"/>
-      <c r="G970" s="130"/>
-      <c r="H970" s="129"/>
-      <c r="I970" s="125"/>
-      <c r="J970" s="124"/>
-      <c r="K970" s="124"/>
-      <c r="L970" s="130"/>
-      <c r="M970" s="124"/>
+      <c r="A970" s="29" t="s">
+        <v>2642</v>
+      </c>
+      <c r="B970" s="100" t="s">
+        <v>1043</v>
+      </c>
+      <c r="C970" s="124" t="s">
+        <v>2639</v>
+      </c>
+      <c r="D970" s="85" t="s">
+        <v>1250</v>
+      </c>
+      <c r="E970" s="83" t="s">
+        <v>2638</v>
+      </c>
+      <c r="F970" s="31" t="s">
+        <v>1771</v>
+      </c>
+      <c r="G970" s="31" t="s">
+        <v>2640</v>
+      </c>
+      <c r="H970" s="29">
+        <v>0</v>
+      </c>
+      <c r="I970" s="120" t="s">
+        <v>71</v>
+      </c>
+      <c r="J970" s="29" t="s">
+        <v>2641</v>
+      </c>
+      <c r="K970" s="29"/>
+      <c r="L970" s="31"/>
+      <c r="M970" s="29"/>
     </row>
     <row r="971" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A971" s="29"/>
-      <c r="B971" s="113"/>
-      <c r="C971" s="82"/>
-      <c r="D971" s="79"/>
-      <c r="E971" s="82"/>
-      <c r="F971" s="126"/>
-      <c r="G971" s="126"/>
-      <c r="H971" s="127"/>
-      <c r="I971" s="19"/>
-      <c r="J971" s="29"/>
+      <c r="A971" s="29" t="s">
+        <v>2646</v>
+      </c>
+      <c r="B971" s="113" t="s">
+        <v>1135</v>
+      </c>
+      <c r="C971" s="82" t="s">
+        <v>1228</v>
+      </c>
+      <c r="D971" s="79" t="s">
+        <v>2643</v>
+      </c>
+      <c r="E971" s="82" t="s">
+        <v>230</v>
+      </c>
+      <c r="F971" s="31" t="s">
+        <v>1772</v>
+      </c>
+      <c r="G971" s="31" t="s">
+        <v>35</v>
+      </c>
+      <c r="H971" s="23" t="s">
+        <v>2647</v>
+      </c>
+      <c r="I971" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="J971" s="29" t="s">
+        <v>2645</v>
+      </c>
       <c r="K971" s="29"/>
-      <c r="L971" s="126"/>
+      <c r="L971" s="31" t="s">
+        <v>2648</v>
+      </c>
       <c r="M971" s="29"/>
     </row>
     <row r="972" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A972" s="29"/>
-      <c r="B972" s="128"/>
-      <c r="C972" s="122"/>
-      <c r="D972" s="123"/>
-      <c r="E972" s="122"/>
-      <c r="F972" s="126"/>
-      <c r="G972" s="126"/>
-      <c r="H972" s="129"/>
-      <c r="I972" s="125"/>
+      <c r="B972" s="100"/>
+      <c r="C972" s="83"/>
+      <c r="D972" s="85"/>
+      <c r="E972" s="83"/>
+      <c r="F972" s="31"/>
+      <c r="G972" s="31"/>
+      <c r="H972" s="29"/>
+      <c r="I972" s="120"/>
       <c r="J972" s="29"/>
       <c r="K972" s="29"/>
-      <c r="L972" s="126"/>
+      <c r="L972" s="31"/>
       <c r="M972" s="29"/>
     </row>
     <row r="973" spans="1:13" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
Added videohub routing for new tv
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43C9FBFF-0FF0-E846-B08C-BF5B18C3C68F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE78FC76-205D-5445-9966-DBDC6D43ED15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3740" yWindow="1740" windowWidth="26500" windowHeight="14260" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
+    <workbookView xWindow="3740" yWindow="1720" windowWidth="26500" windowHeight="14260" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
   <sheets>
     <sheet name="Cables" sheetId="1" r:id="rId1"/>
@@ -46327,7 +46327,7 @@
         <v>1135</v>
       </c>
       <c r="C891" s="83" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="D891" s="83" t="s">
         <v>1135</v>
@@ -46348,7 +46348,7 @@
         <v>71</v>
       </c>
       <c r="J891" s="29" t="s">
-        <v>34</v>
+        <v>2645</v>
       </c>
       <c r="K891" s="29"/>
       <c r="L891" s="31"/>

</xml_diff>

<commit_message>
added missing ndi cable
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1087F3B-767F-F64F-9B35-222FFCEF60AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0D82C1B-214D-C84C-9020-06D0DB94ED72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7120" yWindow="1540" windowWidth="23120" windowHeight="17000" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9128" uniqueCount="2822">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9138" uniqueCount="2825">
   <si>
     <t>Tag</t>
   </si>
@@ -8507,6 +8507,15 @@
   </si>
   <si>
     <t>pt1121</t>
+  </si>
+  <si>
+    <t>2602-2800</t>
+  </si>
+  <si>
+    <t>undoc877</t>
+  </si>
+  <si>
+    <t>Need to record cable id</t>
   </si>
 </sst>
 </file>
@@ -46439,17 +46448,37 @@
       <c r="M876" s="29"/>
     </row>
     <row r="877" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A877" s="29"/>
-      <c r="B877" s="83"/>
-      <c r="C877" s="83"/>
-      <c r="D877" s="85"/>
-      <c r="E877" s="83"/>
-      <c r="F877" s="31"/>
-      <c r="G877" s="31"/>
-      <c r="H877" s="29"/>
-      <c r="I877" s="29"/>
+      <c r="A877" s="29" t="s">
+        <v>2823</v>
+      </c>
+      <c r="B877" s="83" t="s">
+        <v>1121</v>
+      </c>
+      <c r="C877" s="83" t="s">
+        <v>1758</v>
+      </c>
+      <c r="D877" s="85" t="s">
+        <v>2822</v>
+      </c>
+      <c r="E877" s="83" t="s">
+        <v>359</v>
+      </c>
+      <c r="F877" s="31" t="s">
+        <v>1706</v>
+      </c>
+      <c r="G877" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="H877" s="29" t="s">
+        <v>197</v>
+      </c>
+      <c r="I877" s="29" t="s">
+        <v>99</v>
+      </c>
       <c r="J877" s="29"/>
-      <c r="K877" s="29"/>
+      <c r="K877" s="29" t="s">
+        <v>2824</v>
+      </c>
       <c r="L877" s="31"/>
       <c r="M877" s="29"/>
     </row>

</xml_diff>

<commit_message>
corrected incor asset id for 2601-2800
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C0D82C1B-214D-C84C-9020-06D0DB94ED72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D060BD4-17E1-7245-8979-8081A6D8AEAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7120" yWindow="1540" windowWidth="23120" windowHeight="17000" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9138" uniqueCount="2825">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9138" uniqueCount="2824">
   <si>
     <t>Tag</t>
   </si>
@@ -8507,9 +8507,6 @@
   </si>
   <si>
     <t>pt1121</t>
-  </si>
-  <si>
-    <t>2602-2800</t>
   </si>
   <si>
     <t>undoc877</t>
@@ -46449,7 +46446,7 @@
     </row>
     <row r="877" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A877" s="29" t="s">
-        <v>2823</v>
+        <v>2822</v>
       </c>
       <c r="B877" s="83" t="s">
         <v>1121</v>
@@ -46458,7 +46455,7 @@
         <v>1758</v>
       </c>
       <c r="D877" s="85" t="s">
-        <v>2822</v>
+        <v>1123</v>
       </c>
       <c r="E877" s="83" t="s">
         <v>359</v>
@@ -46477,7 +46474,7 @@
       </c>
       <c r="J877" s="29"/>
       <c r="K877" s="29" t="s">
-        <v>2824</v>
+        <v>2823</v>
       </c>
       <c r="L877" s="31"/>
       <c r="M877" s="29"/>

</xml_diff>

<commit_message>
corrected W-cat6-60 thru 63
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DB3EC3D-F758-C044-ADCB-215F8A18BB02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1E2EEBD-7308-5C46-9195-6262185D5291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7120" yWindow="1520" windowWidth="23120" windowHeight="17000" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9897" uniqueCount="2945">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9861" uniqueCount="2941">
   <si>
     <t>Tag</t>
   </si>
@@ -8710,9 +8710,6 @@
     <t>Core</t>
   </si>
   <si>
-    <t>W-CAT6-060</t>
-  </si>
-  <si>
     <t>W-Cat6-060</t>
   </si>
   <si>
@@ -8744,15 +8741,6 @@
   </si>
   <si>
     <t>notag1176</t>
-  </si>
-  <si>
-    <t>W-CAT6-061</t>
-  </si>
-  <si>
-    <t>W-CAT6-062</t>
-  </si>
-  <si>
-    <t>W-CAT6-063</t>
   </si>
   <si>
     <t>W-CAT6-064</t>
@@ -10031,7 +10019,7 @@
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshedBy="Terry Doner" refreshedDate="46030.710642245373" createdVersion="8" refreshedVersion="8" minRefreshableVersion="3" recordCount="442" xr:uid="{966EC718-ADB8-7746-9366-54097C9D57FA}">
   <cacheSource type="worksheet">
-    <worksheetSource ref="A1:M1325" sheet="Cables"/>
+    <worksheetSource ref="A1:M1321" sheet="Cables"/>
   </cacheSource>
   <cacheFields count="12">
     <cacheField name="Tag" numFmtId="0">
@@ -18725,8 +18713,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BD7E3698-8860-904B-8BDB-00EF1039C49C}" name="Table1" displayName="Table1" ref="A1:M1326" totalsRowCount="1" headerRowDxfId="20" dataDxfId="19" tableBorderDxfId="18">
-  <autoFilter ref="A1:M1325" xr:uid="{BD7E3698-8860-904B-8BDB-00EF1039C49C}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BD7E3698-8860-904B-8BDB-00EF1039C49C}" name="Table1" displayName="Table1" ref="A1:M1322" totalsRowCount="1" headerRowDxfId="20" dataDxfId="19" tableBorderDxfId="18">
+  <autoFilter ref="A1:M1321" xr:uid="{BD7E3698-8860-904B-8BDB-00EF1039C49C}"/>
   <tableColumns count="13">
     <tableColumn id="1" xr3:uid="{4D442337-BE86-B24A-84A4-338FB80A6A49}" name="Tag" dataDxfId="17"/>
     <tableColumn id="2" xr3:uid="{74A36D7B-C989-3B4B-B1E5-AB1FA4C2DD45}" name="SrcTag" dataDxfId="16" totalsRowDxfId="4"/>
@@ -19043,7 +19031,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86B91ADC-4569-1C4E-B002-1ED2E647C959}">
-  <dimension ref="A1:W1326"/>
+  <dimension ref="A1:W1322"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.6640625" customWidth="1"/>
@@ -32091,7 +32079,7 @@
     </row>
     <row r="424" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A424" s="29" t="s">
-        <v>2927</v>
+        <v>2923</v>
       </c>
       <c r="B424" s="31" t="s">
         <v>2735</v>
@@ -36091,7 +36079,7 @@
         <v>1823</v>
       </c>
       <c r="C542" s="82" t="s">
-        <v>2909</v>
+        <v>2905</v>
       </c>
       <c r="D542" s="70" t="s">
         <v>1167</v>
@@ -36120,7 +36108,7 @@
         <v>1823</v>
       </c>
       <c r="C543" s="36" t="s">
-        <v>2910</v>
+        <v>2906</v>
       </c>
       <c r="D543" s="70" t="s">
         <v>1168</v>
@@ -56462,7 +56450,7 @@
     </row>
     <row r="1173" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1173" s="29" t="s">
-        <v>2896</v>
+        <v>2895</v>
       </c>
       <c r="B1173" s="135" t="s">
         <v>2860</v>
@@ -56493,7 +56481,7 @@
     </row>
     <row r="1174" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1174" s="29" t="s">
-        <v>2897</v>
+        <v>2896</v>
       </c>
       <c r="B1174" s="135" t="s">
         <v>2860</v>
@@ -56524,7 +56512,7 @@
     </row>
     <row r="1175" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1175" s="29" t="s">
-        <v>2898</v>
+        <v>2897</v>
       </c>
       <c r="B1175" s="135" t="s">
         <v>2860</v>
@@ -56555,7 +56543,7 @@
     </row>
     <row r="1176" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1176" s="29" t="s">
-        <v>2899</v>
+        <v>2898</v>
       </c>
       <c r="B1176" s="135" t="s">
         <v>2860</v>
@@ -56586,7 +56574,7 @@
     </row>
     <row r="1177" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1177" s="29" t="s">
-        <v>2900</v>
+        <v>2899</v>
       </c>
       <c r="B1177" s="135" t="s">
         <v>2860</v>
@@ -56617,16 +56605,16 @@
     </row>
     <row r="1178" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1178" s="29" t="s">
-        <v>2890</v>
+        <v>2889</v>
       </c>
       <c r="B1178" s="135" t="s">
         <v>2860</v>
       </c>
       <c r="C1178" s="125" t="s">
-        <v>2650</v>
+        <v>2657</v>
       </c>
       <c r="D1178" s="126" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="E1178" s="125" t="s">
         <v>2106</v>
@@ -56644,7 +56632,7 @@
         <v>63</v>
       </c>
       <c r="J1178" s="29" t="s">
-        <v>2890</v>
+        <v>2889</v>
       </c>
       <c r="K1178" s="29"/>
       <c r="L1178" s="127"/>
@@ -56652,16 +56640,16 @@
     </row>
     <row r="1179" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1179" s="29" t="s">
-        <v>2891</v>
+        <v>2890</v>
       </c>
       <c r="B1179" s="135" t="s">
         <v>2860</v>
       </c>
       <c r="C1179" s="125" t="s">
-        <v>2651</v>
+        <v>2658</v>
       </c>
       <c r="D1179" s="126" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="E1179" s="125" t="s">
         <v>2657</v>
@@ -56679,7 +56667,7 @@
         <v>63</v>
       </c>
       <c r="J1179" s="29" t="s">
-        <v>2891</v>
+        <v>2890</v>
       </c>
       <c r="K1179" s="29"/>
       <c r="L1179" s="127"/>
@@ -56687,16 +56675,16 @@
     </row>
     <row r="1180" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1180" s="29" t="s">
-        <v>2892</v>
+        <v>2891</v>
       </c>
       <c r="B1180" s="135" t="s">
         <v>2860</v>
       </c>
       <c r="C1180" s="125" t="s">
-        <v>2652</v>
+        <v>2659</v>
       </c>
       <c r="D1180" s="126" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="E1180" s="125" t="s">
         <v>2658</v>
@@ -56714,7 +56702,7 @@
         <v>63</v>
       </c>
       <c r="J1180" s="29" t="s">
-        <v>2892</v>
+        <v>2891</v>
       </c>
       <c r="K1180" s="29"/>
       <c r="L1180" s="127"/>
@@ -56722,16 +56710,16 @@
     </row>
     <row r="1181" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1181" s="29" t="s">
-        <v>2893</v>
+        <v>2892</v>
       </c>
       <c r="B1181" s="135" t="s">
         <v>2860</v>
       </c>
       <c r="C1181" s="125" t="s">
-        <v>2653</v>
+        <v>2660</v>
       </c>
       <c r="D1181" s="126" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="E1181" s="125" t="s">
         <v>2659</v>
@@ -56749,7 +56737,7 @@
         <v>63</v>
       </c>
       <c r="J1181" s="29" t="s">
-        <v>2893</v>
+        <v>2892</v>
       </c>
       <c r="K1181" s="29"/>
       <c r="L1181" s="127"/>
@@ -56757,7 +56745,7 @@
     </row>
     <row r="1182" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1182" s="29" t="s">
-        <v>2894</v>
+        <v>2893</v>
       </c>
       <c r="B1182" s="135" t="s">
         <v>2860</v>
@@ -56774,7 +56762,7 @@
         <v>63</v>
       </c>
       <c r="J1182" s="29" t="s">
-        <v>2894</v>
+        <v>2893</v>
       </c>
       <c r="K1182" s="29" t="s">
         <v>452</v>
@@ -56782,9 +56770,9 @@
       <c r="L1182" s="127"/>
       <c r="M1182" s="29"/>
     </row>
-    <row r="1183" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1183" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1183" s="29" t="s">
-        <v>2895</v>
+        <v>2894</v>
       </c>
       <c r="B1183" s="135" t="s">
         <v>2860</v>
@@ -56801,7 +56789,7 @@
         <v>63</v>
       </c>
       <c r="J1183" s="29" t="s">
-        <v>2895</v>
+        <v>2894</v>
       </c>
       <c r="K1183" s="29" t="s">
         <v>452</v>
@@ -56809,21 +56797,21 @@
       <c r="L1183" s="127"/>
       <c r="M1183" s="29"/>
     </row>
-    <row r="1184" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1184" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A1184" s="29" t="s">
-        <v>2889</v>
-      </c>
-      <c r="B1184" s="135" t="s">
-        <v>2860</v>
+        <v>2900</v>
+      </c>
+      <c r="B1184" s="126" t="s">
+        <v>2926</v>
       </c>
       <c r="C1184" s="125" t="s">
-        <v>2657</v>
-      </c>
-      <c r="D1184" s="126" t="s">
-        <v>2930</v>
+        <v>2660</v>
+      </c>
+      <c r="D1184" s="79" t="s">
+        <v>2735</v>
       </c>
       <c r="E1184" s="125" t="s">
-        <v>1341</v>
+        <v>2644</v>
       </c>
       <c r="F1184" s="127" t="s">
         <v>1800</v>
@@ -56838,7 +56826,9 @@
         <v>99</v>
       </c>
       <c r="J1184" s="29"/>
-      <c r="K1184" s="29"/>
+      <c r="K1184" s="29" t="s">
+        <v>2904</v>
+      </c>
       <c r="L1184" s="127"/>
       <c r="M1184" s="29"/>
     </row>
@@ -56846,17 +56836,17 @@
       <c r="A1185" s="29" t="s">
         <v>2901</v>
       </c>
-      <c r="B1185" s="135" t="s">
-        <v>2860</v>
+      <c r="B1185" s="126" t="s">
+        <v>2926</v>
       </c>
       <c r="C1185" s="125" t="s">
-        <v>2658</v>
+        <v>2661</v>
       </c>
       <c r="D1185" s="126" t="s">
-        <v>2930</v>
+        <v>2735</v>
       </c>
       <c r="E1185" s="125" t="s">
-        <v>1342</v>
+        <v>2102</v>
       </c>
       <c r="F1185" s="127" t="s">
         <v>1800</v>
@@ -56871,7 +56861,9 @@
         <v>99</v>
       </c>
       <c r="J1185" s="29"/>
-      <c r="K1185" s="29"/>
+      <c r="K1185" s="29" t="s">
+        <v>2904</v>
+      </c>
       <c r="L1185" s="127"/>
       <c r="M1185" s="29"/>
     </row>
@@ -56879,17 +56871,17 @@
       <c r="A1186" s="29" t="s">
         <v>2902</v>
       </c>
-      <c r="B1186" s="135" t="s">
-        <v>2860</v>
+      <c r="B1186" s="126" t="s">
+        <v>2926</v>
       </c>
       <c r="C1186" s="125" t="s">
-        <v>2659</v>
+        <v>2662</v>
       </c>
       <c r="D1186" s="126" t="s">
-        <v>2930</v>
+        <v>2735</v>
       </c>
       <c r="E1186" s="125" t="s">
-        <v>1343</v>
+        <v>2552</v>
       </c>
       <c r="F1186" s="127" t="s">
         <v>1800</v>
@@ -56904,7 +56896,9 @@
         <v>99</v>
       </c>
       <c r="J1186" s="29"/>
-      <c r="K1186" s="29"/>
+      <c r="K1186" s="29" t="s">
+        <v>2904</v>
+      </c>
       <c r="L1186" s="127"/>
       <c r="M1186" s="29"/>
     </row>
@@ -56912,20 +56906,20 @@
       <c r="A1187" s="29" t="s">
         <v>2903</v>
       </c>
-      <c r="B1187" s="135" t="s">
-        <v>2860</v>
+      <c r="B1187" s="126" t="s">
+        <v>2926</v>
       </c>
       <c r="C1187" s="125" t="s">
-        <v>2660</v>
+        <v>2663</v>
       </c>
       <c r="D1187" s="126" t="s">
-        <v>2930</v>
+        <v>2735</v>
       </c>
       <c r="E1187" s="125" t="s">
-        <v>1344</v>
+        <v>2286</v>
       </c>
       <c r="F1187" s="127" t="s">
-        <v>1800</v>
+        <v>479</v>
       </c>
       <c r="G1187" s="127" t="s">
         <v>1611</v>
@@ -56937,29 +56931,29 @@
         <v>99</v>
       </c>
       <c r="J1187" s="29"/>
-      <c r="K1187" s="29"/>
+      <c r="K1187" s="29" t="s">
+        <v>2904</v>
+      </c>
       <c r="L1187" s="127"/>
       <c r="M1187" s="29"/>
     </row>
     <row r="1188" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A1188" s="29" t="s">
-        <v>2904</v>
-      </c>
-      <c r="B1188" s="126" t="s">
-        <v>2930</v>
+        <v>2907</v>
+      </c>
+      <c r="B1188" s="80" t="s">
+        <v>2908</v>
       </c>
       <c r="C1188" s="125" t="s">
-        <v>2660</v>
-      </c>
-      <c r="D1188" s="79" t="s">
-        <v>2735</v>
+        <v>2909</v>
+      </c>
+      <c r="D1188" s="126" t="s">
+        <v>2910</v>
       </c>
       <c r="E1188" s="125" t="s">
-        <v>2644</v>
-      </c>
-      <c r="F1188" s="127" t="s">
-        <v>1800</v>
-      </c>
+        <v>2911</v>
+      </c>
+      <c r="F1188" s="127"/>
       <c r="G1188" s="127" t="s">
         <v>1611</v>
       </c>
@@ -56967,34 +56961,30 @@
         <v>26</v>
       </c>
       <c r="I1188" s="119" t="s">
-        <v>99</v>
+        <v>519</v>
       </c>
       <c r="J1188" s="29"/>
-      <c r="K1188" s="29" t="s">
-        <v>2908</v>
-      </c>
+      <c r="K1188" s="29"/>
       <c r="L1188" s="127"/>
       <c r="M1188" s="29"/>
     </row>
     <row r="1189" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1189" s="29" t="s">
-        <v>2905</v>
+        <v>2913</v>
       </c>
       <c r="B1189" s="126" t="s">
-        <v>2930</v>
+        <v>2910</v>
       </c>
       <c r="C1189" s="125" t="s">
-        <v>2661</v>
+        <v>2434</v>
       </c>
       <c r="D1189" s="126" t="s">
-        <v>2735</v>
+        <v>1823</v>
       </c>
       <c r="E1189" s="125" t="s">
-        <v>2102</v>
-      </c>
-      <c r="F1189" s="127" t="s">
-        <v>1800</v>
-      </c>
+        <v>2912</v>
+      </c>
+      <c r="F1189" s="127"/>
       <c r="G1189" s="127" t="s">
         <v>1611</v>
       </c>
@@ -57002,30 +56992,28 @@
         <v>26</v>
       </c>
       <c r="I1189" s="119" t="s">
-        <v>99</v>
+        <v>519</v>
       </c>
       <c r="J1189" s="29"/>
-      <c r="K1189" s="29" t="s">
-        <v>2908</v>
-      </c>
+      <c r="K1189" s="29"/>
       <c r="L1189" s="127"/>
       <c r="M1189" s="29"/>
     </row>
     <row r="1190" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1190" s="29" t="s">
-        <v>2906</v>
-      </c>
-      <c r="B1190" s="126" t="s">
-        <v>2930</v>
+        <v>2916</v>
+      </c>
+      <c r="B1190" s="135" t="s">
+        <v>1823</v>
       </c>
       <c r="C1190" s="125" t="s">
-        <v>2662</v>
+        <v>2915</v>
       </c>
       <c r="D1190" s="126" t="s">
-        <v>2735</v>
+        <v>2914</v>
       </c>
       <c r="E1190" s="125" t="s">
-        <v>2552</v>
+        <v>2434</v>
       </c>
       <c r="F1190" s="127" t="s">
         <v>1800</v>
@@ -57037,33 +57025,31 @@
         <v>26</v>
       </c>
       <c r="I1190" s="119" t="s">
-        <v>99</v>
+        <v>63</v>
       </c>
       <c r="J1190" s="29"/>
-      <c r="K1190" s="29" t="s">
-        <v>2908</v>
-      </c>
+      <c r="K1190" s="29"/>
       <c r="L1190" s="127"/>
       <c r="M1190" s="29"/>
     </row>
-    <row r="1191" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="1191" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1191" s="29" t="s">
-        <v>2907</v>
-      </c>
-      <c r="B1191" s="126" t="s">
-        <v>2930</v>
+        <v>2919</v>
+      </c>
+      <c r="B1191" s="135" t="s">
+        <v>1823</v>
       </c>
       <c r="C1191" s="125" t="s">
-        <v>2663</v>
+        <v>2917</v>
       </c>
       <c r="D1191" s="126" t="s">
-        <v>2735</v>
+        <v>2918</v>
       </c>
       <c r="E1191" s="125" t="s">
-        <v>2286</v>
+        <v>1611</v>
       </c>
       <c r="F1191" s="127" t="s">
-        <v>479</v>
+        <v>1800</v>
       </c>
       <c r="G1191" s="127" t="s">
         <v>1611</v>
@@ -57072,92 +57058,82 @@
         <v>26</v>
       </c>
       <c r="I1191" s="119" t="s">
-        <v>99</v>
+        <v>63</v>
       </c>
       <c r="J1191" s="29"/>
-      <c r="K1191" s="29" t="s">
-        <v>2908</v>
-      </c>
+      <c r="K1191" s="29"/>
       <c r="L1191" s="127"/>
       <c r="M1191" s="29"/>
     </row>
-    <row r="1192" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="1192" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1192" s="29" t="s">
-        <v>2911</v>
-      </c>
-      <c r="B1192" s="80" t="s">
-        <v>2912</v>
-      </c>
-      <c r="C1192" s="125" t="s">
-        <v>2913</v>
-      </c>
-      <c r="D1192" s="126" t="s">
-        <v>2914</v>
-      </c>
-      <c r="E1192" s="125" t="s">
-        <v>2915</v>
-      </c>
-      <c r="F1192" s="127"/>
+        <v>2920</v>
+      </c>
+      <c r="B1192" s="135"/>
+      <c r="C1192" s="125"/>
+      <c r="D1192" s="126"/>
+      <c r="E1192" s="125"/>
+      <c r="F1192" s="127" t="s">
+        <v>30</v>
+      </c>
       <c r="G1192" s="127" t="s">
-        <v>1611</v>
+        <v>30</v>
       </c>
       <c r="H1192" s="128" t="s">
-        <v>26</v>
+        <v>667</v>
       </c>
       <c r="I1192" s="119" t="s">
-        <v>519</v>
+        <v>99</v>
       </c>
       <c r="J1192" s="29"/>
-      <c r="K1192" s="29"/>
-      <c r="L1192" s="127"/>
+      <c r="K1192" s="29" t="s">
+        <v>452</v>
+      </c>
+      <c r="L1192" s="127" t="s">
+        <v>652</v>
+      </c>
       <c r="M1192" s="29"/>
     </row>
     <row r="1193" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1193" s="29" t="s">
-        <v>2917</v>
-      </c>
-      <c r="B1193" s="126" t="s">
-        <v>2914</v>
-      </c>
-      <c r="C1193" s="125" t="s">
-        <v>2434</v>
-      </c>
-      <c r="D1193" s="126" t="s">
-        <v>1823</v>
-      </c>
-      <c r="E1193" s="125" t="s">
-        <v>2916</v>
-      </c>
-      <c r="F1193" s="127"/>
+        <v>2921</v>
+      </c>
+      <c r="B1193" s="135"/>
+      <c r="C1193" s="125"/>
+      <c r="D1193" s="126"/>
+      <c r="E1193" s="125"/>
+      <c r="F1193" s="127" t="s">
+        <v>30</v>
+      </c>
       <c r="G1193" s="127" t="s">
-        <v>1611</v>
+        <v>30</v>
       </c>
       <c r="H1193" s="128" t="s">
-        <v>26</v>
+        <v>2922</v>
       </c>
       <c r="I1193" s="119" t="s">
-        <v>519</v>
+        <v>99</v>
       </c>
       <c r="J1193" s="29"/>
-      <c r="K1193" s="29"/>
-      <c r="L1193" s="127"/>
+      <c r="K1193" s="29" t="s">
+        <v>452</v>
+      </c>
+      <c r="L1193" s="127" t="s">
+        <v>652</v>
+      </c>
       <c r="M1193" s="29"/>
     </row>
     <row r="1194" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1194" s="29" t="s">
-        <v>2920</v>
-      </c>
-      <c r="B1194" s="135" t="s">
-        <v>1823</v>
-      </c>
-      <c r="C1194" s="125" t="s">
-        <v>2919</v>
-      </c>
+        <v>2924</v>
+      </c>
+      <c r="B1194" s="135"/>
+      <c r="C1194" s="125"/>
       <c r="D1194" s="126" t="s">
-        <v>2918</v>
+        <v>2735</v>
       </c>
       <c r="E1194" s="125" t="s">
-        <v>2434</v>
+        <v>2642</v>
       </c>
       <c r="F1194" s="127" t="s">
         <v>1800</v>
@@ -57169,7 +57145,7 @@
         <v>26</v>
       </c>
       <c r="I1194" s="119" t="s">
-        <v>63</v>
+        <v>99</v>
       </c>
       <c r="J1194" s="29"/>
       <c r="K1194" s="29"/>
@@ -57178,19 +57154,15 @@
     </row>
     <row r="1195" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1195" s="29" t="s">
-        <v>2923</v>
-      </c>
-      <c r="B1195" s="135" t="s">
-        <v>1823</v>
-      </c>
-      <c r="C1195" s="125" t="s">
-        <v>2921</v>
-      </c>
+        <v>2925</v>
+      </c>
+      <c r="B1195" s="135"/>
+      <c r="C1195" s="125"/>
       <c r="D1195" s="126" t="s">
-        <v>2922</v>
+        <v>2735</v>
       </c>
       <c r="E1195" s="125" t="s">
-        <v>1611</v>
+        <v>2643</v>
       </c>
       <c r="F1195" s="127" t="s">
         <v>1800</v>
@@ -57202,7 +57174,7 @@
         <v>26</v>
       </c>
       <c r="I1195" s="119" t="s">
-        <v>63</v>
+        <v>99</v>
       </c>
       <c r="J1195" s="29"/>
       <c r="K1195" s="29"/>
@@ -57211,85 +57183,97 @@
     </row>
     <row r="1196" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1196" s="29" t="s">
-        <v>2924</v>
-      </c>
-      <c r="B1196" s="135"/>
-      <c r="C1196" s="125"/>
-      <c r="D1196" s="126"/>
-      <c r="E1196" s="125"/>
+        <v>2927</v>
+      </c>
+      <c r="B1196" s="135" t="s">
+        <v>2926</v>
+      </c>
+      <c r="C1196" s="125" t="s">
+        <v>2526</v>
+      </c>
+      <c r="D1196" s="135" t="s">
+        <v>2926</v>
+      </c>
+      <c r="E1196" s="125" t="s">
+        <v>2556</v>
+      </c>
       <c r="F1196" s="127" t="s">
-        <v>30</v>
+        <v>2646</v>
       </c>
       <c r="G1196" s="127" t="s">
-        <v>30</v>
-      </c>
-      <c r="H1196" s="128" t="s">
-        <v>667</v>
+        <v>1611</v>
+      </c>
+      <c r="H1196" s="128">
+        <v>0</v>
       </c>
       <c r="I1196" s="119" t="s">
-        <v>99</v>
+        <v>519</v>
       </c>
       <c r="J1196" s="29"/>
-      <c r="K1196" s="29" t="s">
-        <v>452</v>
-      </c>
-      <c r="L1196" s="127" t="s">
-        <v>652</v>
-      </c>
+      <c r="K1196" s="29"/>
+      <c r="L1196" s="127"/>
       <c r="M1196" s="29"/>
     </row>
     <row r="1197" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1197" s="29" t="s">
-        <v>2925</v>
-      </c>
-      <c r="B1197" s="135"/>
-      <c r="C1197" s="125"/>
-      <c r="D1197" s="126"/>
-      <c r="E1197" s="125"/>
+        <v>2928</v>
+      </c>
+      <c r="B1197" s="135" t="s">
+        <v>2926</v>
+      </c>
+      <c r="C1197" s="125" t="s">
+        <v>2525</v>
+      </c>
+      <c r="D1197" s="135" t="s">
+        <v>2926</v>
+      </c>
+      <c r="E1197" s="125" t="s">
+        <v>2645</v>
+      </c>
       <c r="F1197" s="127" t="s">
-        <v>30</v>
+        <v>2646</v>
       </c>
       <c r="G1197" s="127" t="s">
-        <v>30</v>
-      </c>
-      <c r="H1197" s="128" t="s">
-        <v>2926</v>
+        <v>1611</v>
+      </c>
+      <c r="H1197" s="128">
+        <v>0</v>
       </c>
       <c r="I1197" s="119" t="s">
-        <v>99</v>
+        <v>519</v>
       </c>
       <c r="J1197" s="29"/>
-      <c r="K1197" s="29" t="s">
-        <v>452</v>
-      </c>
-      <c r="L1197" s="127" t="s">
-        <v>652</v>
-      </c>
+      <c r="K1197" s="29"/>
+      <c r="L1197" s="127"/>
       <c r="M1197" s="29"/>
     </row>
     <row r="1198" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1198" s="29" t="s">
-        <v>2928</v>
-      </c>
-      <c r="B1198" s="135"/>
-      <c r="C1198" s="125"/>
-      <c r="D1198" s="126" t="s">
-        <v>2735</v>
+        <v>2929</v>
+      </c>
+      <c r="B1198" s="135" t="s">
+        <v>2926</v>
+      </c>
+      <c r="C1198" s="125" t="s">
+        <v>2109</v>
+      </c>
+      <c r="D1198" s="135" t="s">
+        <v>2926</v>
       </c>
       <c r="E1198" s="125" t="s">
-        <v>2642</v>
+        <v>2106</v>
       </c>
       <c r="F1198" s="127" t="s">
-        <v>1800</v>
+        <v>2646</v>
       </c>
       <c r="G1198" s="127" t="s">
         <v>1611</v>
       </c>
-      <c r="H1198" s="128" t="s">
-        <v>26</v>
+      <c r="H1198" s="128">
+        <v>0</v>
       </c>
       <c r="I1198" s="119" t="s">
-        <v>99</v>
+        <v>519</v>
       </c>
       <c r="J1198" s="29"/>
       <c r="K1198" s="29"/>
@@ -57298,27 +57282,31 @@
     </row>
     <row r="1199" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1199" s="29" t="s">
-        <v>2929</v>
-      </c>
-      <c r="B1199" s="135"/>
-      <c r="C1199" s="125"/>
-      <c r="D1199" s="126" t="s">
-        <v>2735</v>
+        <v>2930</v>
+      </c>
+      <c r="B1199" s="135" t="s">
+        <v>2926</v>
+      </c>
+      <c r="C1199" s="125" t="s">
+        <v>2650</v>
+      </c>
+      <c r="D1199" s="135" t="s">
+        <v>2926</v>
       </c>
       <c r="E1199" s="125" t="s">
-        <v>2643</v>
+        <v>2657</v>
       </c>
       <c r="F1199" s="127" t="s">
-        <v>1800</v>
+        <v>2646</v>
       </c>
       <c r="G1199" s="127" t="s">
         <v>1611</v>
       </c>
-      <c r="H1199" s="128" t="s">
-        <v>26</v>
+      <c r="H1199" s="128">
+        <v>0</v>
       </c>
       <c r="I1199" s="119" t="s">
-        <v>99</v>
+        <v>519</v>
       </c>
       <c r="J1199" s="29"/>
       <c r="K1199" s="29"/>
@@ -57330,16 +57318,16 @@
         <v>2931</v>
       </c>
       <c r="B1200" s="135" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="C1200" s="125" t="s">
-        <v>2526</v>
+        <v>2651</v>
       </c>
       <c r="D1200" s="135" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="E1200" s="125" t="s">
-        <v>2556</v>
+        <v>2658</v>
       </c>
       <c r="F1200" s="127" t="s">
         <v>2646</v>
@@ -57363,16 +57351,16 @@
         <v>2932</v>
       </c>
       <c r="B1201" s="135" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="C1201" s="125" t="s">
-        <v>2525</v>
+        <v>2652</v>
       </c>
       <c r="D1201" s="135" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="E1201" s="125" t="s">
-        <v>2645</v>
+        <v>2659</v>
       </c>
       <c r="F1201" s="127" t="s">
         <v>2646</v>
@@ -57396,16 +57384,16 @@
         <v>2933</v>
       </c>
       <c r="B1202" s="135" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="C1202" s="125" t="s">
-        <v>2109</v>
+        <v>2653</v>
       </c>
       <c r="D1202" s="135" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="E1202" s="125" t="s">
-        <v>2106</v>
+        <v>2660</v>
       </c>
       <c r="F1202" s="127" t="s">
         <v>2646</v>
@@ -57429,16 +57417,16 @@
         <v>2934</v>
       </c>
       <c r="B1203" s="135" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="C1203" s="125" t="s">
-        <v>2650</v>
+        <v>2654</v>
       </c>
       <c r="D1203" s="135" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="E1203" s="125" t="s">
-        <v>2657</v>
+        <v>2661</v>
       </c>
       <c r="F1203" s="127" t="s">
         <v>2646</v>
@@ -57462,16 +57450,16 @@
         <v>2935</v>
       </c>
       <c r="B1204" s="135" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="C1204" s="125" t="s">
-        <v>2651</v>
+        <v>2655</v>
       </c>
       <c r="D1204" s="135" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="E1204" s="125" t="s">
-        <v>2658</v>
+        <v>2662</v>
       </c>
       <c r="F1204" s="127" t="s">
         <v>2646</v>
@@ -57495,16 +57483,16 @@
         <v>2936</v>
       </c>
       <c r="B1205" s="135" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="C1205" s="125" t="s">
-        <v>2652</v>
+        <v>2656</v>
       </c>
       <c r="D1205" s="135" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="E1205" s="125" t="s">
-        <v>2659</v>
+        <v>2663</v>
       </c>
       <c r="F1205" s="127" t="s">
         <v>2646</v>
@@ -57528,25 +57516,25 @@
         <v>2937</v>
       </c>
       <c r="B1206" s="135" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="C1206" s="125" t="s">
+        <v>2109</v>
+      </c>
+      <c r="D1206" s="135" t="s">
+        <v>2926</v>
+      </c>
+      <c r="E1206" s="125" t="s">
         <v>2653</v>
       </c>
-      <c r="D1206" s="135" t="s">
-        <v>2930</v>
-      </c>
-      <c r="E1206" s="125" t="s">
-        <v>2660</v>
-      </c>
       <c r="F1206" s="127" t="s">
-        <v>2646</v>
+        <v>1800</v>
       </c>
       <c r="G1206" s="127" t="s">
         <v>1611</v>
       </c>
-      <c r="H1206" s="128">
-        <v>0</v>
+      <c r="H1206" s="128" t="s">
+        <v>1780</v>
       </c>
       <c r="I1206" s="119" t="s">
         <v>519</v>
@@ -57561,25 +57549,25 @@
         <v>2938</v>
       </c>
       <c r="B1207" s="135" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="C1207" s="125" t="s">
+        <v>2650</v>
+      </c>
+      <c r="D1207" s="135" t="s">
+        <v>2926</v>
+      </c>
+      <c r="E1207" s="125" t="s">
         <v>2654</v>
       </c>
-      <c r="D1207" s="135" t="s">
-        <v>2930</v>
-      </c>
-      <c r="E1207" s="125" t="s">
-        <v>2661</v>
-      </c>
       <c r="F1207" s="127" t="s">
-        <v>2646</v>
+        <v>1800</v>
       </c>
       <c r="G1207" s="127" t="s">
         <v>1611</v>
       </c>
-      <c r="H1207" s="128">
-        <v>0</v>
+      <c r="H1207" s="128" t="s">
+        <v>1780</v>
       </c>
       <c r="I1207" s="119" t="s">
         <v>519</v>
@@ -57594,25 +57582,25 @@
         <v>2939</v>
       </c>
       <c r="B1208" s="135" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="C1208" s="125" t="s">
+        <v>2651</v>
+      </c>
+      <c r="D1208" s="135" t="s">
+        <v>2926</v>
+      </c>
+      <c r="E1208" s="125" t="s">
         <v>2655</v>
       </c>
-      <c r="D1208" s="135" t="s">
-        <v>2930</v>
-      </c>
-      <c r="E1208" s="125" t="s">
-        <v>2662</v>
-      </c>
       <c r="F1208" s="127" t="s">
-        <v>2646</v>
+        <v>1800</v>
       </c>
       <c r="G1208" s="127" t="s">
         <v>1611</v>
       </c>
-      <c r="H1208" s="128">
-        <v>0</v>
+      <c r="H1208" s="128" t="s">
+        <v>1780</v>
       </c>
       <c r="I1208" s="119" t="s">
         <v>519</v>
@@ -57627,25 +57615,25 @@
         <v>2940</v>
       </c>
       <c r="B1209" s="135" t="s">
-        <v>2930</v>
+        <v>2926</v>
       </c>
       <c r="C1209" s="125" t="s">
+        <v>2652</v>
+      </c>
+      <c r="D1209" s="135" t="s">
+        <v>2926</v>
+      </c>
+      <c r="E1209" s="125" t="s">
         <v>2656</v>
       </c>
-      <c r="D1209" s="135" t="s">
-        <v>2930</v>
-      </c>
-      <c r="E1209" s="125" t="s">
-        <v>2663</v>
-      </c>
       <c r="F1209" s="127" t="s">
-        <v>2646</v>
+        <v>1800</v>
       </c>
       <c r="G1209" s="127" t="s">
         <v>1611</v>
       </c>
-      <c r="H1209" s="128">
-        <v>0</v>
+      <c r="H1209" s="128" t="s">
+        <v>1780</v>
       </c>
       <c r="I1209" s="119" t="s">
         <v>519</v>
@@ -57656,132 +57644,60 @@
       <c r="M1209" s="29"/>
     </row>
     <row r="1210" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1210" s="29" t="s">
-        <v>2941</v>
-      </c>
-      <c r="B1210" s="135" t="s">
-        <v>2930</v>
-      </c>
-      <c r="C1210" s="125" t="s">
-        <v>2109</v>
-      </c>
-      <c r="D1210" s="135" t="s">
-        <v>2930</v>
-      </c>
-      <c r="E1210" s="125" t="s">
-        <v>2653</v>
-      </c>
-      <c r="F1210" s="127" t="s">
-        <v>1800</v>
-      </c>
-      <c r="G1210" s="127" t="s">
-        <v>1611</v>
-      </c>
-      <c r="H1210" s="128" t="s">
-        <v>1780</v>
-      </c>
-      <c r="I1210" s="119" t="s">
-        <v>519</v>
-      </c>
+      <c r="A1210" s="29"/>
+      <c r="B1210" s="135"/>
+      <c r="C1210" s="125"/>
+      <c r="D1210" s="126"/>
+      <c r="E1210" s="125"/>
+      <c r="F1210" s="127"/>
+      <c r="G1210" s="127"/>
+      <c r="H1210" s="128"/>
+      <c r="I1210" s="119"/>
       <c r="J1210" s="29"/>
       <c r="K1210" s="29"/>
       <c r="L1210" s="127"/>
       <c r="M1210" s="29"/>
     </row>
     <row r="1211" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1211" s="29" t="s">
-        <v>2942</v>
-      </c>
-      <c r="B1211" s="135" t="s">
-        <v>2930</v>
-      </c>
-      <c r="C1211" s="125" t="s">
-        <v>2650</v>
-      </c>
-      <c r="D1211" s="135" t="s">
-        <v>2930</v>
-      </c>
-      <c r="E1211" s="125" t="s">
-        <v>2654</v>
-      </c>
-      <c r="F1211" s="127" t="s">
-        <v>1800</v>
-      </c>
-      <c r="G1211" s="127" t="s">
-        <v>1611</v>
-      </c>
-      <c r="H1211" s="128" t="s">
-        <v>1780</v>
-      </c>
-      <c r="I1211" s="119" t="s">
-        <v>519</v>
-      </c>
+      <c r="A1211" s="29"/>
+      <c r="B1211" s="135"/>
+      <c r="C1211" s="125"/>
+      <c r="D1211" s="126"/>
+      <c r="E1211" s="125"/>
+      <c r="F1211" s="127"/>
+      <c r="G1211" s="127"/>
+      <c r="H1211" s="128"/>
+      <c r="I1211" s="119"/>
       <c r="J1211" s="29"/>
       <c r="K1211" s="29"/>
       <c r="L1211" s="127"/>
       <c r="M1211" s="29"/>
     </row>
     <row r="1212" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1212" s="29" t="s">
-        <v>2943</v>
-      </c>
-      <c r="B1212" s="135" t="s">
-        <v>2930</v>
-      </c>
-      <c r="C1212" s="125" t="s">
-        <v>2651</v>
-      </c>
-      <c r="D1212" s="135" t="s">
-        <v>2930</v>
-      </c>
-      <c r="E1212" s="125" t="s">
-        <v>2655</v>
-      </c>
-      <c r="F1212" s="127" t="s">
-        <v>1800</v>
-      </c>
-      <c r="G1212" s="127" t="s">
-        <v>1611</v>
-      </c>
-      <c r="H1212" s="128" t="s">
-        <v>1780</v>
-      </c>
-      <c r="I1212" s="119" t="s">
-        <v>519</v>
-      </c>
+      <c r="A1212" s="29"/>
+      <c r="B1212" s="135"/>
+      <c r="C1212" s="125"/>
+      <c r="D1212" s="126"/>
+      <c r="E1212" s="125"/>
+      <c r="F1212" s="127"/>
+      <c r="G1212" s="127"/>
+      <c r="H1212" s="128"/>
+      <c r="I1212" s="119"/>
       <c r="J1212" s="29"/>
       <c r="K1212" s="29"/>
       <c r="L1212" s="127"/>
       <c r="M1212" s="29"/>
     </row>
     <row r="1213" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1213" s="29" t="s">
-        <v>2944</v>
-      </c>
-      <c r="B1213" s="135" t="s">
-        <v>2930</v>
-      </c>
-      <c r="C1213" s="125" t="s">
-        <v>2652</v>
-      </c>
-      <c r="D1213" s="135" t="s">
-        <v>2930</v>
-      </c>
-      <c r="E1213" s="125" t="s">
-        <v>2656</v>
-      </c>
-      <c r="F1213" s="127" t="s">
-        <v>1800</v>
-      </c>
-      <c r="G1213" s="127" t="s">
-        <v>1611</v>
-      </c>
-      <c r="H1213" s="128" t="s">
-        <v>1780</v>
-      </c>
-      <c r="I1213" s="119" t="s">
-        <v>519</v>
-      </c>
+      <c r="A1213" s="29"/>
+      <c r="B1213" s="135"/>
+      <c r="C1213" s="125"/>
+      <c r="D1213" s="126"/>
+      <c r="E1213" s="125"/>
+      <c r="F1213" s="127"/>
+      <c r="G1213" s="127"/>
+      <c r="H1213" s="128"/>
+      <c r="I1213" s="119"/>
       <c r="J1213" s="29"/>
       <c r="K1213" s="29"/>
       <c r="L1213" s="127"/>
@@ -59393,84 +59309,24 @@
       <c r="M1320" s="29"/>
     </row>
     <row r="1321" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1321" s="29"/>
+      <c r="A1321" s="131"/>
       <c r="B1321" s="135"/>
       <c r="C1321" s="125"/>
       <c r="D1321" s="126"/>
       <c r="E1321" s="125"/>
-      <c r="F1321" s="127"/>
-      <c r="G1321" s="127"/>
-      <c r="H1321" s="128"/>
-      <c r="I1321" s="119"/>
-      <c r="J1321" s="29"/>
-      <c r="K1321" s="29"/>
-      <c r="L1321" s="127"/>
-      <c r="M1321" s="29"/>
+      <c r="F1321" s="132"/>
+      <c r="G1321" s="132"/>
+      <c r="H1321" s="133"/>
+      <c r="I1321" s="134"/>
+      <c r="J1321" s="131"/>
+      <c r="K1321" s="131"/>
+      <c r="L1321" s="132"/>
+      <c r="M1321" s="131"/>
     </row>
     <row r="1322" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1322" s="29"/>
-      <c r="B1322" s="135"/>
-      <c r="C1322" s="125"/>
-      <c r="D1322" s="126"/>
-      <c r="E1322" s="125"/>
-      <c r="F1322" s="127"/>
-      <c r="G1322" s="127"/>
-      <c r="H1322" s="128"/>
-      <c r="I1322" s="119"/>
-      <c r="J1322" s="29"/>
-      <c r="K1322" s="29"/>
-      <c r="L1322" s="127"/>
-      <c r="M1322" s="29"/>
-    </row>
-    <row r="1323" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1323" s="29"/>
-      <c r="B1323" s="135"/>
-      <c r="C1323" s="125"/>
-      <c r="D1323" s="126"/>
-      <c r="E1323" s="125"/>
-      <c r="F1323" s="127"/>
-      <c r="G1323" s="127"/>
-      <c r="H1323" s="128"/>
-      <c r="I1323" s="119"/>
-      <c r="J1323" s="29"/>
-      <c r="K1323" s="29"/>
-      <c r="L1323" s="127"/>
-      <c r="M1323" s="29"/>
-    </row>
-    <row r="1324" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1324" s="29"/>
-      <c r="B1324" s="135"/>
-      <c r="C1324" s="125"/>
-      <c r="D1324" s="126"/>
-      <c r="E1324" s="125"/>
-      <c r="F1324" s="127"/>
-      <c r="G1324" s="127"/>
-      <c r="H1324" s="128"/>
-      <c r="I1324" s="119"/>
-      <c r="J1324" s="29"/>
-      <c r="K1324" s="29"/>
-      <c r="L1324" s="127"/>
-      <c r="M1324" s="29"/>
-    </row>
-    <row r="1325" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1325" s="131"/>
-      <c r="B1325" s="135"/>
-      <c r="C1325" s="125"/>
-      <c r="D1325" s="126"/>
-      <c r="E1325" s="125"/>
-      <c r="F1325" s="132"/>
-      <c r="G1325" s="132"/>
-      <c r="H1325" s="133"/>
-      <c r="I1325" s="134"/>
-      <c r="J1325" s="131"/>
-      <c r="K1325" s="131"/>
-      <c r="L1325" s="132"/>
-      <c r="M1325" s="131"/>
-    </row>
-    <row r="1326" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="B1326" s="83"/>
-      <c r="K1326" s="113"/>
-      <c r="L1326" s="3"/>
+      <c r="B1322" s="83"/>
+      <c r="K1322" s="113"/>
+      <c r="L1322" s="3"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>

<commit_message>
Added radio routes from ULXD hardware
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD290A05-0F58-524B-9B6E-00BD58A919FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{268B8998-2301-2847-A7BB-820BD2A98451}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7120" yWindow="1520" windowWidth="23120" windowHeight="17000" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9993" uniqueCount="2989">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10016" uniqueCount="2996">
   <si>
     <t>Tag</t>
   </si>
@@ -9008,6 +9008,27 @@
   </si>
   <si>
     <t>ZAMU-B009</t>
+  </si>
+  <si>
+    <t>ZAMU-B010</t>
+  </si>
+  <si>
+    <t>ZAMU-G001</t>
+  </si>
+  <si>
+    <t>ZAMU-G002</t>
+  </si>
+  <si>
+    <t>ZAMU-G003</t>
+  </si>
+  <si>
+    <t>ZAMU-B012</t>
+  </si>
+  <si>
+    <t>ZAMU-B015</t>
+  </si>
+  <si>
+    <t>ZAMU-A002 or ZAMU-A003</t>
   </si>
 </sst>
 </file>
@@ -9122,7 +9143,7 @@
       <scheme val="major"/>
     </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -9180,6 +9201,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFBA4EFF"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
         <bgColor theme="4" tint="0.79998168889431442"/>
       </patternFill>
     </fill>
@@ -9423,7 +9450,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="127">
+  <cellXfs count="129">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -9657,6 +9684,12 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -58097,8 +58130,12 @@
       <c r="A1219" s="29" t="s">
         <v>2973</v>
       </c>
-      <c r="B1219" s="125"/>
-      <c r="C1219" s="83"/>
+      <c r="B1219" s="125" t="s">
+        <v>2989</v>
+      </c>
+      <c r="C1219" s="83" t="s">
+        <v>2964</v>
+      </c>
       <c r="D1219" s="100" t="s">
         <v>346</v>
       </c>
@@ -58117,7 +58154,9 @@
       <c r="I1219" s="119" t="s">
         <v>63</v>
       </c>
-      <c r="J1219" s="29"/>
+      <c r="J1219" s="29" t="s">
+        <v>1265</v>
+      </c>
       <c r="K1219" s="29"/>
       <c r="L1219" s="31"/>
       <c r="M1219" s="29"/>
@@ -58126,8 +58165,12 @@
       <c r="A1220" s="29" t="s">
         <v>2974</v>
       </c>
-      <c r="B1220" s="125"/>
-      <c r="C1220" s="83"/>
+      <c r="B1220" s="125" t="s">
+        <v>2990</v>
+      </c>
+      <c r="C1220" s="83" t="s">
+        <v>2964</v>
+      </c>
       <c r="D1220" s="100" t="s">
         <v>346</v>
       </c>
@@ -58146,7 +58189,9 @@
       <c r="I1220" s="119" t="s">
         <v>63</v>
       </c>
-      <c r="J1220" s="29"/>
+      <c r="J1220" s="29" t="s">
+        <v>1266</v>
+      </c>
       <c r="K1220" s="29"/>
       <c r="L1220" s="31"/>
       <c r="M1220" s="29"/>
@@ -58155,8 +58200,12 @@
       <c r="A1221" s="29" t="s">
         <v>2975</v>
       </c>
-      <c r="B1221" s="125"/>
-      <c r="C1221" s="83"/>
+      <c r="B1221" s="128" t="s">
+        <v>2995</v>
+      </c>
+      <c r="C1221" s="83" t="s">
+        <v>2964</v>
+      </c>
       <c r="D1221" s="100" t="s">
         <v>346</v>
       </c>
@@ -58175,7 +58224,9 @@
       <c r="I1221" s="119" t="s">
         <v>63</v>
       </c>
-      <c r="J1221" s="29"/>
+      <c r="J1221" s="29" t="s">
+        <v>1268</v>
+      </c>
       <c r="K1221" s="29"/>
       <c r="L1221" s="31"/>
       <c r="M1221" s="29"/>
@@ -58184,8 +58235,12 @@
       <c r="A1222" s="29" t="s">
         <v>2976</v>
       </c>
-      <c r="B1222" s="125"/>
-      <c r="C1222" s="83"/>
+      <c r="B1222" s="128" t="s">
+        <v>2995</v>
+      </c>
+      <c r="C1222" s="83" t="s">
+        <v>2964</v>
+      </c>
       <c r="D1222" s="100" t="s">
         <v>346</v>
       </c>
@@ -58204,7 +58259,9 @@
       <c r="I1222" s="119" t="s">
         <v>63</v>
       </c>
-      <c r="J1222" s="29"/>
+      <c r="J1222" s="29" t="s">
+        <v>1269</v>
+      </c>
       <c r="K1222" s="29"/>
       <c r="L1222" s="31"/>
       <c r="M1222" s="29"/>
@@ -58213,8 +58270,12 @@
       <c r="A1223" s="29" t="s">
         <v>2977</v>
       </c>
-      <c r="B1223" s="125"/>
-      <c r="C1223" s="83"/>
+      <c r="B1223" s="125" t="s">
+        <v>2993</v>
+      </c>
+      <c r="C1223" s="83" t="s">
+        <v>2964</v>
+      </c>
       <c r="D1223" s="100" t="s">
         <v>347</v>
       </c>
@@ -58233,7 +58294,9 @@
       <c r="I1223" s="119" t="s">
         <v>63</v>
       </c>
-      <c r="J1223" s="29"/>
+      <c r="J1223" s="29" t="s">
+        <v>1270</v>
+      </c>
       <c r="K1223" s="29"/>
       <c r="L1223" s="31"/>
       <c r="M1223" s="29"/>
@@ -58242,8 +58305,12 @@
       <c r="A1224" s="29" t="s">
         <v>2978</v>
       </c>
-      <c r="B1224" s="125"/>
-      <c r="C1224" s="83"/>
+      <c r="B1224" s="125" t="s">
+        <v>2991</v>
+      </c>
+      <c r="C1224" s="83" t="s">
+        <v>2964</v>
+      </c>
       <c r="D1224" s="100" t="s">
         <v>347</v>
       </c>
@@ -58262,7 +58329,9 @@
       <c r="I1224" s="119" t="s">
         <v>63</v>
       </c>
-      <c r="J1224" s="29"/>
+      <c r="J1224" s="29" t="s">
+        <v>2359</v>
+      </c>
       <c r="K1224" s="29"/>
       <c r="L1224" s="31"/>
       <c r="M1224" s="29"/>
@@ -58271,8 +58340,12 @@
       <c r="A1225" s="29" t="s">
         <v>2979</v>
       </c>
-      <c r="B1225" s="125"/>
-      <c r="C1225" s="83"/>
+      <c r="B1225" s="127" t="s">
+        <v>2992</v>
+      </c>
+      <c r="C1225" s="83" t="s">
+        <v>2964</v>
+      </c>
       <c r="D1225" s="100" t="s">
         <v>347</v>
       </c>
@@ -58291,7 +58364,9 @@
       <c r="I1225" s="119" t="s">
         <v>63</v>
       </c>
-      <c r="J1225" s="29"/>
+      <c r="J1225" s="29" t="s">
+        <v>2360</v>
+      </c>
       <c r="K1225" s="29"/>
       <c r="L1225" s="31"/>
       <c r="M1225" s="29"/>
@@ -58300,8 +58375,12 @@
       <c r="A1226" s="29" t="s">
         <v>2980</v>
       </c>
-      <c r="B1226" s="126"/>
-      <c r="C1226" s="83"/>
+      <c r="B1226" s="126" t="s">
+        <v>2994</v>
+      </c>
+      <c r="C1226" s="83" t="s">
+        <v>2964</v>
+      </c>
       <c r="D1226" s="100" t="s">
         <v>347</v>
       </c>

</xml_diff>

<commit_message>
added permanent cables for stage display tv
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFC20681-08D4-8248-A758-51D934B78088}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{229176E8-5063-C94D-B5B8-3A245C21A986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8420" yWindow="1520" windowWidth="21820" windowHeight="17000" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10102" uniqueCount="3052">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10132" uniqueCount="3061">
   <si>
     <t>Tag</t>
   </si>
@@ -9197,6 +9197,33 @@
   </si>
   <si>
     <t>temp cable - true label unknown</t>
+  </si>
+  <si>
+    <t>2605-1402</t>
+  </si>
+  <si>
+    <t>audio-xlr</t>
+  </si>
+  <si>
+    <t>9m</t>
+  </si>
+  <si>
+    <t>ProPresenter Talkback</t>
+  </si>
+  <si>
+    <t>2605-1400</t>
+  </si>
+  <si>
+    <t>2605-1401</t>
+  </si>
+  <si>
+    <t>tbd</t>
+  </si>
+  <si>
+    <t>Stage Display TV</t>
+  </si>
+  <si>
+    <t>jump1242</t>
   </si>
 </sst>
 </file>
@@ -50195,18 +50222,10 @@
       <c r="A975" s="29" t="s">
         <v>2282</v>
       </c>
-      <c r="B975" s="112" t="s">
-        <v>1063</v>
-      </c>
-      <c r="C975" s="82" t="s">
-        <v>1155</v>
-      </c>
-      <c r="D975" s="79" t="s">
-        <v>2279</v>
-      </c>
-      <c r="E975" s="82" t="s">
-        <v>218</v>
-      </c>
+      <c r="B975" s="112"/>
+      <c r="C975" s="82"/>
+      <c r="D975" s="79"/>
+      <c r="E975" s="82"/>
       <c r="F975" s="31" t="s">
         <v>1564</v>
       </c>
@@ -50219,9 +50238,7 @@
       <c r="I975" s="19" t="s">
         <v>99</v>
       </c>
-      <c r="J975" s="29" t="s">
-        <v>2281</v>
-      </c>
+      <c r="J975" s="29"/>
       <c r="K975" s="29"/>
       <c r="L975" s="31" t="s">
         <v>2284</v>
@@ -58952,60 +58969,130 @@
       <c r="M1238" s="29"/>
     </row>
     <row r="1239" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1239" s="29"/>
+      <c r="A1239" s="29" t="s">
+        <v>3052</v>
+      </c>
       <c r="B1239" s="100"/>
       <c r="C1239" s="83"/>
-      <c r="D1239" s="85"/>
+      <c r="D1239" s="85" t="s">
+        <v>2241</v>
+      </c>
       <c r="E1239" s="83"/>
-      <c r="F1239" s="31"/>
-      <c r="G1239" s="31"/>
-      <c r="H1239" s="29"/>
-      <c r="I1239" s="119"/>
-      <c r="J1239" s="29"/>
+      <c r="F1239" s="31" t="s">
+        <v>3053</v>
+      </c>
+      <c r="G1239" s="31" t="s">
+        <v>1495</v>
+      </c>
+      <c r="H1239" s="29" t="s">
+        <v>3054</v>
+      </c>
+      <c r="I1239" s="119" t="s">
+        <v>99</v>
+      </c>
+      <c r="J1239" s="29" t="s">
+        <v>3055</v>
+      </c>
       <c r="K1239" s="29"/>
       <c r="L1239" s="31"/>
       <c r="M1239" s="29"/>
     </row>
     <row r="1240" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1240" s="29"/>
-      <c r="B1240" s="100"/>
-      <c r="C1240" s="83"/>
-      <c r="D1240" s="85"/>
-      <c r="E1240" s="83"/>
-      <c r="F1240" s="31"/>
-      <c r="G1240" s="31"/>
-      <c r="H1240" s="29"/>
-      <c r="I1240" s="119"/>
-      <c r="J1240" s="29"/>
+      <c r="A1240" s="29" t="s">
+        <v>3056</v>
+      </c>
+      <c r="B1240" s="100" t="s">
+        <v>1063</v>
+      </c>
+      <c r="C1240" s="83" t="s">
+        <v>1155</v>
+      </c>
+      <c r="D1240" s="85" t="s">
+        <v>2279</v>
+      </c>
+      <c r="E1240" s="83" t="s">
+        <v>218</v>
+      </c>
+      <c r="F1240" s="31" t="s">
+        <v>1564</v>
+      </c>
+      <c r="G1240" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1240" s="29" t="s">
+        <v>3058</v>
+      </c>
+      <c r="I1240" s="119" t="s">
+        <v>99</v>
+      </c>
+      <c r="J1240" s="29" t="s">
+        <v>3059</v>
+      </c>
       <c r="K1240" s="29"/>
       <c r="L1240" s="31"/>
       <c r="M1240" s="29"/>
     </row>
     <row r="1241" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1241" s="29"/>
-      <c r="B1241" s="100"/>
-      <c r="C1241" s="83"/>
-      <c r="D1241" s="85"/>
-      <c r="E1241" s="83"/>
-      <c r="F1241" s="31"/>
-      <c r="G1241" s="31"/>
-      <c r="H1241" s="29"/>
-      <c r="I1241" s="119"/>
-      <c r="J1241" s="29"/>
+      <c r="A1241" s="29" t="s">
+        <v>3057</v>
+      </c>
+      <c r="B1241" s="29" t="s">
+        <v>1642</v>
+      </c>
+      <c r="C1241" s="83" t="s">
+        <v>2421</v>
+      </c>
+      <c r="D1241" s="85" t="s">
+        <v>2280</v>
+      </c>
+      <c r="E1241" s="83" t="s">
+        <v>2198</v>
+      </c>
+      <c r="F1241" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="G1241" s="31" t="s">
+        <v>1491</v>
+      </c>
+      <c r="H1241" s="29" t="s">
+        <v>3058</v>
+      </c>
+      <c r="I1241" s="119" t="s">
+        <v>99</v>
+      </c>
+      <c r="J1241" s="29" t="s">
+        <v>3059</v>
+      </c>
       <c r="K1241" s="29"/>
       <c r="L1241" s="31"/>
       <c r="M1241" s="29"/>
     </row>
     <row r="1242" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1242" s="29"/>
-      <c r="B1242" s="100"/>
-      <c r="C1242" s="83"/>
-      <c r="D1242" s="85"/>
-      <c r="E1242" s="83"/>
-      <c r="F1242" s="31"/>
-      <c r="G1242" s="31"/>
+      <c r="A1242" s="29" t="s">
+        <v>3060</v>
+      </c>
+      <c r="B1242" s="100" t="s">
+        <v>1685</v>
+      </c>
+      <c r="C1242" s="83" t="s">
+        <v>1271</v>
+      </c>
+      <c r="D1242" s="29" t="s">
+        <v>1642</v>
+      </c>
+      <c r="E1242" s="83" t="s">
+        <v>2414</v>
+      </c>
+      <c r="F1242" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="G1242" s="31" t="s">
+        <v>1491</v>
+      </c>
       <c r="H1242" s="29"/>
-      <c r="I1242" s="119"/>
+      <c r="I1242" s="119" t="s">
+        <v>63</v>
+      </c>
       <c r="J1242" s="29"/>
       <c r="K1242" s="29"/>
       <c r="L1242" s="31"/>

</xml_diff>

<commit_message>
added Nursey call and Propresenter Mic data
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{229176E8-5063-C94D-B5B8-3A245C21A986}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1CF16B82-320E-3346-BCE2-E4E420C70853}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8420" yWindow="1520" windowWidth="21820" windowHeight="17000" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -18,8 +18,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="38" r:id="rId3"/>
-    <pivotCache cacheId="39" r:id="rId4"/>
+    <pivotCache cacheId="42" r:id="rId3"/>
+    <pivotCache cacheId="43" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10132" uniqueCount="3061">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10153" uniqueCount="3069">
   <si>
     <t>Tag</t>
   </si>
@@ -9224,6 +9224,30 @@
   </si>
   <si>
     <t>jump1242</t>
+  </si>
+  <si>
+    <t>25m</t>
+  </si>
+  <si>
+    <t>2605-1500</t>
+  </si>
+  <si>
+    <t>2605-1502</t>
+  </si>
+  <si>
+    <t>2605-1503</t>
+  </si>
+  <si>
+    <t>tbd1243</t>
+  </si>
+  <si>
+    <t>tbd1244</t>
+  </si>
+  <si>
+    <t>not yet</t>
+  </si>
+  <si>
+    <t>Nursery Stream Deck</t>
   </si>
 </sst>
 </file>
@@ -9645,7 +9669,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="130">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -9875,19 +9899,15 @@
     <xf numFmtId="49" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="49" fontId="5" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="5" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -18755,7 +18775,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="38" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="42" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -18818,7 +18838,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="39" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="43" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B56" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -19838,7 +19858,7 @@
       <c r="E15" s="23"/>
       <c r="F15" s="23"/>
       <c r="G15" s="23"/>
-      <c r="H15" s="129"/>
+      <c r="H15" s="29"/>
       <c r="I15" s="119"/>
       <c r="J15" s="23"/>
       <c r="K15" s="23"/>
@@ -19878,7 +19898,7 @@
       <c r="E17" s="23"/>
       <c r="F17" s="23"/>
       <c r="G17" s="23"/>
-      <c r="H17" s="129"/>
+      <c r="H17" s="29"/>
       <c r="I17" s="119"/>
       <c r="J17" s="23"/>
       <c r="K17" s="23"/>
@@ -58007,7 +58027,7 @@
       <c r="A1212" s="29" t="s">
         <v>2830</v>
       </c>
-      <c r="B1212" s="125" t="s">
+      <c r="B1212" s="100" t="s">
         <v>2846</v>
       </c>
       <c r="C1212" s="83" t="s">
@@ -58042,7 +58062,7 @@
       <c r="A1213" s="29" t="s">
         <v>2831</v>
       </c>
-      <c r="B1213" s="125" t="s">
+      <c r="B1213" s="100" t="s">
         <v>2847</v>
       </c>
       <c r="C1213" s="83" t="s">
@@ -58077,7 +58097,7 @@
       <c r="A1214" s="29" t="s">
         <v>2832</v>
       </c>
-      <c r="B1214" s="125" t="s">
+      <c r="B1214" s="100" t="s">
         <v>2848</v>
       </c>
       <c r="C1214" s="83" t="s">
@@ -58112,7 +58132,7 @@
       <c r="A1215" s="29" t="s">
         <v>2833</v>
       </c>
-      <c r="B1215" s="125" t="s">
+      <c r="B1215" s="100" t="s">
         <v>2849</v>
       </c>
       <c r="C1215" s="83" t="s">
@@ -58147,7 +58167,7 @@
       <c r="A1216" s="29" t="s">
         <v>2834</v>
       </c>
-      <c r="B1216" s="125" t="s">
+      <c r="B1216" s="100" t="s">
         <v>2850</v>
       </c>
       <c r="C1216" s="83" t="s">
@@ -58182,7 +58202,7 @@
       <c r="A1217" s="29" t="s">
         <v>2835</v>
       </c>
-      <c r="B1217" s="125" t="s">
+      <c r="B1217" s="100" t="s">
         <v>2851</v>
       </c>
       <c r="C1217" s="83" t="s">
@@ -58217,7 +58237,7 @@
       <c r="A1218" s="29" t="s">
         <v>2836</v>
       </c>
-      <c r="B1218" s="125" t="s">
+      <c r="B1218" s="100" t="s">
         <v>2852</v>
       </c>
       <c r="C1218" s="83" t="s">
@@ -58252,7 +58272,7 @@
       <c r="A1219" s="29" t="s">
         <v>2837</v>
       </c>
-      <c r="B1219" s="125" t="s">
+      <c r="B1219" s="100" t="s">
         <v>2853</v>
       </c>
       <c r="C1219" s="83" t="s">
@@ -58287,7 +58307,7 @@
       <c r="A1220" s="29" t="s">
         <v>2838</v>
       </c>
-      <c r="B1220" s="125" t="s">
+      <c r="B1220" s="100" t="s">
         <v>2854</v>
       </c>
       <c r="C1220" s="83" t="s">
@@ -58322,7 +58342,7 @@
       <c r="A1221" s="29" t="s">
         <v>2839</v>
       </c>
-      <c r="B1221" s="128" t="s">
+      <c r="B1221" s="127" t="s">
         <v>2859</v>
       </c>
       <c r="C1221" s="83" t="s">
@@ -58357,7 +58377,7 @@
       <c r="A1222" s="29" t="s">
         <v>2840</v>
       </c>
-      <c r="B1222" s="128" t="s">
+      <c r="B1222" s="127" t="s">
         <v>2859</v>
       </c>
       <c r="C1222" s="83" t="s">
@@ -58392,7 +58412,7 @@
       <c r="A1223" s="29" t="s">
         <v>2841</v>
       </c>
-      <c r="B1223" s="125" t="s">
+      <c r="B1223" s="100" t="s">
         <v>2857</v>
       </c>
       <c r="C1223" s="83" t="s">
@@ -58427,7 +58447,7 @@
       <c r="A1224" s="29" t="s">
         <v>2842</v>
       </c>
-      <c r="B1224" s="125" t="s">
+      <c r="B1224" s="100" t="s">
         <v>2855</v>
       </c>
       <c r="C1224" s="83" t="s">
@@ -58462,7 +58482,7 @@
       <c r="A1225" s="29" t="s">
         <v>2843</v>
       </c>
-      <c r="B1225" s="127" t="s">
+      <c r="B1225" s="126" t="s">
         <v>2856</v>
       </c>
       <c r="C1225" s="83" t="s">
@@ -58497,7 +58517,7 @@
       <c r="A1226" s="29" t="s">
         <v>2844</v>
       </c>
-      <c r="B1226" s="126" t="s">
+      <c r="B1226" s="125" t="s">
         <v>2858</v>
       </c>
       <c r="C1226" s="83" t="s">
@@ -58972,12 +58992,18 @@
       <c r="A1239" s="29" t="s">
         <v>3052</v>
       </c>
-      <c r="B1239" s="100"/>
-      <c r="C1239" s="83"/>
+      <c r="B1239" s="100" t="s">
+        <v>3062</v>
+      </c>
+      <c r="C1239" s="83" t="s">
+        <v>772</v>
+      </c>
       <c r="D1239" s="85" t="s">
         <v>2241</v>
       </c>
-      <c r="E1239" s="83"/>
+      <c r="E1239" s="83" t="s">
+        <v>2006</v>
+      </c>
       <c r="F1239" s="31" t="s">
         <v>3053</v>
       </c>
@@ -59020,7 +59046,7 @@
         <v>27</v>
       </c>
       <c r="H1240" s="29" t="s">
-        <v>3058</v>
+        <v>3061</v>
       </c>
       <c r="I1240" s="119" t="s">
         <v>99</v>
@@ -59055,7 +59081,7 @@
         <v>1491</v>
       </c>
       <c r="H1241" s="29" t="s">
-        <v>3058</v>
+        <v>1122</v>
       </c>
       <c r="I1241" s="119" t="s">
         <v>99</v>
@@ -59099,31 +59125,67 @@
       <c r="M1242" s="29"/>
     </row>
     <row r="1243" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1243" s="29"/>
-      <c r="B1243" s="100"/>
-      <c r="C1243" s="83"/>
-      <c r="D1243" s="85"/>
-      <c r="E1243" s="83"/>
-      <c r="F1243" s="31"/>
-      <c r="G1243" s="31"/>
+      <c r="A1243" s="29" t="s">
+        <v>3065</v>
+      </c>
+      <c r="B1243" s="100" t="s">
+        <v>3063</v>
+      </c>
+      <c r="C1243" s="83" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1243" s="85" t="s">
+        <v>3064</v>
+      </c>
+      <c r="E1243" s="83" t="s">
+        <v>55</v>
+      </c>
+      <c r="F1243" s="31" t="s">
+        <v>55</v>
+      </c>
+      <c r="G1243" s="31" t="s">
+        <v>55</v>
+      </c>
       <c r="H1243" s="29"/>
-      <c r="I1243" s="119"/>
-      <c r="J1243" s="29"/>
+      <c r="I1243" s="119" t="s">
+        <v>3067</v>
+      </c>
+      <c r="J1243" s="29" t="s">
+        <v>3068</v>
+      </c>
       <c r="K1243" s="29"/>
       <c r="L1243" s="31"/>
       <c r="M1243" s="29"/>
     </row>
     <row r="1244" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1244" s="29"/>
-      <c r="B1244" s="100"/>
-      <c r="C1244" s="83"/>
-      <c r="D1244" s="85"/>
-      <c r="E1244" s="83"/>
-      <c r="F1244" s="31"/>
-      <c r="G1244" s="31"/>
+      <c r="A1244" s="29" t="s">
+        <v>3066</v>
+      </c>
+      <c r="B1244" s="85" t="s">
+        <v>3064</v>
+      </c>
+      <c r="C1244" s="83" t="s">
+        <v>2198</v>
+      </c>
+      <c r="D1244" s="29" t="s">
+        <v>1642</v>
+      </c>
+      <c r="E1244" s="83" t="s">
+        <v>3058</v>
+      </c>
+      <c r="F1244" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="G1244" s="31" t="s">
+        <v>1491</v>
+      </c>
       <c r="H1244" s="29"/>
-      <c r="I1244" s="119"/>
-      <c r="J1244" s="29"/>
+      <c r="I1244" s="119" t="s">
+        <v>3067</v>
+      </c>
+      <c r="J1244" s="29" t="s">
+        <v>3068</v>
+      </c>
       <c r="K1244" s="29"/>
       <c r="L1244" s="31"/>
       <c r="M1244" s="29"/>

</xml_diff>

<commit_message>
addedd recent purchases - stream deck hardware and ProP Mic
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72FB94EC-4CB1-424A-A446-BF6259C8DFAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E943448-C3E1-824D-B179-749F0AFB7992}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8420" yWindow="1520" windowWidth="21820" windowHeight="17000" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10180" uniqueCount="3075">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10212" uniqueCount="3083">
   <si>
     <t>Tag</t>
   </si>
@@ -9266,6 +9266,30 @@
   </si>
   <si>
     <t>2408-2704</t>
+  </si>
+  <si>
+    <t>2605-2503</t>
+  </si>
+  <si>
+    <t>streamdeck</t>
+  </si>
+  <si>
+    <t>.225m</t>
+  </si>
+  <si>
+    <t>2605-2502</t>
+  </si>
+  <si>
+    <t>ProP Stream Deck</t>
+  </si>
+  <si>
+    <t>2605-2504</t>
+  </si>
+  <si>
+    <t>2605-2505</t>
+  </si>
+  <si>
+    <t>~5m</t>
   </si>
 </sst>
 </file>
@@ -9442,7 +9466,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="22">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -9677,11 +9701,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="double">
+        <color rgb="FF4472C4"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF8EA9DB"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="127">
+  <cellXfs count="128">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -9915,6 +9950,9 @@
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="49" fontId="9" fillId="5" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="9" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -59284,46 +59322,110 @@
       <c r="M1246" s="29"/>
     </row>
     <row r="1247" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1247" s="29"/>
-      <c r="B1247" s="100"/>
-      <c r="C1247" s="83"/>
-      <c r="D1247" s="85"/>
-      <c r="E1247" s="83"/>
-      <c r="F1247" s="31"/>
-      <c r="G1247" s="31"/>
-      <c r="H1247" s="29"/>
-      <c r="I1247" s="119"/>
-      <c r="J1247" s="29"/>
+      <c r="A1247" s="29" t="s">
+        <v>3075</v>
+      </c>
+      <c r="B1247" s="100" t="s">
+        <v>3051</v>
+      </c>
+      <c r="C1247" s="83" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1247" s="85" t="s">
+        <v>3076</v>
+      </c>
+      <c r="E1247" s="83" t="s">
+        <v>55</v>
+      </c>
+      <c r="F1247" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1247" s="31" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1247" s="29" t="s">
+        <v>3077</v>
+      </c>
+      <c r="I1247" s="119" t="s">
+        <v>99</v>
+      </c>
+      <c r="J1247" s="29" t="s">
+        <v>3055</v>
+      </c>
       <c r="K1247" s="29"/>
-      <c r="L1247" s="31"/>
+      <c r="L1247" s="31" t="s">
+        <v>641</v>
+      </c>
       <c r="M1247" s="29"/>
     </row>
-    <row r="1248" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1248" s="29"/>
-      <c r="B1248" s="100"/>
-      <c r="C1248" s="83"/>
-      <c r="D1248" s="85"/>
-      <c r="E1248" s="83"/>
-      <c r="F1248" s="31"/>
-      <c r="G1248" s="31"/>
-      <c r="H1248" s="29"/>
-      <c r="I1248" s="119"/>
-      <c r="J1248" s="29"/>
+    <row r="1248" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A1248" s="29" t="s">
+        <v>3078</v>
+      </c>
+      <c r="B1248" s="100" t="s">
+        <v>3051</v>
+      </c>
+      <c r="C1248" s="83" t="s">
+        <v>55</v>
+      </c>
+      <c r="D1248" s="85" t="s">
+        <v>3080</v>
+      </c>
+      <c r="E1248" s="83" t="s">
+        <v>55</v>
+      </c>
+      <c r="F1248" s="31" t="s">
+        <v>24</v>
+      </c>
+      <c r="G1248" s="31" t="s">
+        <v>55</v>
+      </c>
+      <c r="H1248" s="29" t="s">
+        <v>3077</v>
+      </c>
+      <c r="I1248" s="119" t="s">
+        <v>99</v>
+      </c>
+      <c r="J1248" s="29" t="s">
+        <v>3079</v>
+      </c>
       <c r="K1248" s="29"/>
-      <c r="L1248" s="31"/>
+      <c r="L1248" s="31" t="s">
+        <v>641</v>
+      </c>
       <c r="M1248" s="29"/>
     </row>
-    <row r="1249" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1249" s="29"/>
-      <c r="B1249" s="100"/>
-      <c r="C1249" s="83"/>
-      <c r="D1249" s="85"/>
-      <c r="E1249" s="83"/>
-      <c r="F1249" s="31"/>
-      <c r="G1249" s="31"/>
-      <c r="H1249" s="29"/>
-      <c r="I1249" s="119"/>
-      <c r="J1249" s="29"/>
+    <row r="1249" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A1249" s="29" t="s">
+        <v>3081</v>
+      </c>
+      <c r="B1249" s="127" t="s">
+        <v>1639</v>
+      </c>
+      <c r="C1249" s="83" t="s">
+        <v>2301</v>
+      </c>
+      <c r="D1249" s="85" t="s">
+        <v>3051</v>
+      </c>
+      <c r="E1249" s="83" t="s">
+        <v>2198</v>
+      </c>
+      <c r="F1249" s="31" t="s">
+        <v>234</v>
+      </c>
+      <c r="G1249" s="31" t="s">
+        <v>1491</v>
+      </c>
+      <c r="H1249" s="29" t="s">
+        <v>3082</v>
+      </c>
+      <c r="I1249" s="119" t="s">
+        <v>99</v>
+      </c>
+      <c r="J1249" s="29" t="s">
+        <v>3079</v>
+      </c>
       <c r="K1249" s="29"/>
       <c r="L1249" s="31"/>
       <c r="M1249" s="29"/>

</xml_diff>

<commit_message>
added route between ProP StreamDeck and companion
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1EE8331D-0974-9B43-84A0-64E86EA39D2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19488184-23A5-F346-A38C-B3253D85E9D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8420" yWindow="1520" windowWidth="21820" windowHeight="17000" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10212" uniqueCount="3084">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10221" uniqueCount="3088">
   <si>
     <t>Tag</t>
   </si>
@@ -9293,6 +9293,18 @@
   </si>
   <si>
     <t>unk1244</t>
+  </si>
+  <si>
+    <t>rt1250</t>
+  </si>
+  <si>
+    <t>unk1250</t>
+  </si>
+  <si>
+    <t>elgato</t>
+  </si>
+  <si>
+    <t>ProP Stream Deck to Companion</t>
   </si>
 </sst>
 </file>
@@ -59434,16 +59446,36 @@
       <c r="M1249" s="29"/>
     </row>
     <row r="1250" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1250" s="29"/>
-      <c r="B1250" s="100"/>
-      <c r="C1250" s="83"/>
-      <c r="D1250" s="85"/>
-      <c r="E1250" s="83"/>
-      <c r="F1250" s="31"/>
-      <c r="G1250" s="31"/>
-      <c r="H1250" s="29"/>
-      <c r="I1250" s="119"/>
-      <c r="J1250" s="29"/>
+      <c r="A1250" s="29" t="s">
+        <v>3084</v>
+      </c>
+      <c r="B1250" s="100" t="s">
+        <v>3079</v>
+      </c>
+      <c r="C1250" s="83" t="s">
+        <v>3085</v>
+      </c>
+      <c r="D1250" s="85" t="s">
+        <v>56</v>
+      </c>
+      <c r="E1250" s="83" t="s">
+        <v>3085</v>
+      </c>
+      <c r="F1250" s="31" t="s">
+        <v>1563</v>
+      </c>
+      <c r="G1250" s="31" t="s">
+        <v>3086</v>
+      </c>
+      <c r="H1250" s="29">
+        <v>0</v>
+      </c>
+      <c r="I1250" s="119" t="s">
+        <v>63</v>
+      </c>
+      <c r="J1250" s="29" t="s">
+        <v>3087</v>
+      </c>
       <c r="K1250" s="29"/>
       <c r="L1250" s="31"/>
       <c r="M1250" s="29"/>

</xml_diff>

<commit_message>
flipped route direction for companion to stream deck
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{19488184-23A5-F346-A38C-B3253D85E9D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D3472D5-F74C-1E45-9952-B8CFA7F56C70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8420" yWindow="1520" windowWidth="21820" windowHeight="17000" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -9298,13 +9298,13 @@
     <t>rt1250</t>
   </si>
   <si>
-    <t>unk1250</t>
-  </si>
-  <si>
     <t>elgato</t>
   </si>
   <si>
     <t>ProP Stream Deck to Companion</t>
+  </si>
+  <si>
+    <t>5343</t>
   </si>
 </sst>
 </file>
@@ -59445,27 +59445,27 @@
       <c r="L1249" s="31"/>
       <c r="M1249" s="29"/>
     </row>
-    <row r="1250" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1250" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1250" s="29" t="s">
         <v>3084</v>
       </c>
-      <c r="B1250" s="100" t="s">
+      <c r="B1250" s="85" t="s">
+        <v>56</v>
+      </c>
+      <c r="C1250" s="83" t="s">
+        <v>2293</v>
+      </c>
+      <c r="D1250" s="100" t="s">
         <v>3079</v>
       </c>
-      <c r="C1250" s="83" t="s">
-        <v>3085</v>
-      </c>
-      <c r="D1250" s="85" t="s">
-        <v>56</v>
-      </c>
-      <c r="E1250" s="83" t="s">
-        <v>3085</v>
+      <c r="E1250" s="86" t="s">
+        <v>3087</v>
       </c>
       <c r="F1250" s="31" t="s">
         <v>1563</v>
       </c>
       <c r="G1250" s="31" t="s">
-        <v>3086</v>
+        <v>3085</v>
       </c>
       <c r="H1250" s="29">
         <v>0</v>
@@ -59474,16 +59474,16 @@
         <v>63</v>
       </c>
       <c r="J1250" s="29" t="s">
-        <v>3087</v>
+        <v>3086</v>
       </c>
       <c r="K1250" s="29"/>
       <c r="L1250" s="31"/>
       <c r="M1250" s="29"/>
     </row>
-    <row r="1251" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1251" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A1251" s="29"/>
-      <c r="B1251" s="100"/>
-      <c r="C1251" s="83"/>
+      <c r="B1251" s="80"/>
+      <c r="C1251" s="82"/>
       <c r="D1251" s="85"/>
       <c r="E1251" s="83"/>
       <c r="F1251" s="31"/>

</xml_diff>

<commit_message>
fixed duplicate row for 2307-1814
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F50D6A91-8EBF-294D-A172-44E0AA1E7039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84177932-EF07-D444-A20F-8DFAFA599D19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8420" yWindow="1520" windowWidth="21820" windowHeight="17000" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10230" uniqueCount="3089">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10225" uniqueCount="3089">
   <si>
     <t>Tag</t>
   </si>
@@ -19931,25 +19931,15 @@
       <c r="M15" s="24"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A16" s="21" t="s">
-        <v>10</v>
-      </c>
+      <c r="A16" s="21"/>
       <c r="B16" s="22"/>
       <c r="C16" s="25"/>
       <c r="D16" s="22"/>
       <c r="E16" s="23"/>
-      <c r="F16" s="23" t="s">
-        <v>1565</v>
-      </c>
-      <c r="G16" s="23" t="s">
-        <v>27</v>
-      </c>
-      <c r="H16" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="I16" s="23" t="s">
-        <v>63</v>
-      </c>
+      <c r="F16" s="23"/>
+      <c r="G16" s="23"/>
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
       <c r="J16" s="23"/>
       <c r="K16" s="23"/>
       <c r="L16" s="19"/>

</xml_diff>

<commit_message>
changed blank rows to notags
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A293D633-5F1B-8445-B504-6EE97FE41E53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59BA6DEB-29F1-E641-9AD3-E70305E18348}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8420" yWindow="1520" windowWidth="21820" windowHeight="17000" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -18,8 +18,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="8" r:id="rId3"/>
-    <pivotCache cacheId="9" r:id="rId4"/>
+    <pivotCache cacheId="10" r:id="rId3"/>
+    <pivotCache cacheId="11" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10295" uniqueCount="3109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10306" uniqueCount="3120">
   <si>
     <t>Tag</t>
   </si>
@@ -9368,6 +9368,39 @@
   </si>
   <si>
     <t xml:space="preserve">IP Control </t>
+  </si>
+  <si>
+    <t>notag101</t>
+  </si>
+  <si>
+    <t>notag119</t>
+  </si>
+  <si>
+    <t>notag225</t>
+  </si>
+  <si>
+    <t>notag476</t>
+  </si>
+  <si>
+    <t>notag566</t>
+  </si>
+  <si>
+    <t>notag661</t>
+  </si>
+  <si>
+    <t>notag662</t>
+  </si>
+  <si>
+    <t>notag663</t>
+  </si>
+  <si>
+    <t>notag881</t>
+  </si>
+  <si>
+    <t>notag969</t>
+  </si>
+  <si>
+    <t>notag970</t>
   </si>
 </sst>
 </file>
@@ -18900,70 +18933,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="12">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="7"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of Tag" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B56" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -19196,6 +19166,69 @@
     </i>
     <i>
       <x v="53"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Tag" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
     </i>
     <i t="grand">
       <x/>
@@ -22654,7 +22687,9 @@
       <c r="M100" s="20"/>
     </row>
     <row r="101" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A101" s="21"/>
+      <c r="A101" s="21" t="s">
+        <v>3109</v>
+      </c>
       <c r="B101" s="22" t="s">
         <v>53</v>
       </c>
@@ -23220,7 +23255,9 @@
       <c r="M118" s="24"/>
     </row>
     <row r="119" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A119" s="21"/>
+      <c r="A119" s="21" t="s">
+        <v>3110</v>
+      </c>
       <c r="B119" s="22"/>
       <c r="C119" s="23"/>
       <c r="D119" s="22"/>
@@ -26780,7 +26817,9 @@
       <c r="M224" s="29"/>
     </row>
     <row r="225" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A225" s="29"/>
+      <c r="A225" s="29" t="s">
+        <v>3111</v>
+      </c>
       <c r="B225" s="31"/>
       <c r="C225" s="29"/>
       <c r="D225" s="31"/>
@@ -34391,7 +34430,9 @@
       <c r="M475" s="29"/>
     </row>
     <row r="476" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A476" s="29"/>
+      <c r="A476" s="29" t="s">
+        <v>3112</v>
+      </c>
       <c r="B476" s="29"/>
       <c r="C476" s="36"/>
       <c r="D476" s="58"/>
@@ -37367,7 +37408,9 @@
       <c r="M565" s="29"/>
     </row>
     <row r="566" spans="1:13" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A566" s="29"/>
+      <c r="A566" s="29" t="s">
+        <v>3113</v>
+      </c>
       <c r="B566" s="95"/>
       <c r="C566" s="73"/>
       <c r="D566" s="95"/>
@@ -40458,7 +40501,9 @@
       <c r="M660" s="29"/>
     </row>
     <row r="661" spans="1:13" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A661" s="29"/>
+      <c r="A661" s="29" t="s">
+        <v>3114</v>
+      </c>
       <c r="B661" s="83"/>
       <c r="C661" s="29"/>
       <c r="D661" s="84"/>
@@ -40473,7 +40518,9 @@
       <c r="M661" s="29"/>
     </row>
     <row r="662" spans="1:13" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A662" s="29"/>
+      <c r="A662" s="29" t="s">
+        <v>3115</v>
+      </c>
       <c r="B662" s="83"/>
       <c r="C662" s="29"/>
       <c r="D662" s="84"/>
@@ -40488,7 +40535,9 @@
       <c r="M662" s="29"/>
     </row>
     <row r="663" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A663" s="29"/>
+      <c r="A663" s="29" t="s">
+        <v>3116</v>
+      </c>
       <c r="B663" s="83"/>
       <c r="C663" s="29"/>
       <c r="D663" s="84"/>
@@ -47474,7 +47523,9 @@
       <c r="M880" s="29"/>
     </row>
     <row r="881" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A881" s="29"/>
+      <c r="A881" s="29" t="s">
+        <v>3117</v>
+      </c>
       <c r="B881" s="83"/>
       <c r="C881" s="83"/>
       <c r="D881" s="85"/>
@@ -50350,7 +50401,9 @@
       <c r="M968" s="29"/>
     </row>
     <row r="969" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A969" s="29"/>
+      <c r="A969" s="29" t="s">
+        <v>3118</v>
+      </c>
       <c r="B969" s="100"/>
       <c r="C969" s="83"/>
       <c r="D969" s="85"/>
@@ -50365,7 +50418,9 @@
       <c r="M969" s="29"/>
     </row>
     <row r="970" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
-      <c r="A970" s="29"/>
+      <c r="A970" s="29" t="s">
+        <v>3119</v>
+      </c>
       <c r="B970" s="112"/>
       <c r="C970" s="120"/>
       <c r="D970" s="79"/>

</xml_diff>

<commit_message>
Added nursery Streamdeck details
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0F9B77C-171A-F94C-87F5-0E92AED79AC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82F1C579-63CC-234A-A167-B0C99676172F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8420" yWindow="1520" windowWidth="21820" windowHeight="17000" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -18,8 +18,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="10" r:id="rId3"/>
-    <pivotCache cacheId="11" r:id="rId4"/>
+    <pivotCache cacheId="1" r:id="rId3"/>
+    <pivotCache cacheId="2" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10308" uniqueCount="3122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10318" uniqueCount="3125">
   <si>
     <t>Tag</t>
   </si>
@@ -9373,12 +9373,6 @@
     <t>notag101</t>
   </si>
   <si>
-    <t>notag119</t>
-  </si>
-  <si>
-    <t>notag225</t>
-  </si>
-  <si>
     <t>notag476</t>
   </si>
   <si>
@@ -9407,6 +9401,21 @@
   </si>
   <si>
     <t>notag813</t>
+  </si>
+  <si>
+    <t>2606-1000</t>
+  </si>
+  <si>
+    <t>usba-usbc</t>
+  </si>
+  <si>
+    <t>right angle usbc</t>
+  </si>
+  <si>
+    <t>rt225</t>
+  </si>
+  <si>
+    <t>Streamdeck</t>
   </si>
 </sst>
 </file>
@@ -18939,7 +18948,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B56" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -19196,7 +19205,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -23262,18 +23271,26 @@
     </row>
     <row r="119" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A119" s="21" t="s">
-        <v>3110</v>
+        <v>3120</v>
       </c>
       <c r="B119" s="22"/>
       <c r="C119" s="23"/>
       <c r="D119" s="22"/>
       <c r="E119" s="23"/>
-      <c r="F119" s="23"/>
-      <c r="G119" s="23"/>
+      <c r="F119" s="23" t="s">
+        <v>3121</v>
+      </c>
+      <c r="G119" s="23" t="s">
+        <v>52</v>
+      </c>
       <c r="H119" s="23"/>
       <c r="I119" s="23"/>
-      <c r="J119" s="23"/>
-      <c r="K119" s="23"/>
+      <c r="J119" s="23" t="s">
+        <v>439</v>
+      </c>
+      <c r="K119" s="23" t="s">
+        <v>3122</v>
+      </c>
       <c r="L119" s="19"/>
       <c r="M119" s="20"/>
     </row>
@@ -26824,17 +26841,33 @@
     </row>
     <row r="225" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A225" s="29" t="s">
-        <v>3111</v>
-      </c>
-      <c r="B225" s="31"/>
+        <v>3123</v>
+      </c>
+      <c r="B225" s="31" t="s">
+        <v>53</v>
+      </c>
       <c r="C225" s="29"/>
-      <c r="D225" s="31"/>
-      <c r="E225" s="29"/>
-      <c r="F225" s="31"/>
-      <c r="G225" s="31"/>
-      <c r="H225" s="29"/>
-      <c r="I225" s="29"/>
-      <c r="J225" s="29"/>
+      <c r="D225" s="31" t="s">
+        <v>3062</v>
+      </c>
+      <c r="E225" s="29">
+        <v>5343</v>
+      </c>
+      <c r="F225" s="31" t="s">
+        <v>1550</v>
+      </c>
+      <c r="G225" s="31" t="s">
+        <v>3070</v>
+      </c>
+      <c r="H225" s="29">
+        <v>0</v>
+      </c>
+      <c r="I225" s="29" t="s">
+        <v>503</v>
+      </c>
+      <c r="J225" s="29" t="s">
+        <v>3124</v>
+      </c>
       <c r="K225" s="29"/>
       <c r="L225" s="31"/>
       <c r="M225" s="29"/>
@@ -34437,7 +34470,7 @@
     </row>
     <row r="476" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A476" s="29" t="s">
-        <v>3112</v>
+        <v>3110</v>
       </c>
       <c r="B476" s="29"/>
       <c r="C476" s="36"/>
@@ -37415,7 +37448,7 @@
     </row>
     <row r="566" spans="1:13" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A566" s="29" t="s">
-        <v>3113</v>
+        <v>3111</v>
       </c>
       <c r="B566" s="95"/>
       <c r="C566" s="73"/>
@@ -40508,7 +40541,7 @@
     </row>
     <row r="661" spans="1:13" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A661" s="29" t="s">
-        <v>3114</v>
+        <v>3112</v>
       </c>
       <c r="B661" s="83"/>
       <c r="C661" s="29"/>
@@ -40525,7 +40558,7 @@
     </row>
     <row r="662" spans="1:13" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A662" s="29" t="s">
-        <v>3115</v>
+        <v>3113</v>
       </c>
       <c r="B662" s="83"/>
       <c r="C662" s="29"/>
@@ -40542,7 +40575,7 @@
     </row>
     <row r="663" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A663" s="29" t="s">
-        <v>3116</v>
+        <v>3114</v>
       </c>
       <c r="B663" s="83"/>
       <c r="C663" s="29"/>
@@ -45290,7 +45323,7 @@
     </row>
     <row r="811" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A811" s="29" t="s">
-        <v>3120</v>
+        <v>3118</v>
       </c>
       <c r="B811" s="83"/>
       <c r="C811" s="83"/>
@@ -45338,7 +45371,7 @@
     </row>
     <row r="813" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A813" s="29" t="s">
-        <v>3121</v>
+        <v>3119</v>
       </c>
       <c r="B813" s="83"/>
       <c r="C813" s="83"/>
@@ -47534,7 +47567,7 @@
     </row>
     <row r="881" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A881" s="29" t="s">
-        <v>3117</v>
+        <v>3115</v>
       </c>
       <c r="B881" s="83"/>
       <c r="C881" s="83"/>
@@ -50412,7 +50445,7 @@
     </row>
     <row r="969" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A969" s="29" t="s">
-        <v>3118</v>
+        <v>3116</v>
       </c>
       <c r="B969" s="100"/>
       <c r="C969" s="83"/>
@@ -50429,7 +50462,7 @@
     </row>
     <row r="970" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A970" s="29" t="s">
-        <v>3119</v>
+        <v>3117</v>
       </c>
       <c r="B970" s="112"/>
       <c r="C970" s="120"/>

</xml_diff>

<commit_message>
updates driven by cables 2606-1300 and 2606-1301
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82F1C579-63CC-234A-A167-B0C99676172F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7750DE2-E875-DB4D-9001-600A24446C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8420" yWindow="1520" windowWidth="21820" windowHeight="17000" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -18,8 +18,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="1" r:id="rId3"/>
-    <pivotCache cacheId="2" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
+    <pivotCache cacheId="1" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10318" uniqueCount="3125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10366" uniqueCount="3138">
   <si>
     <t>Tag</t>
   </si>
@@ -9373,33 +9373,9 @@
     <t>notag101</t>
   </si>
   <si>
-    <t>notag476</t>
-  </si>
-  <si>
-    <t>notag566</t>
-  </si>
-  <si>
-    <t>notag661</t>
-  </si>
-  <si>
-    <t>notag662</t>
-  </si>
-  <si>
     <t>notag663</t>
   </si>
   <si>
-    <t>notag881</t>
-  </si>
-  <si>
-    <t>notag969</t>
-  </si>
-  <si>
-    <t>notag970</t>
-  </si>
-  <si>
-    <t>notag811</t>
-  </si>
-  <si>
     <t>notag813</t>
   </si>
   <si>
@@ -9416,6 +9392,69 @@
   </si>
   <si>
     <t>Streamdeck</t>
+  </si>
+  <si>
+    <t>1.55m</t>
+  </si>
+  <si>
+    <t>2606-1001</t>
+  </si>
+  <si>
+    <t>LibraryTV control</t>
+  </si>
+  <si>
+    <t>jump1255</t>
+  </si>
+  <si>
+    <t>blank476</t>
+  </si>
+  <si>
+    <t>blank566</t>
+  </si>
+  <si>
+    <t>blank811</t>
+  </si>
+  <si>
+    <t>blank881</t>
+  </si>
+  <si>
+    <t>blank969</t>
+  </si>
+  <si>
+    <t>blank970</t>
+  </si>
+  <si>
+    <t>2606-1300</t>
+  </si>
+  <si>
+    <t>2606-1301</t>
+  </si>
+  <si>
+    <t>47m</t>
+  </si>
+  <si>
+    <t>71m</t>
+  </si>
+  <si>
+    <t>2405-2501-F30</t>
+  </si>
+  <si>
+    <t>Intended to be uplink from NSCU-A001 to cisco switch in rack. Currently used for ITNET for CUMU-G002</t>
+  </si>
+  <si>
+    <t>amprack PP</t>
+  </si>
+  <si>
+    <t>tobe 24</t>
+  </si>
+  <si>
+    <t>Intended to be uplink from 2603-1200 (amp) to 2603-1203. Not yet terminated.</t>
+  </si>
+  <si>
+    <t>4 or 14 ?</t>
+  </si>
+  <si>
+    <t>temp patch awaiting switch</t>
   </si>
 </sst>
 </file>
@@ -18948,7 +18987,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B56" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -19205,7 +19244,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -23271,25 +23310,27 @@
     </row>
     <row r="119" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A119" s="21" t="s">
-        <v>3120</v>
+        <v>3112</v>
       </c>
       <c r="B119" s="22"/>
       <c r="C119" s="23"/>
       <c r="D119" s="22"/>
       <c r="E119" s="23"/>
       <c r="F119" s="23" t="s">
-        <v>3121</v>
+        <v>3113</v>
       </c>
       <c r="G119" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="H119" s="23"/>
+      <c r="H119" s="23" t="s">
+        <v>3117</v>
+      </c>
       <c r="I119" s="23"/>
       <c r="J119" s="23" t="s">
         <v>439</v>
       </c>
       <c r="K119" s="23" t="s">
-        <v>3122</v>
+        <v>3114</v>
       </c>
       <c r="L119" s="19"/>
       <c r="M119" s="20"/>
@@ -26841,7 +26882,7 @@
     </row>
     <row r="225" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A225" s="29" t="s">
-        <v>3123</v>
+        <v>3115</v>
       </c>
       <c r="B225" s="31" t="s">
         <v>53</v>
@@ -26866,7 +26907,7 @@
         <v>503</v>
       </c>
       <c r="J225" s="29" t="s">
-        <v>3124</v>
+        <v>3116</v>
       </c>
       <c r="K225" s="29"/>
       <c r="L225" s="31"/>
@@ -34470,7 +34511,7 @@
     </row>
     <row r="476" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A476" s="29" t="s">
-        <v>3110</v>
+        <v>3121</v>
       </c>
       <c r="B476" s="29"/>
       <c r="C476" s="36"/>
@@ -37448,7 +37489,7 @@
     </row>
     <row r="566" spans="1:13" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A566" s="29" t="s">
-        <v>3111</v>
+        <v>3122</v>
       </c>
       <c r="B566" s="95"/>
       <c r="C566" s="73"/>
@@ -40541,51 +40582,109 @@
     </row>
     <row r="661" spans="1:13" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A661" s="29" t="s">
-        <v>3112</v>
-      </c>
-      <c r="B661" s="83"/>
-      <c r="C661" s="29"/>
-      <c r="D661" s="84"/>
-      <c r="E661" s="73"/>
-      <c r="F661" s="85"/>
-      <c r="G661" s="85"/>
-      <c r="H661" s="23"/>
-      <c r="I661" s="23"/>
-      <c r="J661" s="29"/>
-      <c r="K661" s="29"/>
+        <v>3127</v>
+      </c>
+      <c r="B661" s="83" t="s">
+        <v>3131</v>
+      </c>
+      <c r="C661" s="29">
+        <v>24</v>
+      </c>
+      <c r="D661" s="84" t="s">
+        <v>1852</v>
+      </c>
+      <c r="E661" s="73" t="s">
+        <v>1264</v>
+      </c>
+      <c r="F661" s="85" t="s">
+        <v>231</v>
+      </c>
+      <c r="G661" s="85" t="s">
+        <v>1478</v>
+      </c>
+      <c r="H661" s="23" t="s">
+        <v>3129</v>
+      </c>
+      <c r="I661" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="J661" s="29" t="s">
+        <v>3132</v>
+      </c>
+      <c r="K661" s="29" t="s">
+        <v>465</v>
+      </c>
       <c r="L661" s="31"/>
       <c r="M661" s="29"/>
     </row>
     <row r="662" spans="1:13" ht="18" thickTop="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A662" s="29" t="s">
-        <v>3113</v>
-      </c>
-      <c r="B662" s="83"/>
-      <c r="C662" s="29"/>
-      <c r="D662" s="84"/>
-      <c r="E662" s="73"/>
-      <c r="F662" s="85"/>
-      <c r="G662" s="85"/>
-      <c r="H662" s="23"/>
-      <c r="I662" s="23"/>
-      <c r="J662" s="29"/>
-      <c r="K662" s="29"/>
+        <v>3128</v>
+      </c>
+      <c r="B662" s="83" t="s">
+        <v>3133</v>
+      </c>
+      <c r="C662" s="29" t="s">
+        <v>3134</v>
+      </c>
+      <c r="D662" s="84" t="s">
+        <v>1629</v>
+      </c>
+      <c r="E662" s="73" t="s">
+        <v>1264</v>
+      </c>
+      <c r="F662" s="85" t="s">
+        <v>231</v>
+      </c>
+      <c r="G662" s="85" t="s">
+        <v>1478</v>
+      </c>
+      <c r="H662" s="23" t="s">
+        <v>3130</v>
+      </c>
+      <c r="I662" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="J662" s="29" t="s">
+        <v>3135</v>
+      </c>
+      <c r="K662" s="29" t="s">
+        <v>989</v>
+      </c>
       <c r="L662" s="31"/>
       <c r="M662" s="29"/>
     </row>
     <row r="663" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A663" s="29" t="s">
-        <v>3114</v>
-      </c>
-      <c r="B663" s="83"/>
-      <c r="C663" s="29"/>
-      <c r="D663" s="84"/>
-      <c r="E663" s="73"/>
-      <c r="F663" s="85"/>
-      <c r="G663" s="85"/>
-      <c r="H663" s="23"/>
-      <c r="I663" s="23"/>
-      <c r="J663" s="29"/>
+        <v>3110</v>
+      </c>
+      <c r="B663" s="84" t="s">
+        <v>1629</v>
+      </c>
+      <c r="C663" s="73" t="s">
+        <v>1264</v>
+      </c>
+      <c r="D663" s="84" t="s">
+        <v>1629</v>
+      </c>
+      <c r="E663" s="73" t="s">
+        <v>3136</v>
+      </c>
+      <c r="F663" s="85" t="s">
+        <v>1651</v>
+      </c>
+      <c r="G663" s="85" t="s">
+        <v>1478</v>
+      </c>
+      <c r="H663" s="23" t="s">
+        <v>194</v>
+      </c>
+      <c r="I663" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="J663" s="29" t="s">
+        <v>3137</v>
+      </c>
       <c r="K663" s="29"/>
       <c r="L663" s="31"/>
       <c r="M663" s="29"/>
@@ -45323,7 +45422,7 @@
     </row>
     <row r="811" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A811" s="29" t="s">
-        <v>3118</v>
+        <v>3123</v>
       </c>
       <c r="B811" s="83"/>
       <c r="C811" s="83"/>
@@ -45371,7 +45470,7 @@
     </row>
     <row r="813" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A813" s="29" t="s">
-        <v>3119</v>
+        <v>3111</v>
       </c>
       <c r="B813" s="83"/>
       <c r="C813" s="83"/>
@@ -47567,7 +47666,7 @@
     </row>
     <row r="881" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A881" s="29" t="s">
-        <v>3115</v>
+        <v>3124</v>
       </c>
       <c r="B881" s="83"/>
       <c r="C881" s="83"/>
@@ -50445,7 +50544,7 @@
     </row>
     <row r="969" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A969" s="29" t="s">
-        <v>3116</v>
+        <v>3125</v>
       </c>
       <c r="B969" s="100"/>
       <c r="C969" s="83"/>
@@ -50462,7 +50561,7 @@
     </row>
     <row r="970" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A970" s="29" t="s">
-        <v>3117</v>
+        <v>3126</v>
       </c>
       <c r="B970" s="112"/>
       <c r="C970" s="120"/>
@@ -59855,31 +59954,69 @@
       <c r="M1253" s="29"/>
     </row>
     <row r="1254" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1254" s="29"/>
-      <c r="B1254" s="100"/>
-      <c r="C1254" s="83"/>
-      <c r="D1254" s="85"/>
-      <c r="E1254" s="83"/>
-      <c r="F1254" s="31"/>
-      <c r="G1254" s="31"/>
-      <c r="H1254" s="29"/>
-      <c r="I1254" s="119"/>
-      <c r="J1254" s="29"/>
+      <c r="A1254" s="29" t="s">
+        <v>3118</v>
+      </c>
+      <c r="B1254" s="29" t="s">
+        <v>1629</v>
+      </c>
+      <c r="C1254" s="83" t="s">
+        <v>2397</v>
+      </c>
+      <c r="D1254" s="85" t="s">
+        <v>1494</v>
+      </c>
+      <c r="E1254" s="83" t="s">
+        <v>2183</v>
+      </c>
+      <c r="F1254" s="31" t="s">
+        <v>231</v>
+      </c>
+      <c r="G1254" s="31" t="s">
+        <v>1478</v>
+      </c>
+      <c r="H1254" s="29" t="s">
+        <v>467</v>
+      </c>
+      <c r="I1254" s="119" t="s">
+        <v>96</v>
+      </c>
+      <c r="J1254" s="29" t="s">
+        <v>3119</v>
+      </c>
       <c r="K1254" s="29"/>
       <c r="L1254" s="31"/>
       <c r="M1254" s="29"/>
     </row>
     <row r="1255" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1255" s="29"/>
-      <c r="B1255" s="100"/>
-      <c r="C1255" s="83"/>
-      <c r="D1255" s="85"/>
-      <c r="E1255" s="83"/>
-      <c r="F1255" s="31"/>
-      <c r="G1255" s="31"/>
+      <c r="A1255" s="29" t="s">
+        <v>3120</v>
+      </c>
+      <c r="B1255" s="100" t="s">
+        <v>1672</v>
+      </c>
+      <c r="C1255" s="83" t="s">
+        <v>1259</v>
+      </c>
+      <c r="D1255" s="29" t="s">
+        <v>1629</v>
+      </c>
+      <c r="E1255" s="83" t="s">
+        <v>2390</v>
+      </c>
+      <c r="F1255" s="31" t="s">
+        <v>231</v>
+      </c>
+      <c r="G1255" s="31" t="s">
+        <v>1478</v>
+      </c>
       <c r="H1255" s="29"/>
-      <c r="I1255" s="119"/>
-      <c r="J1255" s="29"/>
+      <c r="I1255" s="119" t="s">
+        <v>60</v>
+      </c>
+      <c r="J1255" s="29" t="s">
+        <v>3119</v>
+      </c>
       <c r="K1255" s="29"/>
       <c r="L1255" s="31"/>
       <c r="M1255" s="29"/>

</xml_diff>

<commit_message>
updates regarding 2405-2501 and NSCU-A004
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7C817C3-3CAD-F846-A4FA-27B42C6807FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E6842CB-D194-5D4E-B03F-8FC3ABD56680}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="8420" yWindow="1520" windowWidth="21820" windowHeight="18020" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -9436,9 +9436,6 @@
     <t>2405-2501-F30</t>
   </si>
   <si>
-    <t>amprack PP</t>
-  </si>
-  <si>
     <t>temp patch awaiting switch</t>
   </si>
   <si>
@@ -9524,15 +9521,18 @@
 Not sure which one it will be.</t>
   </si>
   <si>
-    <t>Intended to be uplink from NSCU-A001 to cisco switch in rack. 
-Currently used for ITNET for CUMU-G002</t>
-  </si>
-  <si>
-    <t>Intended to be uplink from 2603-1200 (amp) to 2603-1203. 
+    <t>ITNet to PP</t>
+  </si>
+  <si>
+    <t>Intended to be uplink from NSCU-A001 to NSCU-A004. 
+Temp used for ITNET for CUMU-G002.</t>
+  </si>
+  <si>
+    <t>2405-2501 PP</t>
+  </si>
+  <si>
+    <t>Intended to be uplink from 2603-1200 to 2603-1203. 
 Not yet terminated.</t>
-  </si>
-  <si>
-    <t>ITNet to PP</t>
   </si>
 </sst>
 </file>
@@ -40712,10 +40712,10 @@
         <v>3127</v>
       </c>
       <c r="B662" s="83" t="s">
-        <v>3131</v>
+        <v>3161</v>
       </c>
       <c r="C662" s="128" t="s">
-        <v>3133</v>
+        <v>3132</v>
       </c>
       <c r="D662" s="84" t="s">
         <v>1629</v>
@@ -40736,7 +40736,7 @@
         <v>96</v>
       </c>
       <c r="J662" s="130" t="s">
-        <v>3161</v>
+        <v>3162</v>
       </c>
       <c r="K662" s="128" t="s">
         <v>989</v>
@@ -40773,7 +40773,7 @@
         <v>60</v>
       </c>
       <c r="J663" s="29" t="s">
-        <v>3132</v>
+        <v>3131</v>
       </c>
       <c r="K663" s="29"/>
       <c r="L663" s="31"/>
@@ -47540,7 +47540,7 @@
         <v>96</v>
       </c>
       <c r="J874" s="29" t="s">
-        <v>3162</v>
+        <v>3159</v>
       </c>
       <c r="K874" s="29"/>
       <c r="L874" s="31"/>
@@ -60113,7 +60113,7 @@
     </row>
     <row r="1256" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1256" s="29" t="s">
-        <v>3134</v>
+        <v>3133</v>
       </c>
       <c r="B1256" s="100" t="s">
         <v>3130</v>
@@ -60146,7 +60146,7 @@
     </row>
     <row r="1257" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1257" s="29" t="s">
-        <v>3135</v>
+        <v>3134</v>
       </c>
       <c r="B1257" s="100" t="s">
         <v>3130</v>
@@ -60179,7 +60179,7 @@
     </row>
     <row r="1258" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1258" s="29" t="s">
-        <v>3136</v>
+        <v>3135</v>
       </c>
       <c r="B1258" s="100" t="s">
         <v>3130</v>
@@ -60212,7 +60212,7 @@
     </row>
     <row r="1259" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1259" s="29" t="s">
-        <v>3137</v>
+        <v>3136</v>
       </c>
       <c r="B1259" s="100" t="s">
         <v>3130</v>
@@ -60245,7 +60245,7 @@
     </row>
     <row r="1260" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1260" s="29" t="s">
-        <v>3138</v>
+        <v>3137</v>
       </c>
       <c r="B1260" s="100" t="s">
         <v>3130</v>
@@ -60278,7 +60278,7 @@
     </row>
     <row r="1261" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1261" s="29" t="s">
-        <v>3139</v>
+        <v>3138</v>
       </c>
       <c r="B1261" s="100" t="s">
         <v>3130</v>
@@ -60311,7 +60311,7 @@
     </row>
     <row r="1262" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1262" s="29" t="s">
-        <v>3140</v>
+        <v>3139</v>
       </c>
       <c r="B1262" s="100" t="s">
         <v>3130</v>
@@ -60344,7 +60344,7 @@
     </row>
     <row r="1263" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1263" s="29" t="s">
-        <v>3141</v>
+        <v>3140</v>
       </c>
       <c r="B1263" s="100" t="s">
         <v>3130</v>
@@ -60377,7 +60377,7 @@
     </row>
     <row r="1264" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1264" s="29" t="s">
-        <v>3142</v>
+        <v>3141</v>
       </c>
       <c r="B1264" s="100" t="s">
         <v>3130</v>
@@ -60410,7 +60410,7 @@
     </row>
     <row r="1265" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1265" s="29" t="s">
-        <v>3143</v>
+        <v>3142</v>
       </c>
       <c r="B1265" s="100" t="s">
         <v>3130</v>
@@ -60443,7 +60443,7 @@
     </row>
     <row r="1266" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1266" s="29" t="s">
-        <v>3144</v>
+        <v>3143</v>
       </c>
       <c r="B1266" s="100" t="s">
         <v>3130</v>
@@ -60476,7 +60476,7 @@
     </row>
     <row r="1267" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1267" s="29" t="s">
-        <v>3145</v>
+        <v>3144</v>
       </c>
       <c r="B1267" s="100" t="s">
         <v>3130</v>
@@ -60509,7 +60509,7 @@
     </row>
     <row r="1268" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1268" s="29" t="s">
-        <v>3146</v>
+        <v>3145</v>
       </c>
       <c r="B1268" s="100" t="s">
         <v>3130</v>
@@ -60542,7 +60542,7 @@
     </row>
     <row r="1269" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1269" s="29" t="s">
-        <v>3147</v>
+        <v>3146</v>
       </c>
       <c r="B1269" s="100" t="s">
         <v>3130</v>
@@ -60575,7 +60575,7 @@
     </row>
     <row r="1270" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1270" s="29" t="s">
-        <v>3148</v>
+        <v>3147</v>
       </c>
       <c r="B1270" s="100" t="s">
         <v>3130</v>
@@ -60608,7 +60608,7 @@
     </row>
     <row r="1271" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1271" s="29" t="s">
-        <v>3149</v>
+        <v>3148</v>
       </c>
       <c r="B1271" s="100" t="s">
         <v>3130</v>
@@ -60641,7 +60641,7 @@
     </row>
     <row r="1272" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1272" s="29" t="s">
-        <v>3150</v>
+        <v>3149</v>
       </c>
       <c r="B1272" s="100" t="s">
         <v>3130</v>
@@ -60674,7 +60674,7 @@
     </row>
     <row r="1273" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1273" s="29" t="s">
-        <v>3151</v>
+        <v>3150</v>
       </c>
       <c r="B1273" s="100" t="s">
         <v>3130</v>
@@ -60707,7 +60707,7 @@
     </row>
     <row r="1274" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1274" s="29" t="s">
-        <v>3152</v>
+        <v>3151</v>
       </c>
       <c r="B1274" s="100" t="s">
         <v>3130</v>
@@ -60740,7 +60740,7 @@
     </row>
     <row r="1275" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1275" s="29" t="s">
-        <v>3153</v>
+        <v>3152</v>
       </c>
       <c r="B1275" s="100" t="s">
         <v>3130</v>
@@ -60773,7 +60773,7 @@
     </row>
     <row r="1276" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1276" s="29" t="s">
-        <v>3154</v>
+        <v>3153</v>
       </c>
       <c r="B1276" s="100" t="s">
         <v>3130</v>
@@ -60806,7 +60806,7 @@
     </row>
     <row r="1277" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1277" s="29" t="s">
-        <v>3155</v>
+        <v>3154</v>
       </c>
       <c r="B1277" s="100" t="s">
         <v>3130</v>
@@ -60839,7 +60839,7 @@
     </row>
     <row r="1278" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1278" s="29" t="s">
-        <v>3156</v>
+        <v>3155</v>
       </c>
       <c r="B1278" s="100" t="s">
         <v>3130</v>
@@ -60872,7 +60872,7 @@
     </row>
     <row r="1279" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1279" s="29" t="s">
-        <v>3157</v>
+        <v>3156</v>
       </c>
       <c r="B1279" s="100" t="s">
         <v>3130</v>
@@ -60905,7 +60905,7 @@
     </row>
     <row r="1280" spans="1:13" s="131" customFormat="1" ht="64" x14ac:dyDescent="0.2">
       <c r="A1280" s="128" t="s">
-        <v>3158</v>
+        <v>3157</v>
       </c>
       <c r="B1280" s="100" t="s">
         <v>242</v>
@@ -60932,7 +60932,7 @@
         <v>60</v>
       </c>
       <c r="J1280" s="130" t="s">
-        <v>3159</v>
+        <v>3158</v>
       </c>
       <c r="K1280" s="128"/>
       <c r="L1280" s="83"/>

</xml_diff>

<commit_message>
Updated for new 2nd stage display route:
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6912888F-FCB2-1349-93EF-DB73BD8D23D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0638DE10-C301-5B47-B85E-F2A46D486308}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3640" yWindow="1520" windowWidth="26600" windowHeight="18020" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10793" uniqueCount="3204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10815" uniqueCount="3212">
   <si>
     <t>Tag</t>
   </si>
@@ -9656,6 +9656,30 @@
   </si>
   <si>
     <t>notag1312</t>
+  </si>
+  <si>
+    <t>2606-1600</t>
+  </si>
+  <si>
+    <t>sdi_5</t>
+  </si>
+  <si>
+    <t>2nd stage display layout</t>
+  </si>
+  <si>
+    <t>avshop #461859</t>
+  </si>
+  <si>
+    <t>rack internal</t>
+  </si>
+  <si>
+    <t>rt1314</t>
+  </si>
+  <si>
+    <t>bmd</t>
+  </si>
+  <si>
+    <t>managed via videohubControl</t>
   </si>
 </sst>
 </file>
@@ -61971,7 +61995,7 @@
       <c r="L1311" s="31"/>
       <c r="M1311" s="29"/>
     </row>
-    <row r="1312" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="1312" spans="1:13" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1312" s="29" t="s">
         <v>3203</v>
       </c>
@@ -61996,33 +62020,79 @@
       <c r="L1312" s="31"/>
       <c r="M1312" s="29"/>
     </row>
-    <row r="1313" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1313" s="29"/>
-      <c r="B1313" s="100"/>
-      <c r="C1313" s="83"/>
-      <c r="D1313" s="85"/>
-      <c r="E1313" s="83"/>
-      <c r="F1313" s="31"/>
-      <c r="G1313" s="31"/>
-      <c r="H1313" s="29"/>
-      <c r="I1313" s="119"/>
-      <c r="J1313" s="29"/>
+    <row r="1313" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+      <c r="A1313" s="29" t="s">
+        <v>3204</v>
+      </c>
+      <c r="B1313" s="80" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1313" s="82" t="s">
+        <v>3205</v>
+      </c>
+      <c r="D1313" s="100" t="s">
+        <v>1050</v>
+      </c>
+      <c r="E1313" s="83" t="s">
+        <v>2229</v>
+      </c>
+      <c r="F1313" s="31" t="s">
+        <v>1552</v>
+      </c>
+      <c r="G1313" s="31" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1313" s="29" t="s">
+        <v>451</v>
+      </c>
+      <c r="I1313" s="119" t="s">
+        <v>96</v>
+      </c>
+      <c r="J1313" s="29" t="s">
+        <v>3206</v>
+      </c>
       <c r="K1313" s="29"/>
-      <c r="L1313" s="31"/>
-      <c r="M1313" s="29"/>
+      <c r="L1313" s="31" t="s">
+        <v>3207</v>
+      </c>
+      <c r="M1313" s="29" t="s">
+        <v>3208</v>
+      </c>
     </row>
     <row r="1314" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1314" s="29"/>
-      <c r="B1314" s="100"/>
-      <c r="C1314" s="83"/>
-      <c r="D1314" s="85"/>
-      <c r="E1314" s="83"/>
-      <c r="F1314" s="31"/>
-      <c r="G1314" s="31"/>
-      <c r="H1314" s="29"/>
-      <c r="I1314" s="119"/>
-      <c r="J1314" s="29"/>
-      <c r="K1314" s="29"/>
+      <c r="A1314" s="29" t="s">
+        <v>3209</v>
+      </c>
+      <c r="B1314" s="100" t="s">
+        <v>1050</v>
+      </c>
+      <c r="C1314" s="83" t="s">
+        <v>2229</v>
+      </c>
+      <c r="D1314" s="85" t="s">
+        <v>1050</v>
+      </c>
+      <c r="E1314" s="83" t="s">
+        <v>1883</v>
+      </c>
+      <c r="F1314" s="31" t="s">
+        <v>1550</v>
+      </c>
+      <c r="G1314" s="31" t="s">
+        <v>3210</v>
+      </c>
+      <c r="H1314" s="29">
+        <v>0</v>
+      </c>
+      <c r="I1314" s="119" t="s">
+        <v>503</v>
+      </c>
+      <c r="J1314" s="29" t="s">
+        <v>3206</v>
+      </c>
+      <c r="K1314" s="29" t="s">
+        <v>3211</v>
+      </c>
       <c r="L1314" s="31"/>
       <c r="M1314" s="29"/>
     </row>

</xml_diff>

<commit_message>
typo in patch panel name
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{644CC564-F402-A34A-A0DC-4E1965B1DF68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AE3FB06-C1B8-664C-912D-97F86E26744A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3640" yWindow="1520" windowWidth="26600" windowHeight="18020" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10951" uniqueCount="3256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10951" uniqueCount="3255">
   <si>
     <t>Tag</t>
   </si>
@@ -9803,9 +9803,6 @@
   </si>
   <si>
     <t>jump1334</t>
-  </si>
-  <si>
-    <t>2405-2501-F03</t>
   </si>
   <si>
     <t>NSCU-A001 to NSCU-A003 link</t>
@@ -23608,7 +23605,7 @@
     </row>
     <row r="118" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A118" s="21" t="s">
-        <v>3255</v>
+        <v>3254</v>
       </c>
       <c r="B118" s="22"/>
       <c r="C118" s="23"/>
@@ -62661,7 +62658,7 @@
         <v>96</v>
       </c>
       <c r="J1331" s="29" t="s">
-        <v>3254</v>
+        <v>3253</v>
       </c>
       <c r="K1331" s="29"/>
       <c r="L1331" s="136"/>
@@ -62692,7 +62689,7 @@
         <v>96</v>
       </c>
       <c r="J1332" s="29" t="s">
-        <v>3254</v>
+        <v>3253</v>
       </c>
       <c r="K1332" s="29"/>
       <c r="L1332" s="136"/>
@@ -62723,7 +62720,7 @@
         <v>96</v>
       </c>
       <c r="J1333" s="29" t="s">
-        <v>3254</v>
+        <v>3253</v>
       </c>
       <c r="K1333" s="29"/>
       <c r="L1333" s="136"/>
@@ -62740,7 +62737,7 @@
         <v>1228</v>
       </c>
       <c r="D1334" s="133" t="s">
-        <v>3253</v>
+        <v>3093</v>
       </c>
       <c r="E1334" s="134" t="s">
         <v>2281</v>
@@ -62754,7 +62751,7 @@
         <v>96</v>
       </c>
       <c r="J1334" s="29" t="s">
-        <v>3254</v>
+        <v>3253</v>
       </c>
       <c r="K1334" s="29"/>
       <c r="L1334" s="136"/>

</xml_diff>

<commit_message>
added a blank for testing
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E5E6497-65FD-B94F-BC9D-5792B5415208}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE392FE4-4E2F-E346-BADB-D99B5DE1D71A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3640" yWindow="1520" windowWidth="26600" windowHeight="18020" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11452" uniqueCount="3374">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11454" uniqueCount="3375">
   <si>
     <t>Tag</t>
   </si>
@@ -10166,6 +10166,9 @@
   </si>
   <si>
     <t>i875</t>
+  </si>
+  <si>
+    <t>blank1402</t>
   </si>
 </sst>
 </file>
@@ -65148,7 +65151,9 @@
       <c r="M1401" s="29"/>
     </row>
     <row r="1402" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1402" s="29"/>
+      <c r="A1402" s="29" t="s">
+        <v>3374</v>
+      </c>
       <c r="B1402" s="100"/>
       <c r="C1402" s="83"/>
       <c r="D1402" s="85"/>
@@ -65157,7 +65162,9 @@
       <c r="G1402" s="136"/>
       <c r="H1402" s="137"/>
       <c r="I1402" s="119"/>
-      <c r="J1402" s="29"/>
+      <c r="J1402" s="29" t="s">
+        <v>418</v>
+      </c>
       <c r="K1402" s="29"/>
       <c r="L1402" s="136"/>
       <c r="M1402" s="29"/>

</xml_diff>

<commit_message>
Updated Reference Monitor connections
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C7A13DC-4EB1-004D-B70D-001D485E3EFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA9CE644-643A-CF4E-85CB-8ECB85202FA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1820" yWindow="760" windowWidth="26600" windowHeight="18020" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -18,8 +18,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="5" r:id="rId3"/>
-    <pivotCache cacheId="6" r:id="rId4"/>
+    <pivotCache cacheId="8" r:id="rId3"/>
+    <pivotCache cacheId="9" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11617" uniqueCount="3391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11626" uniqueCount="3395">
   <si>
     <t>Tag</t>
   </si>
@@ -10217,6 +10217,18 @@
   </si>
   <si>
     <t>notag1190</t>
+  </si>
+  <si>
+    <t>2607-0700</t>
+  </si>
+  <si>
+    <t>audio_out</t>
+  </si>
+  <si>
+    <t>rca_in</t>
+  </si>
+  <si>
+    <t>audio_trs18_rca</t>
   </si>
 </sst>
 </file>
@@ -19723,7 +19735,70 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Tag" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B56" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -19956,69 +20031,6 @@
     </i>
     <i>
       <x v="53"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of Tag" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="12">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="7"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
     </i>
     <i t="grand">
       <x/>
@@ -65863,15 +65875,33 @@
       <c r="M1425" s="29"/>
     </row>
     <row r="1426" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1426" s="29"/>
-      <c r="B1426" s="100"/>
-      <c r="C1426" s="83"/>
-      <c r="D1426" s="85"/>
-      <c r="E1426" s="83"/>
-      <c r="F1426" s="31"/>
-      <c r="G1426" s="31"/>
-      <c r="H1426" s="29"/>
-      <c r="I1426" s="119"/>
+      <c r="A1426" s="29" t="s">
+        <v>3391</v>
+      </c>
+      <c r="B1426" s="100" t="s">
+        <v>55</v>
+      </c>
+      <c r="C1426" s="83" t="s">
+        <v>3392</v>
+      </c>
+      <c r="D1426" s="85" t="s">
+        <v>176</v>
+      </c>
+      <c r="E1426" s="83" t="s">
+        <v>3393</v>
+      </c>
+      <c r="F1426" s="31" t="s">
+        <v>3394</v>
+      </c>
+      <c r="G1426" s="31" t="s">
+        <v>1452</v>
+      </c>
+      <c r="H1426" s="29" t="s">
+        <v>192</v>
+      </c>
+      <c r="I1426" s="119" t="s">
+        <v>96</v>
+      </c>
       <c r="J1426" s="29"/>
       <c r="K1426" s="29"/>
       <c r="L1426" s="31"/>

</xml_diff>

<commit_message>
Added Ma3 loaner console
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA9CE644-643A-CF4E-85CB-8ECB85202FA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13E07ABF-A40E-034E-9E82-139F36E4A6CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1820" yWindow="760" windowWidth="26600" windowHeight="18020" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -18,8 +18,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="8" r:id="rId3"/>
-    <pivotCache cacheId="9" r:id="rId4"/>
+    <pivotCache cacheId="12" r:id="rId3"/>
+    <pivotCache cacheId="13" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11626" uniqueCount="3395">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11635" uniqueCount="3398">
   <si>
     <t>Tag</t>
   </si>
@@ -10229,6 +10229,15 @@
   </si>
   <si>
     <t>audio_trs18_rca</t>
+  </si>
+  <si>
+    <t>notag1427</t>
+  </si>
+  <si>
+    <t>demoma3</t>
+  </si>
+  <si>
+    <t>NIC1</t>
   </si>
 </sst>
 </file>
@@ -19735,7 +19744,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -19798,7 +19807,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="13" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B56" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -65908,15 +65917,33 @@
       <c r="M1426" s="29"/>
     </row>
     <row r="1427" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1427" s="29"/>
-      <c r="B1427" s="100"/>
-      <c r="C1427" s="83"/>
-      <c r="D1427" s="85"/>
-      <c r="E1427" s="83"/>
-      <c r="F1427" s="31"/>
-      <c r="G1427" s="31"/>
-      <c r="H1427" s="29"/>
-      <c r="I1427" s="119"/>
+      <c r="A1427" s="29" t="s">
+        <v>3395</v>
+      </c>
+      <c r="B1427" s="100" t="s">
+        <v>248</v>
+      </c>
+      <c r="C1427" s="83" t="s">
+        <v>1195</v>
+      </c>
+      <c r="D1427" s="85" t="s">
+        <v>3396</v>
+      </c>
+      <c r="E1427" s="83" t="s">
+        <v>3397</v>
+      </c>
+      <c r="F1427" s="31" t="s">
+        <v>229</v>
+      </c>
+      <c r="G1427" s="31" t="s">
+        <v>1449</v>
+      </c>
+      <c r="H1427" s="29" t="s">
+        <v>288</v>
+      </c>
+      <c r="I1427" s="119" t="s">
+        <v>60</v>
+      </c>
       <c r="J1427" s="29"/>
       <c r="K1427" s="29"/>
       <c r="L1427" s="31"/>

</xml_diff>

<commit_message>
added new Lighting gear
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10621"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7501D6B-632D-CD4B-9EE9-CED1646E218B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5146414-A083-EF47-9924-A6D3A9DB6270}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1820" yWindow="760" windowWidth="26600" windowHeight="18020" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -18,8 +18,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="12" r:id="rId3"/>
-    <pivotCache cacheId="13" r:id="rId4"/>
+    <pivotCache cacheId="0" r:id="rId3"/>
+    <pivotCache cacheId="1" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11635" uniqueCount="3398">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11705" uniqueCount="3425">
   <si>
     <t>Tag</t>
   </si>
@@ -10238,6 +10238,87 @@
   </si>
   <si>
     <t>NIC1</t>
+  </si>
+  <si>
+    <t>2607-1000</t>
+  </si>
+  <si>
+    <t>2607-2100</t>
+  </si>
+  <si>
+    <t>DP1</t>
+  </si>
+  <si>
+    <t>2607-1002</t>
+  </si>
+  <si>
+    <t>DisplayPort</t>
+  </si>
+  <si>
+    <t>1.8M</t>
+  </si>
+  <si>
+    <t>DP2</t>
+  </si>
+  <si>
+    <t>2607-1001</t>
+  </si>
+  <si>
+    <t>2607-1003</t>
+  </si>
+  <si>
+    <t>2607-1004</t>
+  </si>
+  <si>
+    <t>2607-1005</t>
+  </si>
+  <si>
+    <t>USB3.0-1</t>
+  </si>
+  <si>
+    <t>USB3.0-2</t>
+  </si>
+  <si>
+    <t>USBC</t>
+  </si>
+  <si>
+    <t>USB3A-USBC</t>
+  </si>
+  <si>
+    <t>usc</t>
+  </si>
+  <si>
+    <t>2607-1006</t>
+  </si>
+  <si>
+    <t>2607-1007</t>
+  </si>
+  <si>
+    <t>usbc-usbc</t>
+  </si>
+  <si>
+    <t>1.78m</t>
+  </si>
+  <si>
+    <t>Neysh 98610</t>
+  </si>
+  <si>
+    <t>2607-1008</t>
+  </si>
+  <si>
+    <t>2607-1009</t>
+  </si>
+  <si>
+    <t>IEC14</t>
+  </si>
+  <si>
+    <t>nema15p-IEC13</t>
+  </si>
+  <si>
+    <t>120vpower</t>
+  </si>
+  <si>
+    <t>pdistro1</t>
   </si>
 </sst>
 </file>
@@ -19753,7 +19834,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -19816,7 +19897,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="13" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B56" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -65959,123 +66040,263 @@
       <c r="M1427" s="29"/>
     </row>
     <row r="1428" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1428" s="29"/>
-      <c r="B1428" s="100"/>
-      <c r="C1428" s="83"/>
-      <c r="D1428" s="85"/>
-      <c r="E1428" s="83"/>
-      <c r="F1428" s="31"/>
-      <c r="G1428" s="31"/>
-      <c r="H1428" s="29"/>
-      <c r="I1428" s="119"/>
+      <c r="A1428" s="29" t="s">
+        <v>3401</v>
+      </c>
+      <c r="B1428" s="100" t="s">
+        <v>3399</v>
+      </c>
+      <c r="C1428" s="83" t="s">
+        <v>3400</v>
+      </c>
+      <c r="D1428" s="85" t="s">
+        <v>3398</v>
+      </c>
+      <c r="E1428" s="83" t="s">
+        <v>3400</v>
+      </c>
+      <c r="F1428" s="31" t="s">
+        <v>3402</v>
+      </c>
+      <c r="G1428" s="31" t="s">
+        <v>3402</v>
+      </c>
+      <c r="H1428" s="29" t="s">
+        <v>3403</v>
+      </c>
+      <c r="I1428" s="119" t="s">
+        <v>96</v>
+      </c>
       <c r="J1428" s="29"/>
       <c r="K1428" s="29"/>
-      <c r="L1428" s="31"/>
+      <c r="L1428" s="31" t="s">
+        <v>3418</v>
+      </c>
       <c r="M1428" s="29"/>
     </row>
     <row r="1429" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1429" s="29"/>
-      <c r="B1429" s="100"/>
-      <c r="C1429" s="83"/>
-      <c r="D1429" s="85"/>
-      <c r="E1429" s="83"/>
-      <c r="F1429" s="31"/>
-      <c r="G1429" s="31"/>
-      <c r="H1429" s="29"/>
-      <c r="I1429" s="119"/>
+      <c r="A1429" s="29" t="s">
+        <v>3406</v>
+      </c>
+      <c r="B1429" s="100" t="s">
+        <v>3399</v>
+      </c>
+      <c r="C1429" s="83" t="s">
+        <v>3404</v>
+      </c>
+      <c r="D1429" s="85" t="s">
+        <v>3405</v>
+      </c>
+      <c r="E1429" s="83" t="s">
+        <v>3400</v>
+      </c>
+      <c r="F1429" s="31" t="s">
+        <v>3402</v>
+      </c>
+      <c r="G1429" s="31" t="s">
+        <v>3402</v>
+      </c>
+      <c r="H1429" s="29" t="s">
+        <v>3403</v>
+      </c>
+      <c r="I1429" s="119" t="s">
+        <v>96</v>
+      </c>
       <c r="J1429" s="29"/>
       <c r="K1429" s="29"/>
-      <c r="L1429" s="31"/>
+      <c r="L1429" s="31" t="s">
+        <v>3418</v>
+      </c>
       <c r="M1429" s="29"/>
     </row>
     <row r="1430" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1430" s="29"/>
-      <c r="B1430" s="100"/>
-      <c r="C1430" s="83"/>
-      <c r="D1430" s="85"/>
-      <c r="E1430" s="83"/>
-      <c r="F1430" s="31"/>
-      <c r="G1430" s="31"/>
-      <c r="H1430" s="29"/>
-      <c r="I1430" s="119"/>
+      <c r="A1430" s="29" t="s">
+        <v>3407</v>
+      </c>
+      <c r="B1430" s="100" t="s">
+        <v>3399</v>
+      </c>
+      <c r="C1430" s="83" t="s">
+        <v>3409</v>
+      </c>
+      <c r="D1430" s="85" t="s">
+        <v>3398</v>
+      </c>
+      <c r="E1430" s="83" t="s">
+        <v>3411</v>
+      </c>
+      <c r="F1430" s="31" t="s">
+        <v>3412</v>
+      </c>
+      <c r="G1430" s="31" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1430" s="29" t="s">
+        <v>3403</v>
+      </c>
+      <c r="I1430" s="119" t="s">
+        <v>96</v>
+      </c>
       <c r="J1430" s="29"/>
       <c r="K1430" s="29"/>
-      <c r="L1430" s="31"/>
+      <c r="L1430" s="31" t="s">
+        <v>3418</v>
+      </c>
       <c r="M1430" s="29"/>
     </row>
     <row r="1431" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1431" s="29"/>
-      <c r="B1431" s="100"/>
-      <c r="C1431" s="83"/>
-      <c r="D1431" s="85"/>
-      <c r="E1431" s="83"/>
-      <c r="F1431" s="31"/>
-      <c r="G1431" s="31"/>
-      <c r="H1431" s="29"/>
-      <c r="I1431" s="119"/>
+      <c r="A1431" s="29" t="s">
+        <v>3408</v>
+      </c>
+      <c r="B1431" s="100" t="s">
+        <v>3399</v>
+      </c>
+      <c r="C1431" s="83" t="s">
+        <v>3410</v>
+      </c>
+      <c r="D1431" s="85" t="s">
+        <v>3405</v>
+      </c>
+      <c r="E1431" s="83" t="s">
+        <v>3411</v>
+      </c>
+      <c r="F1431" s="31" t="s">
+        <v>3412</v>
+      </c>
+      <c r="G1431" s="31" t="s">
+        <v>52</v>
+      </c>
+      <c r="H1431" s="29" t="s">
+        <v>3403</v>
+      </c>
+      <c r="I1431" s="119" t="s">
+        <v>96</v>
+      </c>
       <c r="J1431" s="29"/>
       <c r="K1431" s="29"/>
-      <c r="L1431" s="31"/>
+      <c r="L1431" s="31" t="s">
+        <v>3418</v>
+      </c>
       <c r="M1431" s="29"/>
     </row>
     <row r="1432" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1432" s="29"/>
+      <c r="A1432" s="29" t="s">
+        <v>3414</v>
+      </c>
       <c r="B1432" s="100"/>
       <c r="C1432" s="83"/>
       <c r="D1432" s="85"/>
       <c r="E1432" s="83"/>
-      <c r="F1432" s="31"/>
-      <c r="G1432" s="31"/>
-      <c r="H1432" s="29"/>
-      <c r="I1432" s="119"/>
+      <c r="F1432" s="31" t="s">
+        <v>3416</v>
+      </c>
+      <c r="G1432" s="31" t="s">
+        <v>3413</v>
+      </c>
+      <c r="H1432" s="29" t="s">
+        <v>3417</v>
+      </c>
+      <c r="I1432" s="119" t="s">
+        <v>96</v>
+      </c>
       <c r="J1432" s="29"/>
       <c r="K1432" s="29"/>
-      <c r="L1432" s="31"/>
+      <c r="L1432" s="31" t="s">
+        <v>3418</v>
+      </c>
       <c r="M1432" s="29"/>
     </row>
     <row r="1433" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1433" s="29"/>
+      <c r="A1433" s="29" t="s">
+        <v>3415</v>
+      </c>
       <c r="B1433" s="100"/>
       <c r="C1433" s="83"/>
       <c r="D1433" s="85"/>
       <c r="E1433" s="83"/>
-      <c r="F1433" s="31"/>
-      <c r="G1433" s="31"/>
-      <c r="H1433" s="29"/>
-      <c r="I1433" s="119"/>
+      <c r="F1433" s="31" t="s">
+        <v>3416</v>
+      </c>
+      <c r="G1433" s="31" t="s">
+        <v>3413</v>
+      </c>
+      <c r="H1433" s="29" t="s">
+        <v>3417</v>
+      </c>
+      <c r="I1433" s="119" t="s">
+        <v>96</v>
+      </c>
       <c r="J1433" s="29"/>
       <c r="K1433" s="29"/>
-      <c r="L1433" s="31"/>
+      <c r="L1433" s="31" t="s">
+        <v>3418</v>
+      </c>
       <c r="M1433" s="29"/>
     </row>
     <row r="1434" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1434" s="29"/>
-      <c r="B1434" s="100"/>
+      <c r="A1434" s="29" t="s">
+        <v>3419</v>
+      </c>
+      <c r="B1434" s="100" t="s">
+        <v>3424</v>
+      </c>
       <c r="C1434" s="83"/>
-      <c r="D1434" s="85"/>
-      <c r="E1434" s="83"/>
-      <c r="F1434" s="31"/>
-      <c r="G1434" s="31"/>
-      <c r="H1434" s="29"/>
-      <c r="I1434" s="119"/>
+      <c r="D1434" s="85" t="s">
+        <v>3398</v>
+      </c>
+      <c r="E1434" s="83" t="s">
+        <v>3421</v>
+      </c>
+      <c r="F1434" s="31" t="s">
+        <v>3422</v>
+      </c>
+      <c r="G1434" s="31" t="s">
+        <v>3423</v>
+      </c>
+      <c r="H1434" s="29" t="s">
+        <v>3403</v>
+      </c>
+      <c r="I1434" s="119" t="s">
+        <v>96</v>
+      </c>
       <c r="J1434" s="29"/>
       <c r="K1434" s="29"/>
-      <c r="L1434" s="31"/>
+      <c r="L1434" s="31" t="s">
+        <v>3418</v>
+      </c>
       <c r="M1434" s="29"/>
     </row>
     <row r="1435" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1435" s="29"/>
-      <c r="B1435" s="100"/>
+      <c r="A1435" s="29" t="s">
+        <v>3420</v>
+      </c>
+      <c r="B1435" s="100" t="s">
+        <v>3424</v>
+      </c>
       <c r="C1435" s="83"/>
-      <c r="D1435" s="85"/>
-      <c r="E1435" s="83"/>
-      <c r="F1435" s="31"/>
-      <c r="G1435" s="31"/>
-      <c r="H1435" s="29"/>
-      <c r="I1435" s="119"/>
+      <c r="D1435" s="85" t="s">
+        <v>3405</v>
+      </c>
+      <c r="E1435" s="83" t="s">
+        <v>3421</v>
+      </c>
+      <c r="F1435" s="31" t="s">
+        <v>3422</v>
+      </c>
+      <c r="G1435" s="31" t="s">
+        <v>3423</v>
+      </c>
+      <c r="H1435" s="29" t="s">
+        <v>3403</v>
+      </c>
+      <c r="I1435" s="119" t="s">
+        <v>96</v>
+      </c>
       <c r="J1435" s="29"/>
       <c r="K1435" s="29"/>
-      <c r="L1435" s="31"/>
+      <c r="L1435" s="31" t="s">
+        <v>3418</v>
+      </c>
       <c r="M1435" s="29"/>
     </row>
     <row r="1436" spans="1:13" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
added temp lighting network cable
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6326689D-19A7-1649-85B8-595A5FCD323B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4861DD1-5721-3143-A8E5-70FFE9D8677B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1820" yWindow="760" windowWidth="26600" windowHeight="18020" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -18,8 +18,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="8" r:id="rId3"/>
-    <pivotCache cacheId="9" r:id="rId4"/>
+    <pivotCache cacheId="10" r:id="rId3"/>
+    <pivotCache cacheId="11" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11706" uniqueCount="3427">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11708" uniqueCount="3429">
   <si>
     <t>Tag</t>
   </si>
@@ -10325,6 +10325,12 @@
   </si>
   <si>
     <t>to_mixer+C238</t>
+  </si>
+  <si>
+    <t>LAN1</t>
+  </si>
+  <si>
+    <t>temp lighting</t>
   </si>
 </sst>
 </file>
@@ -19840,7 +19846,70 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="9" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Tag" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B56" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -20073,69 +20142,6 @@
     </i>
     <i>
       <x v="53"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of Tag" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="12">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="7"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
     </i>
     <i t="grand">
       <x/>
@@ -24280,11 +24286,17 @@
         <v>284</v>
       </c>
       <c r="B125" s="22" t="s">
-        <v>416</v>
-      </c>
-      <c r="C125" s="23"/>
-      <c r="D125" s="22"/>
-      <c r="E125" s="23"/>
+        <v>250</v>
+      </c>
+      <c r="C125" s="23">
+        <v>7</v>
+      </c>
+      <c r="D125" s="22" t="s">
+        <v>3425</v>
+      </c>
+      <c r="E125" s="23" t="s">
+        <v>3427</v>
+      </c>
       <c r="F125" s="23" t="s">
         <v>224</v>
       </c>
@@ -24296,7 +24308,7 @@
         <v>96</v>
       </c>
       <c r="J125" s="23" t="s">
-        <v>416</v>
+        <v>3428</v>
       </c>
       <c r="K125" s="23"/>
       <c r="L125" s="19"/>

</xml_diff>

<commit_message>
added the hdmi2-sdi path for cumu-g002
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4861DD1-5721-3143-A8E5-70FFE9D8677B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EECB6EE-D7AA-174D-8658-6FDA9F1B9C16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1820" yWindow="760" windowWidth="26600" windowHeight="18020" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -18,8 +18,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="10" r:id="rId3"/>
-    <pivotCache cacheId="11" r:id="rId4"/>
+    <pivotCache cacheId="12" r:id="rId3"/>
+    <pivotCache cacheId="13" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11708" uniqueCount="3429">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11721" uniqueCount="3431">
   <si>
     <t>Tag</t>
   </si>
@@ -10331,6 +10331,12 @@
   </si>
   <si>
     <t>temp lighting</t>
+  </si>
+  <si>
+    <t>hdmi2</t>
+  </si>
+  <si>
+    <t>2607-1400</t>
   </si>
 </sst>
 </file>
@@ -19846,70 +19852,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="10" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="12">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="7"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of Tag" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="11" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="13" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B56" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -20142,6 +20085,69 @@
     </i>
     <i>
       <x v="53"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Tag" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
     </i>
     <i t="grand">
       <x/>
@@ -24387,10 +24393,18 @@
       <c r="A129" s="21" t="s">
         <v>292</v>
       </c>
-      <c r="B129" s="31"/>
-      <c r="C129" s="23"/>
-      <c r="D129" s="22"/>
-      <c r="E129" s="23"/>
+      <c r="B129" s="31" t="s">
+        <v>42</v>
+      </c>
+      <c r="C129" s="23" t="s">
+        <v>30</v>
+      </c>
+      <c r="D129" s="22" t="s">
+        <v>1603</v>
+      </c>
+      <c r="E129" s="23" t="s">
+        <v>3429</v>
+      </c>
       <c r="F129" s="23" t="s">
         <v>30</v>
       </c>
@@ -24404,7 +24418,7 @@
         <v>96</v>
       </c>
       <c r="J129" s="23" t="s">
-        <v>416</v>
+        <v>2982</v>
       </c>
       <c r="K129" s="23" t="s">
         <v>295</v>
@@ -66320,16 +66334,34 @@
       <c r="M1435" s="29"/>
     </row>
     <row r="1436" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1436" s="29"/>
-      <c r="B1436" s="100"/>
-      <c r="C1436" s="83"/>
-      <c r="D1436" s="85"/>
-      <c r="E1436" s="83"/>
-      <c r="F1436" s="31"/>
-      <c r="G1436" s="31"/>
+      <c r="A1436" s="29" t="s">
+        <v>3430</v>
+      </c>
+      <c r="B1436" s="100" t="s">
+        <v>1020</v>
+      </c>
+      <c r="C1436" s="83" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1436" s="85" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1436" s="83" t="s">
+        <v>213</v>
+      </c>
+      <c r="F1436" s="31" t="s">
+        <v>1521</v>
+      </c>
+      <c r="G1436" s="31" t="s">
+        <v>27</v>
+      </c>
       <c r="H1436" s="29"/>
-      <c r="I1436" s="119"/>
-      <c r="J1436" s="29"/>
+      <c r="I1436" s="119" t="s">
+        <v>96</v>
+      </c>
+      <c r="J1436" s="29" t="s">
+        <v>2982</v>
+      </c>
       <c r="K1436" s="29"/>
       <c r="L1436" s="31"/>
       <c r="M1436" s="29"/>

</xml_diff>

<commit_message>
added cables for nursery TV and Stream Deck
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10713"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F2FBCC0-A9AC-EB4D-B95A-689EAD54826F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2412CF21-32B5-0D45-A7EC-5A927DB71B4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1820" yWindow="760" windowWidth="26600" windowHeight="18020" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -18,8 +18,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="12" r:id="rId3"/>
-    <pivotCache cacheId="13" r:id="rId4"/>
+    <pivotCache cacheId="3" r:id="rId3"/>
+    <pivotCache cacheId="4" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11717" uniqueCount="3430">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11752" uniqueCount="3436">
   <si>
     <t>Tag</t>
   </si>
@@ -9720,15 +9720,6 @@
     <t>need to confirm</t>
   </si>
   <si>
-    <t>blank116</t>
-  </si>
-  <si>
-    <t>blank117</t>
-  </si>
-  <si>
-    <t>blank114</t>
-  </si>
-  <si>
     <t>2606-2300</t>
   </si>
   <si>
@@ -10081,9 +10072,6 @@
   </si>
   <si>
     <t>unk1394</t>
-  </si>
-  <si>
-    <t>blank115</t>
   </si>
   <si>
     <t>G2 AVNet</t>
@@ -10334,6 +10322,36 @@
   </si>
   <si>
     <t>2607-1400</t>
+  </si>
+  <si>
+    <t>2608-1900</t>
+  </si>
+  <si>
+    <t>45m</t>
+  </si>
+  <si>
+    <t>Nursery TV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Meant for Remote control but TV doesn't support it. </t>
+  </si>
+  <si>
+    <t>Nursery Call Panel</t>
+  </si>
+  <si>
+    <t>2608-1901</t>
+  </si>
+  <si>
+    <t>jump116</t>
+  </si>
+  <si>
+    <t>jump117</t>
+  </si>
+  <si>
+    <t>2602-1800-F38:B1-F2-R202:Down conduit:B1-F2-R208:B1-F1-R112:B1-F0-R026:B1-F0-R027:B1-F0-R025:B1-F0-F027</t>
+  </si>
+  <si>
+    <t>2602-1800-F38:B1-F2-R202:Down conduit:B1-F2-R208:B1-F1-R112:B1-F0-R026:B1-F0-R027:B1-F0-R025:B1-F0-F029</t>
   </si>
 </sst>
 </file>
@@ -10779,7 +10797,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="138">
+  <cellXfs count="139">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -11044,6 +11062,7 @@
     <xf numFmtId="49" fontId="8" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -19849,7 +19868,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="13" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B56" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -20106,7 +20125,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="12" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="3" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -23105,16 +23124,16 @@
         <v>167</v>
       </c>
       <c r="C84" s="23" t="s">
-        <v>3357</v>
+        <v>3353</v>
       </c>
       <c r="D84" s="22" t="s">
         <v>175</v>
       </c>
       <c r="E84" s="23" t="s">
-        <v>3358</v>
+        <v>3354</v>
       </c>
       <c r="F84" s="23" t="s">
-        <v>3354</v>
+        <v>3350</v>
       </c>
       <c r="G84" s="23"/>
       <c r="H84" s="23" t="s">
@@ -23135,7 +23154,7 @@
         <v>179</v>
       </c>
       <c r="B85" s="22" t="s">
-        <v>3352</v>
+        <v>3348</v>
       </c>
       <c r="C85" s="23" t="s">
         <v>241</v>
@@ -23515,10 +23534,10 @@
     </row>
     <row r="98" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A98" s="29" t="s">
-        <v>3359</v>
+        <v>3355</v>
       </c>
       <c r="B98" s="100" t="s">
-        <v>3352</v>
+        <v>3348</v>
       </c>
       <c r="C98" s="83" t="s">
         <v>1608</v>
@@ -23548,7 +23567,7 @@
     </row>
     <row r="99" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A99" s="21" t="s">
-        <v>3353</v>
+        <v>3349</v>
       </c>
       <c r="B99" s="22" t="s">
         <v>55</v>
@@ -23867,7 +23886,7 @@
         <v>24</v>
       </c>
       <c r="D109" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E109" s="23" t="s">
         <v>2252</v>
@@ -23885,7 +23904,7 @@
         <v>96</v>
       </c>
       <c r="J109" s="23" t="s">
-        <v>3256</v>
+        <v>3253</v>
       </c>
       <c r="K109" s="23"/>
       <c r="L109" s="19"/>
@@ -23955,7 +23974,7 @@
     </row>
     <row r="112" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A112" s="21" t="s">
-        <v>3355</v>
+        <v>3351</v>
       </c>
       <c r="B112" s="22" t="s">
         <v>167</v>
@@ -23964,7 +23983,7 @@
         <v>1608</v>
       </c>
       <c r="D112" s="22" t="s">
-        <v>3352</v>
+        <v>3348</v>
       </c>
       <c r="E112" s="23" t="s">
         <v>202</v>
@@ -23988,7 +24007,7 @@
     </row>
     <row r="113" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A113" s="21" t="s">
-        <v>3356</v>
+        <v>3352</v>
       </c>
       <c r="B113" s="22" t="s">
         <v>167</v>
@@ -23997,7 +24016,7 @@
         <v>241</v>
       </c>
       <c r="D113" s="22" t="s">
-        <v>3352</v>
+        <v>3348</v>
       </c>
       <c r="E113" s="23" t="s">
         <v>203</v>
@@ -24021,68 +24040,142 @@
     </row>
     <row r="114" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A114" s="21" t="s">
-        <v>3227</v>
-      </c>
-      <c r="B114" s="22"/>
-      <c r="C114" s="23"/>
-      <c r="D114" s="22"/>
-      <c r="E114" s="23"/>
-      <c r="F114" s="23"/>
-      <c r="G114" s="22"/>
-      <c r="H114" s="23"/>
-      <c r="I114" s="23"/>
-      <c r="J114" s="23"/>
-      <c r="K114" s="23"/>
+        <v>3426</v>
+      </c>
+      <c r="B114" s="22" t="s">
+        <v>1598</v>
+      </c>
+      <c r="C114" s="23" t="s">
+        <v>2361</v>
+      </c>
+      <c r="D114" s="22" t="s">
+        <v>89</v>
+      </c>
+      <c r="E114" s="23" t="s">
+        <v>2146</v>
+      </c>
+      <c r="F114" s="23" t="s">
+        <v>228</v>
+      </c>
+      <c r="G114" s="22" t="s">
+        <v>1447</v>
+      </c>
+      <c r="H114" s="23" t="s">
+        <v>3427</v>
+      </c>
+      <c r="I114" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="J114" s="23" t="s">
+        <v>3428</v>
+      </c>
+      <c r="K114" s="23" t="s">
+        <v>3429</v>
+      </c>
       <c r="L114" s="23"/>
-      <c r="M114" s="24"/>
+      <c r="M114" s="24" t="s">
+        <v>3434</v>
+      </c>
     </row>
     <row r="115" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A115" s="21" t="s">
-        <v>3346</v>
-      </c>
-      <c r="B115" s="22"/>
-      <c r="C115" s="23"/>
-      <c r="D115" s="22"/>
-      <c r="E115" s="23"/>
-      <c r="F115" s="23"/>
-      <c r="G115" s="23"/>
-      <c r="H115" s="23"/>
-      <c r="I115" s="23"/>
-      <c r="J115" s="23"/>
+        <v>3431</v>
+      </c>
+      <c r="B115" s="22" t="s">
+        <v>1598</v>
+      </c>
+      <c r="C115" s="23" t="s">
+        <v>2362</v>
+      </c>
+      <c r="D115" s="22" t="s">
+        <v>2959</v>
+      </c>
+      <c r="E115" s="23" t="s">
+        <v>2146</v>
+      </c>
+      <c r="F115" s="23" t="s">
+        <v>228</v>
+      </c>
+      <c r="G115" s="22" t="s">
+        <v>1447</v>
+      </c>
+      <c r="H115" s="23" t="s">
+        <v>3048</v>
+      </c>
+      <c r="I115" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="J115" s="23" t="s">
+        <v>3430</v>
+      </c>
       <c r="K115" s="23"/>
-      <c r="L115" s="19"/>
-      <c r="M115" s="20"/>
+      <c r="L115" s="138"/>
+      <c r="M115" s="19" t="s">
+        <v>3435</v>
+      </c>
     </row>
     <row r="116" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A116" s="28" t="s">
-        <v>3225</v>
-      </c>
-      <c r="B116" s="22"/>
-      <c r="C116" s="23"/>
-      <c r="D116" s="22"/>
-      <c r="E116" s="23"/>
-      <c r="F116" s="23"/>
-      <c r="G116" s="23"/>
+        <v>3432</v>
+      </c>
+      <c r="B116" s="22" t="s">
+        <v>1640</v>
+      </c>
+      <c r="C116" s="23">
+        <v>15</v>
+      </c>
+      <c r="D116" s="22" t="s">
+        <v>1598</v>
+      </c>
+      <c r="E116" s="23" t="s">
+        <v>2354</v>
+      </c>
+      <c r="F116" s="23" t="s">
+        <v>228</v>
+      </c>
+      <c r="G116" s="22" t="s">
+        <v>1447</v>
+      </c>
       <c r="H116" s="23"/>
-      <c r="I116" s="23"/>
-      <c r="J116" s="23"/>
+      <c r="I116" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="J116" s="23" t="s">
+        <v>3428</v>
+      </c>
       <c r="K116" s="23"/>
       <c r="L116" s="23"/>
       <c r="M116" s="24"/>
     </row>
     <row r="117" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A117" s="21" t="s">
-        <v>3226</v>
-      </c>
-      <c r="B117" s="22"/>
-      <c r="C117" s="23"/>
-      <c r="D117" s="22"/>
-      <c r="E117" s="23"/>
-      <c r="F117" s="23"/>
-      <c r="G117" s="23"/>
+        <v>3433</v>
+      </c>
+      <c r="B117" s="22" t="s">
+        <v>1640</v>
+      </c>
+      <c r="C117" s="23">
+        <v>16</v>
+      </c>
+      <c r="D117" s="22" t="s">
+        <v>1598</v>
+      </c>
+      <c r="E117" s="23" t="s">
+        <v>2355</v>
+      </c>
+      <c r="F117" s="23" t="s">
+        <v>228</v>
+      </c>
+      <c r="G117" s="22" t="s">
+        <v>1447</v>
+      </c>
       <c r="H117" s="23"/>
-      <c r="I117" s="23"/>
-      <c r="J117" s="23"/>
+      <c r="I117" s="23" t="s">
+        <v>60</v>
+      </c>
+      <c r="J117" s="23" t="s">
+        <v>3430</v>
+      </c>
       <c r="K117" s="23"/>
       <c r="L117" s="19"/>
       <c r="M117" s="20"/>
@@ -24287,10 +24380,10 @@
         <v>7</v>
       </c>
       <c r="D125" s="22" t="s">
-        <v>3424</v>
+        <v>3420</v>
       </c>
       <c r="E125" s="23" t="s">
-        <v>3426</v>
+        <v>3422</v>
       </c>
       <c r="F125" s="23" t="s">
         <v>223</v>
@@ -24303,7 +24396,7 @@
         <v>96</v>
       </c>
       <c r="J125" s="23" t="s">
-        <v>3427</v>
+        <v>3423</v>
       </c>
       <c r="K125" s="23"/>
       <c r="L125" s="19"/>
@@ -24392,7 +24485,7 @@
         <v>1602</v>
       </c>
       <c r="E129" s="23" t="s">
-        <v>3428</v>
+        <v>3424</v>
       </c>
       <c r="F129" s="23" t="s">
         <v>30</v>
@@ -27965,7 +28058,7 @@
         <v>465</v>
       </c>
       <c r="C234" s="29" t="s">
-        <v>3425</v>
+        <v>3421</v>
       </c>
       <c r="D234" s="31" t="s">
         <v>620</v>
@@ -28101,10 +28194,10 @@
         <v>545</v>
       </c>
       <c r="B239" s="126" t="s">
-        <v>3424</v>
+        <v>3420</v>
       </c>
       <c r="C239" s="29" t="s">
-        <v>3423</v>
+        <v>3419</v>
       </c>
       <c r="D239" s="31" t="s">
         <v>480</v>
@@ -28126,7 +28219,7 @@
       </c>
       <c r="J239" s="29"/>
       <c r="K239" s="29" t="s">
-        <v>3422</v>
+        <v>3418</v>
       </c>
       <c r="L239" s="31"/>
       <c r="M239" s="29"/>
@@ -29287,7 +29380,7 @@
         <v>17</v>
       </c>
       <c r="D279" s="31" t="s">
-        <v>3245</v>
+        <v>3242</v>
       </c>
       <c r="E279" s="29" t="s">
         <v>2146</v>
@@ -29305,7 +29398,7 @@
         <v>96</v>
       </c>
       <c r="J279" s="29" t="s">
-        <v>3246</v>
+        <v>3243</v>
       </c>
       <c r="K279" s="29"/>
       <c r="L279" s="31"/>
@@ -33653,7 +33746,7 @@
         <v>96</v>
       </c>
       <c r="J425" s="31" t="s">
-        <v>3349</v>
+        <v>3345</v>
       </c>
       <c r="K425" s="29"/>
       <c r="L425" s="31"/>
@@ -41433,7 +41526,7 @@
         <v>96</v>
       </c>
       <c r="J661" s="130" t="s">
-        <v>3350</v>
+        <v>3346</v>
       </c>
       <c r="K661" s="128" t="s">
         <v>441</v>
@@ -48132,7 +48225,7 @@
         <v>96</v>
       </c>
       <c r="J870" s="85" t="s">
-        <v>3347</v>
+        <v>3343</v>
       </c>
       <c r="K870" s="29"/>
       <c r="L870" s="31"/>
@@ -48282,7 +48375,7 @@
     </row>
     <row r="875" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A875" s="29" t="s">
-        <v>3360</v>
+        <v>3356</v>
       </c>
       <c r="B875" s="58" t="s">
         <v>25</v>
@@ -58597,7 +58690,7 @@
     </row>
     <row r="1188" spans="1:13" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="A1188" s="29" t="s">
-        <v>3386</v>
+        <v>3382</v>
       </c>
       <c r="B1188" s="80"/>
       <c r="C1188" s="83"/>
@@ -58614,7 +58707,7 @@
     </row>
     <row r="1189" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1189" s="29" t="s">
-        <v>3387</v>
+        <v>3383</v>
       </c>
       <c r="B1189" s="85" t="s">
         <v>2585</v>
@@ -58645,7 +58738,7 @@
     </row>
     <row r="1190" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1190" s="29" t="s">
-        <v>3388</v>
+        <v>3384</v>
       </c>
       <c r="B1190" s="100" t="s">
         <v>1642</v>
@@ -61681,7 +61774,7 @@
     </row>
     <row r="1280" spans="1:13" s="131" customFormat="1" ht="64" x14ac:dyDescent="0.2">
       <c r="A1280" s="128" t="s">
-        <v>3254</v>
+        <v>3251</v>
       </c>
       <c r="B1280" s="100" t="s">
         <v>236</v>
@@ -62842,7 +62935,7 @@
         <v>96</v>
       </c>
       <c r="J1320" s="29" t="s">
-        <v>3351</v>
+        <v>3347</v>
       </c>
       <c r="K1320" s="29" t="s">
         <v>441</v>
@@ -63274,7 +63367,7 @@
         <v>96</v>
       </c>
       <c r="J1335" s="29" t="s">
-        <v>3348</v>
+        <v>3344</v>
       </c>
       <c r="K1335" s="29"/>
       <c r="L1335" s="31"/>
@@ -63433,25 +63526,25 @@
     </row>
     <row r="1341" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1341" s="29" t="s">
-        <v>3228</v>
+        <v>3225</v>
       </c>
       <c r="B1341" s="100" t="s">
-        <v>3241</v>
+        <v>3238</v>
       </c>
       <c r="C1341" s="83" t="s">
-        <v>3230</v>
+        <v>3227</v>
       </c>
       <c r="D1341" s="85" t="s">
-        <v>3229</v>
+        <v>3226</v>
       </c>
       <c r="E1341" s="83" t="s">
-        <v>3230</v>
+        <v>3227</v>
       </c>
       <c r="F1341" s="31" t="s">
         <v>883</v>
       </c>
       <c r="G1341" s="31" t="s">
-        <v>3292</v>
+        <v>3289</v>
       </c>
       <c r="H1341" s="29"/>
       <c r="I1341" s="119" t="s">
@@ -63459,23 +63552,23 @@
       </c>
       <c r="J1341" s="29"/>
       <c r="K1341" s="29" t="s">
-        <v>3240</v>
+        <v>3237</v>
       </c>
       <c r="L1341" s="31"/>
       <c r="M1341" s="29"/>
     </row>
     <row r="1342" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1342" s="29" t="s">
-        <v>3231</v>
+        <v>3228</v>
       </c>
       <c r="B1342" s="85" t="s">
-        <v>3229</v>
+        <v>3226</v>
       </c>
       <c r="C1342" s="83" t="s">
         <v>697</v>
       </c>
       <c r="D1342" s="85" t="s">
-        <v>3244</v>
+        <v>3241</v>
       </c>
       <c r="E1342" s="83" t="s">
         <v>441</v>
@@ -63499,22 +63592,22 @@
     </row>
     <row r="1343" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1343" s="29" t="s">
-        <v>3232</v>
+        <v>3229</v>
       </c>
       <c r="B1343" s="85" t="s">
-        <v>3244</v>
+        <v>3241</v>
       </c>
       <c r="C1343" s="83" t="s">
         <v>2525</v>
       </c>
       <c r="D1343" s="85" t="s">
-        <v>3233</v>
+        <v>3230</v>
       </c>
       <c r="E1343" s="83" t="s">
         <v>436</v>
       </c>
       <c r="F1343" s="31" t="s">
-        <v>3234</v>
+        <v>3231</v>
       </c>
       <c r="G1343" s="31" t="s">
         <v>1447</v>
@@ -63532,16 +63625,16 @@
     </row>
     <row r="1344" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1344" s="29" t="s">
-        <v>3235</v>
+        <v>3232</v>
       </c>
       <c r="B1344" s="85" t="s">
+        <v>3230</v>
+      </c>
+      <c r="C1344" s="83" t="s">
         <v>3233</v>
       </c>
-      <c r="C1344" s="83" t="s">
-        <v>3236</v>
-      </c>
       <c r="D1344" s="85" t="s">
-        <v>3237</v>
+        <v>3234</v>
       </c>
       <c r="E1344" s="83" t="s">
         <v>436</v>
@@ -63565,13 +63658,13 @@
     </row>
     <row r="1345" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1345" s="29" t="s">
-        <v>3239</v>
+        <v>3236</v>
       </c>
       <c r="B1345" s="85" t="s">
-        <v>3233</v>
+        <v>3230</v>
       </c>
       <c r="C1345" s="83" t="s">
-        <v>3238</v>
+        <v>3235</v>
       </c>
       <c r="D1345" s="85" t="s">
         <v>3050</v>
@@ -63600,7 +63693,7 @@
     </row>
     <row r="1346" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1346" s="29" t="s">
-        <v>3242</v>
+        <v>3239</v>
       </c>
       <c r="B1346" s="85" t="s">
         <v>3050</v>
@@ -63612,7 +63705,7 @@
         <v>236</v>
       </c>
       <c r="E1346" s="83" t="s">
-        <v>3243</v>
+        <v>3240</v>
       </c>
       <c r="F1346" s="31"/>
       <c r="G1346" s="31" t="s">
@@ -63629,7 +63722,7 @@
     </row>
     <row r="1347" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1347" s="29" t="s">
-        <v>3255</v>
+        <v>3252</v>
       </c>
       <c r="B1347" s="100" t="s">
         <v>236</v>
@@ -63638,10 +63731,10 @@
         <v>1200</v>
       </c>
       <c r="D1347" s="136" t="s">
-        <v>3247</v>
+        <v>3244</v>
       </c>
       <c r="E1347" s="83" t="s">
-        <v>3248</v>
+        <v>3245</v>
       </c>
       <c r="F1347" s="31" t="s">
         <v>228</v>
@@ -63654,17 +63747,17 @@
         <v>60</v>
       </c>
       <c r="J1347" s="29" t="s">
-        <v>3250</v>
+        <v>3247</v>
       </c>
       <c r="K1347" s="29" t="s">
-        <v>3249</v>
+        <v>3246</v>
       </c>
       <c r="L1347" s="31"/>
       <c r="M1347" s="29"/>
     </row>
     <row r="1348" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1348" s="29" t="s">
-        <v>3252</v>
+        <v>3249</v>
       </c>
       <c r="B1348" s="100" t="s">
         <v>236</v>
@@ -63673,7 +63766,7 @@
         <v>1232</v>
       </c>
       <c r="D1348" s="85" t="s">
-        <v>3251</v>
+        <v>3248</v>
       </c>
       <c r="E1348" s="83" t="s">
         <v>2146</v>
@@ -63693,7 +63786,7 @@
     </row>
     <row r="1349" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1349" s="29" t="s">
-        <v>3253</v>
+        <v>3250</v>
       </c>
       <c r="B1349" s="100" t="s">
         <v>236</v>
@@ -63718,16 +63811,16 @@
     </row>
     <row r="1350" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1350" s="29" t="s">
-        <v>3258</v>
+        <v>3255</v>
       </c>
       <c r="B1350" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1350" s="83" t="s">
         <v>2250</v>
       </c>
       <c r="D1350" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1350" s="83" t="s">
         <v>2344</v>
@@ -63749,16 +63842,16 @@
     </row>
     <row r="1351" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1351" s="29" t="s">
-        <v>3259</v>
+        <v>3256</v>
       </c>
       <c r="B1351" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1351" s="83" t="s">
         <v>2251</v>
       </c>
       <c r="D1351" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1351" s="83" t="s">
         <v>2345</v>
@@ -63780,16 +63873,16 @@
     </row>
     <row r="1352" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1352" s="29" t="s">
-        <v>3260</v>
+        <v>3257</v>
       </c>
       <c r="B1352" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1352" s="83" t="s">
         <v>2252</v>
       </c>
       <c r="D1352" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1352" s="83" t="s">
         <v>2346</v>
@@ -63811,16 +63904,16 @@
     </row>
     <row r="1353" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1353" s="29" t="s">
-        <v>3261</v>
+        <v>3258</v>
       </c>
       <c r="B1353" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1353" s="83" t="s">
         <v>2253</v>
       </c>
       <c r="D1353" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1353" s="83" t="s">
         <v>1818</v>
@@ -63842,16 +63935,16 @@
     </row>
     <row r="1354" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1354" s="29" t="s">
-        <v>3262</v>
+        <v>3259</v>
       </c>
       <c r="B1354" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1354" s="83" t="s">
         <v>2249</v>
       </c>
       <c r="D1354" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1354" s="83" t="s">
         <v>2254</v>
@@ -63873,16 +63966,16 @@
     </row>
     <row r="1355" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1355" s="29" t="s">
-        <v>3263</v>
+        <v>3260</v>
       </c>
       <c r="B1355" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1355" s="83" t="s">
         <v>2350</v>
       </c>
       <c r="D1355" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1355" s="83" t="s">
         <v>1998</v>
@@ -63904,16 +63997,16 @@
     </row>
     <row r="1356" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1356" s="29" t="s">
-        <v>3264</v>
+        <v>3261</v>
       </c>
       <c r="B1356" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1356" s="83" t="s">
         <v>2246</v>
       </c>
       <c r="D1356" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1356" s="83" t="s">
         <v>2255</v>
@@ -63935,16 +64028,16 @@
     </row>
     <row r="1357" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1357" s="29" t="s">
-        <v>3265</v>
+        <v>3262</v>
       </c>
       <c r="B1357" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1357" s="83" t="s">
         <v>2247</v>
       </c>
       <c r="D1357" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1357" s="83" t="s">
         <v>2256</v>
@@ -63966,16 +64059,16 @@
     </row>
     <row r="1358" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1358" s="29" t="s">
-        <v>3266</v>
+        <v>3263</v>
       </c>
       <c r="B1358" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1358" s="83" t="s">
         <v>2248</v>
       </c>
       <c r="D1358" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1358" s="83" t="s">
         <v>2229</v>
@@ -63997,16 +64090,16 @@
     </row>
     <row r="1359" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1359" s="29" t="s">
-        <v>3267</v>
+        <v>3264</v>
       </c>
       <c r="B1359" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1359" s="83" t="s">
         <v>2351</v>
       </c>
       <c r="D1359" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1359" s="83" t="s">
         <v>2257</v>
@@ -64028,16 +64121,16 @@
     </row>
     <row r="1360" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1360" s="29" t="s">
-        <v>3268</v>
+        <v>3265</v>
       </c>
       <c r="B1360" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1360" s="83" t="s">
         <v>1812</v>
       </c>
       <c r="D1360" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1360" s="83" t="s">
         <v>1814</v>
@@ -64059,16 +64152,16 @@
     </row>
     <row r="1361" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1361" s="29" t="s">
-        <v>3269</v>
+        <v>3266</v>
       </c>
       <c r="B1361" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1361" s="83" t="s">
         <v>2231</v>
       </c>
       <c r="D1361" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1361" s="83" t="s">
         <v>1932</v>
@@ -64090,16 +64183,16 @@
     </row>
     <row r="1362" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1362" s="29" t="s">
-        <v>3270</v>
+        <v>3267</v>
       </c>
       <c r="B1362" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1362" s="83" t="s">
         <v>1819</v>
       </c>
       <c r="D1362" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1362" s="83" t="s">
         <v>1816</v>
@@ -64121,16 +64214,16 @@
     </row>
     <row r="1363" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1363" s="29" t="s">
-        <v>3271</v>
+        <v>3268</v>
       </c>
       <c r="B1363" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1363" s="83" t="s">
         <v>1820</v>
       </c>
       <c r="D1363" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1363" s="83" t="s">
         <v>1815</v>
@@ -64152,16 +64245,16 @@
     </row>
     <row r="1364" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1364" s="29" t="s">
-        <v>3272</v>
+        <v>3269</v>
       </c>
       <c r="B1364" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1364" s="83" t="s">
         <v>2228</v>
       </c>
       <c r="D1364" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1364" s="83" t="s">
         <v>2258</v>
@@ -64183,16 +64276,16 @@
     </row>
     <row r="1365" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1365" s="29" t="s">
-        <v>3273</v>
+        <v>3270</v>
       </c>
       <c r="B1365" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1365" s="83" t="s">
         <v>2227</v>
       </c>
       <c r="D1365" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1365" s="83" t="s">
         <v>2347</v>
@@ -64214,16 +64307,16 @@
     </row>
     <row r="1366" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1366" s="29" t="s">
-        <v>3274</v>
+        <v>3271</v>
       </c>
       <c r="B1366" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1366" s="83" t="s">
         <v>1824</v>
       </c>
       <c r="D1366" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1366" s="83" t="s">
         <v>1821</v>
@@ -64245,16 +64338,16 @@
     </row>
     <row r="1367" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1367" s="29" t="s">
-        <v>3275</v>
+        <v>3272</v>
       </c>
       <c r="B1367" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1367" s="83" t="s">
         <v>2352</v>
       </c>
       <c r="D1367" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1367" s="83" t="s">
         <v>2359</v>
@@ -64276,16 +64369,16 @@
     </row>
     <row r="1368" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1368" s="29" t="s">
-        <v>3276</v>
+        <v>3273</v>
       </c>
       <c r="B1368" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1368" s="83" t="s">
         <v>2353</v>
       </c>
       <c r="D1368" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1368" s="83" t="s">
         <v>2360</v>
@@ -64307,16 +64400,16 @@
     </row>
     <row r="1369" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1369" s="29" t="s">
-        <v>3277</v>
+        <v>3274</v>
       </c>
       <c r="B1369" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1369" s="83" t="s">
         <v>2354</v>
       </c>
       <c r="D1369" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1369" s="83" t="s">
         <v>2361</v>
@@ -64338,16 +64431,16 @@
     </row>
     <row r="1370" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1370" s="29" t="s">
-        <v>3278</v>
+        <v>3275</v>
       </c>
       <c r="B1370" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1370" s="83" t="s">
         <v>2355</v>
       </c>
       <c r="D1370" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1370" s="83" t="s">
         <v>2362</v>
@@ -64369,16 +64462,16 @@
     </row>
     <row r="1371" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1371" s="29" t="s">
-        <v>3279</v>
+        <v>3276</v>
       </c>
       <c r="B1371" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1371" s="83" t="s">
         <v>2356</v>
       </c>
       <c r="D1371" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1371" s="83" t="s">
         <v>2363</v>
@@ -64400,16 +64493,16 @@
     </row>
     <row r="1372" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1372" s="29" t="s">
-        <v>3280</v>
+        <v>3277</v>
       </c>
       <c r="B1372" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1372" s="83" t="s">
         <v>2357</v>
       </c>
       <c r="D1372" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1372" s="83" t="s">
         <v>2364</v>
@@ -64431,16 +64524,16 @@
     </row>
     <row r="1373" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1373" s="29" t="s">
-        <v>3281</v>
+        <v>3278</v>
       </c>
       <c r="B1373" s="22" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1373" s="83" t="s">
         <v>2358</v>
       </c>
       <c r="D1373" s="89" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1373" s="83" t="s">
         <v>2365</v>
@@ -64462,7 +64555,7 @@
     </row>
     <row r="1374" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1374" s="29" t="s">
-        <v>3283</v>
+        <v>3280</v>
       </c>
       <c r="B1374" s="85" t="s">
         <v>3050</v>
@@ -64471,7 +64564,7 @@
         <v>1818</v>
       </c>
       <c r="D1374" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1374" s="83" t="s">
         <v>2250</v>
@@ -64487,7 +64580,7 @@
         <v>96</v>
       </c>
       <c r="J1374" s="29" t="s">
-        <v>3284</v>
+        <v>3281</v>
       </c>
       <c r="K1374" s="29"/>
       <c r="L1374" s="31"/>
@@ -64495,7 +64588,7 @@
     </row>
     <row r="1375" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1375" s="29" t="s">
-        <v>3285</v>
+        <v>3282</v>
       </c>
       <c r="B1375" s="85" t="s">
         <v>3050</v>
@@ -64504,7 +64597,7 @@
         <v>2254</v>
       </c>
       <c r="D1375" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1375" s="83" t="s">
         <v>2227</v>
@@ -64526,7 +64619,7 @@
     </row>
     <row r="1376" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1376" s="29" t="s">
-        <v>3286</v>
+        <v>3283</v>
       </c>
       <c r="B1376" s="85" t="s">
         <v>3050</v>
@@ -64535,13 +64628,13 @@
         <v>2255</v>
       </c>
       <c r="D1376" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="E1376" s="83" t="s">
         <v>1824</v>
       </c>
       <c r="F1376" s="31" t="s">
-        <v>3287</v>
+        <v>3284</v>
       </c>
       <c r="G1376" s="31" t="s">
         <v>1447</v>
@@ -64551,7 +64644,7 @@
         <v>96</v>
       </c>
       <c r="J1376" s="29" t="s">
-        <v>3282</v>
+        <v>3279</v>
       </c>
       <c r="K1376" s="29"/>
       <c r="L1376" s="31"/>
@@ -64559,7 +64652,7 @@
     </row>
     <row r="1377" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1377" s="29" t="s">
-        <v>3288</v>
+        <v>3285</v>
       </c>
       <c r="B1377" s="85" t="s">
         <v>3050</v>
@@ -64568,13 +64661,13 @@
         <v>2229</v>
       </c>
       <c r="D1377" s="85" t="s">
-        <v>3290</v>
+        <v>3287</v>
       </c>
       <c r="E1377" s="83" t="s">
-        <v>3289</v>
+        <v>3286</v>
       </c>
       <c r="F1377" s="31" t="s">
-        <v>3287</v>
+        <v>3284</v>
       </c>
       <c r="G1377" s="31" t="s">
         <v>1447</v>
@@ -64584,7 +64677,7 @@
         <v>96</v>
       </c>
       <c r="J1377" s="29" t="s">
-        <v>3291</v>
+        <v>3288</v>
       </c>
       <c r="K1377" s="29"/>
       <c r="L1377" s="31"/>
@@ -64592,16 +64685,16 @@
     </row>
     <row r="1378" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1378" s="29" t="s">
-        <v>3308</v>
+        <v>3305</v>
       </c>
       <c r="B1378" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1378" s="83" t="s">
         <v>2344</v>
       </c>
       <c r="D1378" s="85" t="s">
-        <v>3293</v>
+        <v>3290</v>
       </c>
       <c r="E1378" s="83" t="s">
         <v>2146</v>
@@ -64615,7 +64708,7 @@
         <v>60</v>
       </c>
       <c r="J1378" s="29" t="s">
-        <v>3332</v>
+        <v>3329</v>
       </c>
       <c r="K1378" s="29"/>
       <c r="L1378" s="31"/>
@@ -64623,16 +64716,16 @@
     </row>
     <row r="1379" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1379" s="29" t="s">
-        <v>3309</v>
+        <v>3306</v>
       </c>
       <c r="B1379" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1379" s="83" t="s">
         <v>2345</v>
       </c>
       <c r="D1379" s="85" t="s">
-        <v>3294</v>
+        <v>3291</v>
       </c>
       <c r="E1379" s="83" t="s">
         <v>2146</v>
@@ -64646,7 +64739,7 @@
         <v>60</v>
       </c>
       <c r="J1379" s="29" t="s">
-        <v>3333</v>
+        <v>3330</v>
       </c>
       <c r="K1379" s="29"/>
       <c r="L1379" s="31"/>
@@ -64654,16 +64747,16 @@
     </row>
     <row r="1380" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1380" s="29" t="s">
-        <v>3310</v>
+        <v>3307</v>
       </c>
       <c r="B1380" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1380" s="83" t="s">
         <v>2346</v>
       </c>
       <c r="D1380" s="85" t="s">
-        <v>3295</v>
+        <v>3292</v>
       </c>
       <c r="E1380" s="83" t="s">
         <v>2146</v>
@@ -64677,7 +64770,7 @@
         <v>60</v>
       </c>
       <c r="J1380" s="29" t="s">
-        <v>3334</v>
+        <v>3331</v>
       </c>
       <c r="K1380" s="29"/>
       <c r="L1380" s="31"/>
@@ -64685,16 +64778,16 @@
     </row>
     <row r="1381" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1381" s="29" t="s">
-        <v>3311</v>
+        <v>3308</v>
       </c>
       <c r="B1381" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1381" s="83" t="s">
         <v>1818</v>
       </c>
       <c r="D1381" s="85" t="s">
-        <v>3296</v>
+        <v>3293</v>
       </c>
       <c r="E1381" s="83" t="s">
         <v>2146</v>
@@ -64708,7 +64801,7 @@
         <v>60</v>
       </c>
       <c r="J1381" s="29" t="s">
-        <v>3335</v>
+        <v>3332</v>
       </c>
       <c r="K1381" s="29"/>
       <c r="L1381" s="31"/>
@@ -64716,16 +64809,16 @@
     </row>
     <row r="1382" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1382" s="29" t="s">
-        <v>3312</v>
+        <v>3309</v>
       </c>
       <c r="B1382" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1382" s="83" t="s">
         <v>2254</v>
       </c>
       <c r="D1382" s="85" t="s">
-        <v>3297</v>
+        <v>3294</v>
       </c>
       <c r="E1382" s="83" t="s">
         <v>2146</v>
@@ -64739,7 +64832,7 @@
         <v>60</v>
       </c>
       <c r="J1382" s="29" t="s">
-        <v>3336</v>
+        <v>3333</v>
       </c>
       <c r="K1382" s="29"/>
       <c r="L1382" s="31"/>
@@ -64747,16 +64840,16 @@
     </row>
     <row r="1383" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1383" s="29" t="s">
-        <v>3313</v>
+        <v>3310</v>
       </c>
       <c r="B1383" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1383" s="83" t="s">
         <v>1998</v>
       </c>
       <c r="D1383" s="85" t="s">
-        <v>3298</v>
+        <v>3295</v>
       </c>
       <c r="E1383" s="83" t="s">
         <v>2146</v>
@@ -64770,7 +64863,7 @@
         <v>60</v>
       </c>
       <c r="J1383" s="29" t="s">
-        <v>3337</v>
+        <v>3334</v>
       </c>
       <c r="K1383" s="29"/>
       <c r="L1383" s="31"/>
@@ -64778,16 +64871,16 @@
     </row>
     <row r="1384" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1384" s="29" t="s">
-        <v>3314</v>
+        <v>3311</v>
       </c>
       <c r="B1384" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1384" s="83" t="s">
         <v>2255</v>
       </c>
       <c r="D1384" s="85" t="s">
-        <v>3299</v>
+        <v>3296</v>
       </c>
       <c r="E1384" s="83" t="s">
         <v>2146</v>
@@ -64801,7 +64894,7 @@
         <v>60</v>
       </c>
       <c r="J1384" s="29" t="s">
-        <v>3338</v>
+        <v>3335</v>
       </c>
       <c r="K1384" s="29"/>
       <c r="L1384" s="31"/>
@@ -64809,16 +64902,16 @@
     </row>
     <row r="1385" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1385" s="29" t="s">
-        <v>3315</v>
+        <v>3312</v>
       </c>
       <c r="B1385" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1385" s="83" t="s">
         <v>2256</v>
       </c>
       <c r="D1385" s="85" t="s">
-        <v>3300</v>
+        <v>3297</v>
       </c>
       <c r="E1385" s="83" t="s">
         <v>2146</v>
@@ -64832,7 +64925,7 @@
         <v>60</v>
       </c>
       <c r="J1385" s="29" t="s">
-        <v>3339</v>
+        <v>3336</v>
       </c>
       <c r="K1385" s="29"/>
       <c r="L1385" s="31"/>
@@ -64840,16 +64933,16 @@
     </row>
     <row r="1386" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1386" s="29" t="s">
-        <v>3316</v>
+        <v>3313</v>
       </c>
       <c r="B1386" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1386" s="83" t="s">
         <v>2229</v>
       </c>
       <c r="D1386" s="85" t="s">
-        <v>3301</v>
+        <v>3298</v>
       </c>
       <c r="E1386" s="83" t="s">
         <v>2146</v>
@@ -64863,7 +64956,7 @@
         <v>60</v>
       </c>
       <c r="J1386" s="29" t="s">
-        <v>3340</v>
+        <v>3337</v>
       </c>
       <c r="K1386" s="29"/>
       <c r="L1386" s="31"/>
@@ -64871,10 +64964,10 @@
     </row>
     <row r="1387" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1387" s="29" t="s">
-        <v>3324</v>
+        <v>3321</v>
       </c>
       <c r="B1387" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1387" s="83" t="s">
         <v>2257</v>
@@ -64888,7 +64981,7 @@
         <v>60</v>
       </c>
       <c r="J1387" s="29" t="s">
-        <v>3344</v>
+        <v>3341</v>
       </c>
       <c r="K1387" s="29"/>
       <c r="L1387" s="31"/>
@@ -64896,16 +64989,16 @@
     </row>
     <row r="1388" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1388" s="29" t="s">
-        <v>3317</v>
+        <v>3314</v>
       </c>
       <c r="B1388" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1388" s="83" t="s">
         <v>1814</v>
       </c>
       <c r="D1388" s="85" t="s">
-        <v>3302</v>
+        <v>3299</v>
       </c>
       <c r="E1388" s="83" t="s">
         <v>2146</v>
@@ -64919,7 +65012,7 @@
         <v>60</v>
       </c>
       <c r="J1388" s="29" t="s">
-        <v>3341</v>
+        <v>3338</v>
       </c>
       <c r="K1388" s="29"/>
       <c r="L1388" s="31"/>
@@ -64927,16 +65020,16 @@
     </row>
     <row r="1389" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1389" s="29" t="s">
-        <v>3318</v>
+        <v>3315</v>
       </c>
       <c r="B1389" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1389" s="83" t="s">
         <v>1932</v>
       </c>
       <c r="D1389" s="85" t="s">
-        <v>3303</v>
+        <v>3300</v>
       </c>
       <c r="E1389" s="83" t="s">
         <v>2146</v>
@@ -64950,7 +65043,7 @@
         <v>60</v>
       </c>
       <c r="J1389" s="29" t="s">
-        <v>3342</v>
+        <v>3339</v>
       </c>
       <c r="K1389" s="29"/>
       <c r="L1389" s="31"/>
@@ -64958,16 +65051,16 @@
     </row>
     <row r="1390" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1390" s="29" t="s">
-        <v>3319</v>
+        <v>3316</v>
       </c>
       <c r="B1390" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1390" s="83" t="s">
         <v>1816</v>
       </c>
       <c r="D1390" s="85" t="s">
-        <v>3304</v>
+        <v>3301</v>
       </c>
       <c r="E1390" s="83" t="s">
         <v>2146</v>
@@ -64981,7 +65074,7 @@
         <v>60</v>
       </c>
       <c r="J1390" s="29" t="s">
-        <v>3342</v>
+        <v>3339</v>
       </c>
       <c r="K1390" s="29"/>
       <c r="L1390" s="31"/>
@@ -64989,16 +65082,16 @@
     </row>
     <row r="1391" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1391" s="29" t="s">
-        <v>3320</v>
+        <v>3317</v>
       </c>
       <c r="B1391" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1391" s="83" t="s">
         <v>1815</v>
       </c>
       <c r="D1391" s="85" t="s">
-        <v>3305</v>
+        <v>3302</v>
       </c>
       <c r="E1391" s="83" t="s">
         <v>2146</v>
@@ -65012,7 +65105,7 @@
         <v>60</v>
       </c>
       <c r="J1391" s="29" t="s">
-        <v>3342</v>
+        <v>3339</v>
       </c>
       <c r="K1391" s="29"/>
       <c r="L1391" s="31"/>
@@ -65020,16 +65113,16 @@
     </row>
     <row r="1392" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1392" s="29" t="s">
-        <v>3321</v>
+        <v>3318</v>
       </c>
       <c r="B1392" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1392" s="83" t="s">
         <v>2258</v>
       </c>
       <c r="D1392" s="85" t="s">
-        <v>3306</v>
+        <v>3303</v>
       </c>
       <c r="E1392" s="83" t="s">
         <v>2146</v>
@@ -65043,7 +65136,7 @@
         <v>60</v>
       </c>
       <c r="J1392" s="29" t="s">
-        <v>3342</v>
+        <v>3339</v>
       </c>
       <c r="K1392" s="29"/>
       <c r="L1392" s="31"/>
@@ -65051,16 +65144,16 @@
     </row>
     <row r="1393" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1393" s="29" t="s">
-        <v>3322</v>
+        <v>3319</v>
       </c>
       <c r="B1393" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1393" s="83" t="s">
         <v>2347</v>
       </c>
       <c r="D1393" s="85" t="s">
-        <v>3307</v>
+        <v>3304</v>
       </c>
       <c r="E1393" s="83" t="s">
         <v>2146</v>
@@ -65074,7 +65167,7 @@
         <v>60</v>
       </c>
       <c r="J1393" s="29" t="s">
-        <v>3343</v>
+        <v>3340</v>
       </c>
       <c r="K1393" s="29"/>
       <c r="L1393" s="31"/>
@@ -65082,10 +65175,10 @@
     </row>
     <row r="1394" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1394" s="29" t="s">
-        <v>3323</v>
+        <v>3320</v>
       </c>
       <c r="B1394" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1394" s="83" t="s">
         <v>1821</v>
@@ -65094,7 +65187,7 @@
         <v>246</v>
       </c>
       <c r="E1394" s="83" t="s">
-        <v>3345</v>
+        <v>3342</v>
       </c>
       <c r="F1394" s="31"/>
       <c r="G1394" s="31" t="s">
@@ -65105,7 +65198,7 @@
         <v>60</v>
       </c>
       <c r="J1394" s="29" t="s">
-        <v>3282</v>
+        <v>3279</v>
       </c>
       <c r="K1394" s="29"/>
       <c r="L1394" s="31"/>
@@ -65113,10 +65206,10 @@
     </row>
     <row r="1395" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1395" s="29" t="s">
-        <v>3325</v>
+        <v>3322</v>
       </c>
       <c r="B1395" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1395" s="83" t="s">
         <v>2359</v>
@@ -65130,7 +65223,7 @@
         <v>60</v>
       </c>
       <c r="J1395" s="29" t="s">
-        <v>3344</v>
+        <v>3341</v>
       </c>
       <c r="K1395" s="29"/>
       <c r="L1395" s="31"/>
@@ -65138,10 +65231,10 @@
     </row>
     <row r="1396" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1396" s="29" t="s">
-        <v>3326</v>
+        <v>3323</v>
       </c>
       <c r="B1396" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1396" s="83" t="s">
         <v>2360</v>
@@ -65155,7 +65248,7 @@
         <v>60</v>
       </c>
       <c r="J1396" s="29" t="s">
-        <v>3344</v>
+        <v>3341</v>
       </c>
       <c r="K1396" s="29"/>
       <c r="L1396" s="31"/>
@@ -65163,10 +65256,10 @@
     </row>
     <row r="1397" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1397" s="29" t="s">
-        <v>3327</v>
+        <v>3324</v>
       </c>
       <c r="B1397" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1397" s="83" t="s">
         <v>2361</v>
@@ -65180,7 +65273,7 @@
         <v>60</v>
       </c>
       <c r="J1397" s="29" t="s">
-        <v>3344</v>
+        <v>3341</v>
       </c>
       <c r="K1397" s="29"/>
       <c r="L1397" s="31"/>
@@ -65188,10 +65281,10 @@
     </row>
     <row r="1398" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1398" s="29" t="s">
-        <v>3328</v>
+        <v>3325</v>
       </c>
       <c r="B1398" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1398" s="83" t="s">
         <v>2362</v>
@@ -65205,7 +65298,7 @@
         <v>60</v>
       </c>
       <c r="J1398" s="29" t="s">
-        <v>3344</v>
+        <v>3341</v>
       </c>
       <c r="K1398" s="29"/>
       <c r="L1398" s="31"/>
@@ -65213,10 +65306,10 @@
     </row>
     <row r="1399" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1399" s="29" t="s">
-        <v>3329</v>
+        <v>3326</v>
       </c>
       <c r="B1399" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1399" s="83" t="s">
         <v>2363</v>
@@ -65230,7 +65323,7 @@
         <v>60</v>
       </c>
       <c r="J1399" s="29" t="s">
-        <v>3344</v>
+        <v>3341</v>
       </c>
       <c r="K1399" s="29"/>
       <c r="L1399" s="31"/>
@@ -65238,10 +65331,10 @@
     </row>
     <row r="1400" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1400" s="29" t="s">
-        <v>3330</v>
+        <v>3327</v>
       </c>
       <c r="B1400" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1400" s="83" t="s">
         <v>2364</v>
@@ -65255,7 +65348,7 @@
         <v>60</v>
       </c>
       <c r="J1400" s="29" t="s">
-        <v>3344</v>
+        <v>3341</v>
       </c>
       <c r="K1400" s="29"/>
       <c r="L1400" s="31"/>
@@ -65263,10 +65356,10 @@
     </row>
     <row r="1401" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1401" s="29" t="s">
-        <v>3331</v>
+        <v>3328</v>
       </c>
       <c r="B1401" s="100" t="s">
-        <v>3257</v>
+        <v>3254</v>
       </c>
       <c r="C1401" s="83" t="s">
         <v>2365</v>
@@ -65280,7 +65373,7 @@
         <v>60</v>
       </c>
       <c r="J1401" s="29" t="s">
-        <v>3344</v>
+        <v>3341</v>
       </c>
       <c r="K1401" s="29"/>
       <c r="L1401" s="31"/>
@@ -65288,7 +65381,7 @@
     </row>
     <row r="1402" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1402" s="29" t="s">
-        <v>3361</v>
+        <v>3357</v>
       </c>
       <c r="B1402" s="100" t="s">
         <v>884</v>
@@ -65321,7 +65414,7 @@
     </row>
     <row r="1403" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1403" s="29" t="s">
-        <v>3362</v>
+        <v>3358</v>
       </c>
       <c r="B1403" s="100" t="s">
         <v>884</v>
@@ -65352,7 +65445,7 @@
     </row>
     <row r="1404" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1404" s="29" t="s">
-        <v>3363</v>
+        <v>3359</v>
       </c>
       <c r="B1404" s="100" t="s">
         <v>884</v>
@@ -65383,7 +65476,7 @@
     </row>
     <row r="1405" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1405" s="29" t="s">
-        <v>3364</v>
+        <v>3360</v>
       </c>
       <c r="B1405" s="100" t="s">
         <v>884</v>
@@ -65414,7 +65507,7 @@
     </row>
     <row r="1406" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1406" s="29" t="s">
-        <v>3365</v>
+        <v>3361</v>
       </c>
       <c r="B1406" s="100" t="s">
         <v>884</v>
@@ -65443,7 +65536,7 @@
     </row>
     <row r="1407" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1407" s="29" t="s">
-        <v>3366</v>
+        <v>3362</v>
       </c>
       <c r="B1407" s="100" t="s">
         <v>884</v>
@@ -65468,7 +65561,7 @@
         <v>60</v>
       </c>
       <c r="J1407" s="29" t="s">
-        <v>3385</v>
+        <v>3381</v>
       </c>
       <c r="K1407" s="29"/>
       <c r="L1407" s="31"/>
@@ -65476,7 +65569,7 @@
     </row>
     <row r="1408" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1408" s="29" t="s">
-        <v>3367</v>
+        <v>3363</v>
       </c>
       <c r="B1408" s="100" t="s">
         <v>884</v>
@@ -65505,7 +65598,7 @@
     </row>
     <row r="1409" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1409" s="29" t="s">
-        <v>3368</v>
+        <v>3364</v>
       </c>
       <c r="B1409" s="100" t="s">
         <v>884</v>
@@ -65534,7 +65627,7 @@
     </row>
     <row r="1410" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1410" s="29" t="s">
-        <v>3369</v>
+        <v>3365</v>
       </c>
       <c r="B1410" s="100" t="s">
         <v>884</v>
@@ -65563,7 +65656,7 @@
     </row>
     <row r="1411" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1411" s="29" t="s">
-        <v>3370</v>
+        <v>3366</v>
       </c>
       <c r="B1411" s="100" t="s">
         <v>884</v>
@@ -65592,7 +65685,7 @@
     </row>
     <row r="1412" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1412" s="29" t="s">
-        <v>3371</v>
+        <v>3367</v>
       </c>
       <c r="B1412" s="100" t="s">
         <v>884</v>
@@ -65621,7 +65714,7 @@
     </row>
     <row r="1413" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1413" s="29" t="s">
-        <v>3372</v>
+        <v>3368</v>
       </c>
       <c r="B1413" s="100" t="s">
         <v>884</v>
@@ -65650,7 +65743,7 @@
     </row>
     <row r="1414" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1414" s="29" t="s">
-        <v>3373</v>
+        <v>3369</v>
       </c>
       <c r="B1414" s="100" t="s">
         <v>884</v>
@@ -65679,7 +65772,7 @@
     </row>
     <row r="1415" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1415" s="29" t="s">
-        <v>3374</v>
+        <v>3370</v>
       </c>
       <c r="B1415" s="100" t="s">
         <v>884</v>
@@ -65708,7 +65801,7 @@
     </row>
     <row r="1416" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1416" s="29" t="s">
-        <v>3375</v>
+        <v>3371</v>
       </c>
       <c r="B1416" s="100" t="s">
         <v>884</v>
@@ -65737,7 +65830,7 @@
     </row>
     <row r="1417" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1417" s="29" t="s">
-        <v>3376</v>
+        <v>3372</v>
       </c>
       <c r="B1417" s="100" t="s">
         <v>884</v>
@@ -65766,7 +65859,7 @@
     </row>
     <row r="1418" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1418" s="29" t="s">
-        <v>3377</v>
+        <v>3373</v>
       </c>
       <c r="B1418" s="100" t="s">
         <v>884</v>
@@ -65795,7 +65888,7 @@
     </row>
     <row r="1419" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1419" s="29" t="s">
-        <v>3378</v>
+        <v>3374</v>
       </c>
       <c r="B1419" s="100" t="s">
         <v>884</v>
@@ -65824,7 +65917,7 @@
     </row>
     <row r="1420" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1420" s="29" t="s">
-        <v>3379</v>
+        <v>3375</v>
       </c>
       <c r="B1420" s="100" t="s">
         <v>884</v>
@@ -65853,7 +65946,7 @@
     </row>
     <row r="1421" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1421" s="29" t="s">
-        <v>3380</v>
+        <v>3376</v>
       </c>
       <c r="B1421" s="100" t="s">
         <v>884</v>
@@ -65882,7 +65975,7 @@
     </row>
     <row r="1422" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1422" s="29" t="s">
-        <v>3381</v>
+        <v>3377</v>
       </c>
       <c r="B1422" s="100" t="s">
         <v>884</v>
@@ -65911,7 +66004,7 @@
     </row>
     <row r="1423" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1423" s="29" t="s">
-        <v>3382</v>
+        <v>3378</v>
       </c>
       <c r="B1423" s="100" t="s">
         <v>884</v>
@@ -65940,7 +66033,7 @@
     </row>
     <row r="1424" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1424" s="29" t="s">
-        <v>3383</v>
+        <v>3379</v>
       </c>
       <c r="B1424" s="100" t="s">
         <v>884</v>
@@ -65969,7 +66062,7 @@
     </row>
     <row r="1425" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1425" s="29" t="s">
-        <v>3384</v>
+        <v>3380</v>
       </c>
       <c r="B1425" s="100" t="s">
         <v>884</v>
@@ -65998,22 +66091,22 @@
     </row>
     <row r="1426" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1426" s="29" t="s">
-        <v>3389</v>
+        <v>3385</v>
       </c>
       <c r="B1426" s="100" t="s">
         <v>55</v>
       </c>
       <c r="C1426" s="83" t="s">
-        <v>3390</v>
+        <v>3386</v>
       </c>
       <c r="D1426" s="85" t="s">
         <v>176</v>
       </c>
       <c r="E1426" s="83" t="s">
-        <v>3391</v>
+        <v>3387</v>
       </c>
       <c r="F1426" s="31" t="s">
-        <v>3392</v>
+        <v>3388</v>
       </c>
       <c r="G1426" s="31" t="s">
         <v>1450</v>
@@ -66031,7 +66124,7 @@
     </row>
     <row r="1427" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1427" s="29" t="s">
-        <v>3393</v>
+        <v>3389</v>
       </c>
       <c r="B1427" s="100" t="s">
         <v>247</v>
@@ -66040,10 +66133,10 @@
         <v>1193</v>
       </c>
       <c r="D1427" s="137" t="s">
-        <v>3394</v>
+        <v>3390</v>
       </c>
       <c r="E1427" s="83" t="s">
-        <v>3395</v>
+        <v>3391</v>
       </c>
       <c r="F1427" s="31" t="s">
         <v>228</v>
@@ -66064,28 +66157,28 @@
     </row>
     <row r="1428" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1428" s="29" t="s">
-        <v>3398</v>
+        <v>3394</v>
       </c>
       <c r="B1428" s="100" t="s">
-        <v>3424</v>
+        <v>3420</v>
       </c>
       <c r="C1428" s="83" t="s">
-        <v>3397</v>
+        <v>3393</v>
       </c>
       <c r="D1428" s="85" t="s">
+        <v>3392</v>
+      </c>
+      <c r="E1428" s="83" t="s">
+        <v>3393</v>
+      </c>
+      <c r="F1428" s="31" t="s">
+        <v>3395</v>
+      </c>
+      <c r="G1428" s="31" t="s">
+        <v>3395</v>
+      </c>
+      <c r="H1428" s="29" t="s">
         <v>3396</v>
-      </c>
-      <c r="E1428" s="83" t="s">
-        <v>3397</v>
-      </c>
-      <c r="F1428" s="31" t="s">
-        <v>3399</v>
-      </c>
-      <c r="G1428" s="31" t="s">
-        <v>3399</v>
-      </c>
-      <c r="H1428" s="29" t="s">
-        <v>3400</v>
       </c>
       <c r="I1428" s="119" t="s">
         <v>96</v>
@@ -66093,34 +66186,34 @@
       <c r="J1428" s="29"/>
       <c r="K1428" s="29"/>
       <c r="L1428" s="31" t="s">
-        <v>3415</v>
+        <v>3411</v>
       </c>
       <c r="M1428" s="29"/>
     </row>
     <row r="1429" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1429" s="29" t="s">
-        <v>3403</v>
+        <v>3399</v>
       </c>
       <c r="B1429" s="100" t="s">
-        <v>3424</v>
+        <v>3420</v>
       </c>
       <c r="C1429" s="83" t="s">
-        <v>3401</v>
+        <v>3397</v>
       </c>
       <c r="D1429" s="85" t="s">
-        <v>3402</v>
+        <v>3398</v>
       </c>
       <c r="E1429" s="83" t="s">
-        <v>3397</v>
+        <v>3393</v>
       </c>
       <c r="F1429" s="31" t="s">
-        <v>3399</v>
+        <v>3395</v>
       </c>
       <c r="G1429" s="31" t="s">
-        <v>3399</v>
+        <v>3395</v>
       </c>
       <c r="H1429" s="29" t="s">
-        <v>3400</v>
+        <v>3396</v>
       </c>
       <c r="I1429" s="119" t="s">
         <v>96</v>
@@ -66128,34 +66221,34 @@
       <c r="J1429" s="29"/>
       <c r="K1429" s="29"/>
       <c r="L1429" s="31" t="s">
-        <v>3415</v>
+        <v>3411</v>
       </c>
       <c r="M1429" s="29"/>
     </row>
     <row r="1430" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1430" s="29" t="s">
+        <v>3400</v>
+      </c>
+      <c r="B1430" s="100" t="s">
+        <v>3420</v>
+      </c>
+      <c r="C1430" s="83" t="s">
+        <v>3402</v>
+      </c>
+      <c r="D1430" s="85" t="s">
+        <v>3392</v>
+      </c>
+      <c r="E1430" s="83" t="s">
         <v>3404</v>
       </c>
-      <c r="B1430" s="100" t="s">
-        <v>3424</v>
-      </c>
-      <c r="C1430" s="83" t="s">
-        <v>3406</v>
-      </c>
-      <c r="D1430" s="85" t="s">
-        <v>3396</v>
-      </c>
-      <c r="E1430" s="83" t="s">
-        <v>3408</v>
-      </c>
       <c r="F1430" s="31" t="s">
-        <v>3409</v>
+        <v>3405</v>
       </c>
       <c r="G1430" s="31" t="s">
         <v>52</v>
       </c>
       <c r="H1430" s="29" t="s">
-        <v>3400</v>
+        <v>3396</v>
       </c>
       <c r="I1430" s="119" t="s">
         <v>96</v>
@@ -66163,34 +66256,34 @@
       <c r="J1430" s="29"/>
       <c r="K1430" s="29"/>
       <c r="L1430" s="31" t="s">
-        <v>3415</v>
+        <v>3411</v>
       </c>
       <c r="M1430" s="29"/>
     </row>
     <row r="1431" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1431" s="29" t="s">
+        <v>3401</v>
+      </c>
+      <c r="B1431" s="100" t="s">
+        <v>3420</v>
+      </c>
+      <c r="C1431" s="83" t="s">
+        <v>3403</v>
+      </c>
+      <c r="D1431" s="85" t="s">
+        <v>3398</v>
+      </c>
+      <c r="E1431" s="83" t="s">
+        <v>3404</v>
+      </c>
+      <c r="F1431" s="31" t="s">
         <v>3405</v>
-      </c>
-      <c r="B1431" s="100" t="s">
-        <v>3424</v>
-      </c>
-      <c r="C1431" s="83" t="s">
-        <v>3407</v>
-      </c>
-      <c r="D1431" s="85" t="s">
-        <v>3402</v>
-      </c>
-      <c r="E1431" s="83" t="s">
-        <v>3408</v>
-      </c>
-      <c r="F1431" s="31" t="s">
-        <v>3409</v>
       </c>
       <c r="G1431" s="31" t="s">
         <v>52</v>
       </c>
       <c r="H1431" s="29" t="s">
-        <v>3400</v>
+        <v>3396</v>
       </c>
       <c r="I1431" s="119" t="s">
         <v>96</v>
@@ -66198,26 +66291,26 @@
       <c r="J1431" s="29"/>
       <c r="K1431" s="29"/>
       <c r="L1431" s="31" t="s">
-        <v>3415</v>
+        <v>3411</v>
       </c>
       <c r="M1431" s="29"/>
     </row>
     <row r="1432" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1432" s="29" t="s">
-        <v>3411</v>
+        <v>3407</v>
       </c>
       <c r="B1432" s="100"/>
       <c r="C1432" s="83"/>
       <c r="D1432" s="85"/>
       <c r="E1432" s="83"/>
       <c r="F1432" s="31" t="s">
-        <v>3413</v>
+        <v>3409</v>
       </c>
       <c r="G1432" s="31" t="s">
+        <v>3406</v>
+      </c>
+      <c r="H1432" s="29" t="s">
         <v>3410</v>
-      </c>
-      <c r="H1432" s="29" t="s">
-        <v>3414</v>
       </c>
       <c r="I1432" s="119" t="s">
         <v>96</v>
@@ -66225,26 +66318,26 @@
       <c r="J1432" s="29"/>
       <c r="K1432" s="29"/>
       <c r="L1432" s="31" t="s">
-        <v>3415</v>
+        <v>3411</v>
       </c>
       <c r="M1432" s="29"/>
     </row>
     <row r="1433" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1433" s="29" t="s">
-        <v>3412</v>
+        <v>3408</v>
       </c>
       <c r="B1433" s="100"/>
       <c r="C1433" s="83"/>
       <c r="D1433" s="85"/>
       <c r="E1433" s="83"/>
       <c r="F1433" s="31" t="s">
-        <v>3413</v>
+        <v>3409</v>
       </c>
       <c r="G1433" s="31" t="s">
+        <v>3406</v>
+      </c>
+      <c r="H1433" s="29" t="s">
         <v>3410</v>
-      </c>
-      <c r="H1433" s="29" t="s">
-        <v>3414</v>
       </c>
       <c r="I1433" s="119" t="s">
         <v>96</v>
@@ -66252,32 +66345,32 @@
       <c r="J1433" s="29"/>
       <c r="K1433" s="29"/>
       <c r="L1433" s="31" t="s">
-        <v>3415</v>
+        <v>3411</v>
       </c>
       <c r="M1433" s="29"/>
     </row>
     <row r="1434" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1434" s="29" t="s">
-        <v>3416</v>
+        <v>3412</v>
       </c>
       <c r="B1434" s="100" t="s">
-        <v>3421</v>
+        <v>3417</v>
       </c>
       <c r="C1434" s="83"/>
       <c r="D1434" s="85" t="s">
+        <v>3392</v>
+      </c>
+      <c r="E1434" s="83" t="s">
+        <v>3414</v>
+      </c>
+      <c r="F1434" s="31" t="s">
+        <v>3415</v>
+      </c>
+      <c r="G1434" s="31" t="s">
+        <v>3416</v>
+      </c>
+      <c r="H1434" s="29" t="s">
         <v>3396</v>
-      </c>
-      <c r="E1434" s="83" t="s">
-        <v>3418</v>
-      </c>
-      <c r="F1434" s="31" t="s">
-        <v>3419</v>
-      </c>
-      <c r="G1434" s="31" t="s">
-        <v>3420</v>
-      </c>
-      <c r="H1434" s="29" t="s">
-        <v>3400</v>
       </c>
       <c r="I1434" s="119" t="s">
         <v>96</v>
@@ -66285,32 +66378,32 @@
       <c r="J1434" s="29"/>
       <c r="K1434" s="29"/>
       <c r="L1434" s="31" t="s">
-        <v>3415</v>
+        <v>3411</v>
       </c>
       <c r="M1434" s="29"/>
     </row>
     <row r="1435" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1435" s="29" t="s">
+        <v>3413</v>
+      </c>
+      <c r="B1435" s="100" t="s">
         <v>3417</v>
-      </c>
-      <c r="B1435" s="100" t="s">
-        <v>3421</v>
       </c>
       <c r="C1435" s="83"/>
       <c r="D1435" s="85" t="s">
-        <v>3402</v>
+        <v>3398</v>
       </c>
       <c r="E1435" s="83" t="s">
-        <v>3418</v>
+        <v>3414</v>
       </c>
       <c r="F1435" s="31" t="s">
-        <v>3419</v>
+        <v>3415</v>
       </c>
       <c r="G1435" s="31" t="s">
-        <v>3420</v>
+        <v>3416</v>
       </c>
       <c r="H1435" s="29" t="s">
-        <v>3400</v>
+        <v>3396</v>
       </c>
       <c r="I1435" s="119" t="s">
         <v>96</v>
@@ -66318,13 +66411,13 @@
       <c r="J1435" s="29"/>
       <c r="K1435" s="29"/>
       <c r="L1435" s="31" t="s">
-        <v>3415</v>
+        <v>3411</v>
       </c>
       <c r="M1435" s="29"/>
     </row>
     <row r="1436" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1436" s="29" t="s">
-        <v>3429</v>
+        <v>3425</v>
       </c>
       <c r="B1436" s="100" t="s">
         <v>1019</v>

</xml_diff>

<commit_message>
added software to cumu-g002
</commit_message>
<xml_diff>
--- a/cables.xlsx
+++ b/cables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/donert/Documents/UACTech/uacdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B2F75D2-87FD-844C-A32F-4E2D3D8E174B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F9CF204-C7F9-F64D-92A0-67E085CA71B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1820" yWindow="760" windowWidth="26600" windowHeight="18020" xr2:uid="{288904EE-D384-EA4C-9B98-052B972FB267}"/>
   </bookViews>
@@ -18,8 +18,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="5" r:id="rId3"/>
-    <pivotCache cacheId="6" r:id="rId4"/>
+    <pivotCache cacheId="1" r:id="rId3"/>
+    <pivotCache cacheId="2" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11761" uniqueCount="3440">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11772" uniqueCount="3446">
   <si>
     <t>Tag</t>
   </si>
@@ -10364,6 +10364,24 @@
   </si>
   <si>
     <t>output2</t>
+  </si>
+  <si>
+    <t>2608-2901</t>
+  </si>
+  <si>
+    <t>2608-2900</t>
+  </si>
+  <si>
+    <t>USB</t>
+  </si>
+  <si>
+    <t>.51m</t>
+  </si>
+  <si>
+    <t>grandMA3 Redundant interface</t>
+  </si>
+  <si>
+    <t>Christie 44339</t>
   </si>
 </sst>
 </file>
@@ -19879,7 +19897,70 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="6" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Count of Tag" fld="0" subtotal="count" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{10F736CA-5D69-4D44-A803-D4241D124F38}" name="PivotTable1" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="A3:B56" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField dataField="1" showAll="0"/>
@@ -20112,69 +20193,6 @@
     </i>
     <i>
       <x v="53"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Count of Tag" fld="0" subtotal="count" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{331FD294-EE6F-3D4E-A534-813A4D9D566E}" name="PivotTable2" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="E5:F10" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="12">
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="7"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
     </i>
     <i t="grand">
       <x/>
@@ -66478,18 +66496,40 @@
       <c r="M1436" s="29"/>
     </row>
     <row r="1437" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A1437" s="29"/>
-      <c r="B1437" s="100"/>
-      <c r="C1437" s="83"/>
-      <c r="D1437" s="85"/>
-      <c r="E1437" s="83"/>
-      <c r="F1437" s="31"/>
-      <c r="G1437" s="31"/>
-      <c r="H1437" s="29"/>
-      <c r="I1437" s="119"/>
-      <c r="J1437" s="29"/>
+      <c r="A1437" s="29" t="s">
+        <v>3440</v>
+      </c>
+      <c r="B1437" s="100" t="s">
+        <v>704</v>
+      </c>
+      <c r="C1437" s="83" t="s">
+        <v>3403</v>
+      </c>
+      <c r="D1437" s="85" t="s">
+        <v>3441</v>
+      </c>
+      <c r="E1437" s="83" t="s">
+        <v>3442</v>
+      </c>
+      <c r="F1437" s="31" t="s">
+        <v>3408</v>
+      </c>
+      <c r="G1437" s="31" t="s">
+        <v>3442</v>
+      </c>
+      <c r="H1437" s="29" t="s">
+        <v>3443</v>
+      </c>
+      <c r="I1437" s="119" t="s">
+        <v>96</v>
+      </c>
+      <c r="J1437" s="29" t="s">
+        <v>3444</v>
+      </c>
       <c r="K1437" s="29"/>
-      <c r="L1437" s="31"/>
+      <c r="L1437" s="31" t="s">
+        <v>3445</v>
+      </c>
       <c r="M1437" s="29"/>
     </row>
     <row r="1438" spans="1:13" x14ac:dyDescent="0.2">

</xml_diff>